<commit_message>
Refactor health record management by removing the PDF generation code from utils.js and updating the index.js to utilize Puppeteer for report generation. Simplified error handling in error.json and updated health summaries in output.json to reflect patient recovery from Alcohol Withdrawal.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:Q23"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -466,6 +466,9 @@
       <c r="P1" t="str">
         <v>Total Tokens</v>
       </c>
+      <c r="Q1" t="str">
+        <v>Model</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1217,9 +1220,344 @@
         <v>1545</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-01-30T12:24:25.024Z</v>
+      </c>
+      <c r="B17" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D17">
+        <v>36</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Asthma Attack</v>
+      </c>
+      <c r="F17" t="str">
+        <v>68e36fbc9950693f31349cc7</v>
+      </c>
+      <c r="G17" t="str">
+        <v>John Doe is experiencing significant asthma symptoms, including difficulty breathing and an inability to talk or eat. His overall vital signs are stable, but attention is needed for his asthma management.</v>
+      </c>
+      <c r="H17" t="str">
+        <v>HIGH: Critical asthma symptoms detected. Immediate medical evaluation is recommended.</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Blood Pressure: 120/80, Heart Rate: 70, Oxygen Level: 98%, Body Temperature: 98.6°F, Blood Sugar: 100 mg/dL. Vital signs are stable.</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Routine activities such as meals and rest are crucial for managing asthma symptoms.</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Avoid triggers like dust and smoke. Consider breathing exercises and keeping fast-relief inhaler accessible.</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Monitor asthma symptoms closely. Ensure medication adherence and consider follow-up appointments.</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Schedule a follow-up consultation with your healthcare provider and review asthma action plan.</v>
+      </c>
+      <c r="N17">
+        <v>1048</v>
+      </c>
+      <c r="O17">
+        <v>236</v>
+      </c>
+      <c r="P17">
+        <v>1284</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-02-06T13:41:53.644Z</v>
+      </c>
+      <c r="B18" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D18">
+        <v>36</v>
+      </c>
+      <c r="G18" t="str">
+        <v>John Doe has successfully cured his alcohol withdrawal condition. His vital signs are stable within normal ranges but require monitoring to ensure continued well-being.</v>
+      </c>
+      <c r="H18" t="str">
+        <v>LOW: Monitor for any resurgence of symptoms related to alcohol withdrawal.</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Blood Pressure: 120/80 | Heart Rate: 70 bpm | Oxygen Level: 98% | Body Temperature: 98.6°F | Blood Sugar: 100 mg/dL</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Regular meals appear to positively impact blood sugar levels. | Engagement in daily routines seems to help stabilize heart rate and blood pressure.</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Maintain a balanced diet to support recovery. | Stay hydrated and continue regular physical activities. | Consider relaxation techniques like meditation to support mental health.</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Continue monitoring withdrawal symptoms and maintain a healthy lifestyle. | Follow up in two weeks to review overall health progress.</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Schedule a follow-up appointment with a healthcare provider. | Keep a daily log of any symptoms or changes in health. | Engage in scheduled activities and try to maintain a structured routine.</v>
+      </c>
+      <c r="N18">
+        <v>1079</v>
+      </c>
+      <c r="O18">
+        <v>290</v>
+      </c>
+      <c r="P18">
+        <v>1369</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-02-06T13:45:46.363Z</v>
+      </c>
+      <c r="B19" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D19">
+        <v>36</v>
+      </c>
+      <c r="G19" t="str">
+        <v>John Doe has shown consistent vital signs with no major irregularities detected during the past week. However, he experienced episodes of confusion and sweating.</v>
+      </c>
+      <c r="H19" t="str">
+        <v>MEDIUM: Episodes of confusion have been reported with increasing severity. Monitoring is advised.</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Blood pressure is stable at 120/80. | Heart rate remains at a healthy 70 bpm. | Oxygen level is within normal limits at 98%. | Body temperature is steady at 98.6°F. | Blood sugar levels are consistently at 100.</v>
+      </c>
+      <c r="J19" t="str">
+        <v>John participates in breakfast daily at 10:00 AM, which may help regulate his blood sugar levels.</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Consider maintaining a consistent meal schedule to support overall health.</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Continued observation required for symptoms of confusion and sweating. Encourage patient to report any worsening symptoms.</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Schedule a follow-up appointment to further assess the episodes of confusion. | Monitor daily activities and symptoms closely.</v>
+      </c>
+      <c r="N19">
+        <v>1079</v>
+      </c>
+      <c r="O19">
+        <v>261</v>
+      </c>
+      <c r="P19">
+        <v>1340</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-02-06T13:57:01.277Z</v>
+      </c>
+      <c r="B20" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D20">
+        <v>36</v>
+      </c>
+      <c r="G20" t="str">
+        <v>John Doe has shown improvement in managing his alcohol withdrawal symptoms, with no current critical alerts. Vital signs are stable.</v>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v>Blood pressure: 120/80, Heart rate: 70, Oxygen level: 98%, Body temperature: 98.6°F, Blood sugar: 100 mg/dL</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Regular meals and a consistent sleep schedule have positively influenced vital signs.</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Continue to maintain a balanced diet with plenty of hydration and nutrients. | Incorporate light physical activities to support overall health.</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Johnson's vital signs and symptoms have been stable. Regular check-ins are recommended.</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Schedule a follow-up appointment in two weeks. | Monitor symptoms closely and seek help if they worsen.</v>
+      </c>
+      <c r="N20">
+        <v>1079</v>
+      </c>
+      <c r="O20">
+        <v>204</v>
+      </c>
+      <c r="P20">
+        <v>1283</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-02-06T13:57:19.212Z</v>
+      </c>
+      <c r="B21" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D21">
+        <v>36</v>
+      </c>
+      <c r="G21" t="str">
+        <v>John Doe has shown improvement since his conditions related to alcohol withdrawal. His vital signs are stable, indicating good health management over the past week.</v>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v>Blood Pressure: 120/80 mmHg; Heart Rate: 70 bpm; Oxygen Level: 98%; Body Temperature: 98.6°F; Blood Sugar: 100 mg/dL</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Routine breakfast in the canteen has been consistent, contributing positively to his overall health.</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Maintain consistent meal times to help stabilize energy levels. | Stay hydrated and engage in regular physical activity to aid recovery and overall wellness.</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Continued monitoring of symptoms is recommended. No immediate concerns noted.</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Keep a daily log of symptoms and vital signs for further assessment. | Schedule a follow-up appointment with the healthcare provider next week.</v>
+      </c>
+      <c r="N21">
+        <v>1079</v>
+      </c>
+      <c r="O21">
+        <v>220</v>
+      </c>
+      <c r="P21">
+        <v>1299</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-02-06T13:58:02.085Z</v>
+      </c>
+      <c r="B22" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D22">
+        <v>36</v>
+      </c>
+      <c r="G22" t="str">
+        <v>John Doe has recently recovered from Alcohol Withdrawal. His vital signs remain stable, and he is maintaining a regular routine.</v>
+      </c>
+      <c r="H22" t="str">
+        <v>LOW: Symptom severity for confusion and sweating shows fluctuations, but no urgent concerns detected.</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Blood Pressure: 120/80, Heart Rate: 70, Oxygen Level: 98%, Body Temperature: 98.6°F, Blood Sugar: 100 mg/dL.</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Regular meals and hydration contribute positively to symptom management.</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Maintain a balanced diet and stay hydrated to support recovery.</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Continue monitoring symptoms; consider regular check-ins for support.</v>
+      </c>
+      <c r="M22" t="str">
+        <v>Schedule a follow-up appointment for ongoing assessment.</v>
+      </c>
+      <c r="N22">
+        <v>1079</v>
+      </c>
+      <c r="O22">
+        <v>203</v>
+      </c>
+      <c r="P22">
+        <v>1282</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-02-09T06:18:23.765Z</v>
+      </c>
+      <c r="B23" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D23">
+        <v>36</v>
+      </c>
+      <c r="G23" t="str">
+        <v>John Doe has shown significant improvement in managing his health after recovering from Alcohol Withdrawal. His vital signs are stable, and there are no critical alerts at this time.</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v>Blood Pressure: 120/80 | Heart Rate: 70 bpm | Oxygen Level: 98% | Body Temperature: 98.6°F | Blood Sugar: 100 mg/dL</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Regular meals and maintaining hydration have contributed positively to his overall well-being. | Activity routines such as breakfast at 10:00 AM help in achieving consistent vital signs.</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Continue to maintain a balanced diet rich in fruits and vegetables. | Stay hydrated by drinking plenty of water throughout the day. | Engage in regular physical activity to support mental and physical health.</v>
+      </c>
+      <c r="L23" t="str">
+        <v>John has shown considerable resilience in managing his symptoms post-recovery. Continue to monitor for any changes.</v>
+      </c>
+      <c r="M23" t="str">
+        <v>Schedule a follow-up appointment with the healthcare provider in the next month. | Maintain a daily log of symptoms and vital signs to discuss in the next visit.</v>
+      </c>
+      <c r="N23">
+        <v>1079</v>
+      </c>
+      <c r="O23">
+        <v>273</v>
+      </c>
+      <c r="P23">
+        <v>1352</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update health record management by modifying the saveToExcel function to include payload data. Adjusted health summaries in output.json to reflect patient recovery from Alcohol Withdrawal, enhancing clarity in health alerts and next steps. Updated index.js to pass the payload when saving records.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:R24"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -469,6 +469,9 @@
       <c r="Q1" t="str">
         <v>Model</v>
       </c>
+      <c r="R1" t="str">
+        <v>Payload Data</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1555,9 +1558,59 @@
         <v>gpt-4o-mini</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-02-09T13:40:22.413Z</v>
+      </c>
+      <c r="B24" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D24">
+        <v>36</v>
+      </c>
+      <c r="G24" t="str">
+        <v>John Doe has successfully recovered from Alcohol Withdrawal. His vital signs are stable, and he has shown improvement in symptoms over time.</v>
+      </c>
+      <c r="H24" t="str">
+        <v>LOW: Symptoms of confusion and sweating were recorded but are currently not severe.</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Blood Pressure: 120/80, Heart Rate: 70, Oxygen Level: 98%, Body Temperature: 98.6°F, Blood Sugar: 100 mg/dL</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Routine activities like breakfast are consistent and likely contributing to stable vital signs.</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Maintain a balanced diet and stay hydrated to support overall health.</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Continue monitoring symptoms and maintain regular check-ins to ensure ongoing recovery.</v>
+      </c>
+      <c r="M24" t="str">
+        <v>Schedule a follow-up appointment to review progress and address any remaining concerns.</v>
+      </c>
+      <c r="N24">
+        <v>771</v>
+      </c>
+      <c r="O24">
+        <v>214</v>
+      </c>
+      <c r="P24">
+        <v>985</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+      <c r="R24" t="str">
+        <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":1,"recorded_at":"2026-02-06T11:14:39.036Z"},{"severity":6,"recorded_at":"2026-02-06T11:12:05.141Z"},{"severity":7,"recorded_at":"2026-02-06T11:05:49.613Z"}],"baselines":{"patient_baseline":null}},{"title":"sweating","records":[{"severity":1,"recorded_at":"2026-02-06T11:14:39.036Z"},{"severity":6,"recorded_at":"2026-02-06T11:12:05.141Z"},{"severity":5,"recorded_at":"2026-02-06T11:05:49.613Z"}],"baselines":{"patient_baseline":null}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"},{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"},{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"},{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"}],"activities":[{"_id":{"$oid":"66e2761ae288f29d07a1d094"},"attendees":[],"facility_id":{"$oid":"66b4cce3b672e092b873cace"},"name":"Breakfast","from_date":{"$date":"2024-09-13T00:00:00.000Z"},"from_time":"10:00","to_time":"10:30","description":"The attitude of gratitude is the highest Lunch.","location":"Canteen","createdAt":{"$date":"2024-09-12T05:03:22.594Z"},"updatedAt":{"$date":"2024-09-12T05:03:22.604Z"},"__v":0,"image":"8187733396.png"}]}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R24"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update error handling in error.json and refactor index.js to improve model validation and error reporting. Added detailed error messages for unsupported models in the chat completions endpoint and enhanced the response handling logic to capture and log errors effectively.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R24"/>
+  <dimension ref="A1:R25"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1608,9 +1608,59 @@
         <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":1,"recorded_at":"2026-02-06T11:14:39.036Z"},{"severity":6,"recorded_at":"2026-02-06T11:12:05.141Z"},{"severity":7,"recorded_at":"2026-02-06T11:05:49.613Z"}],"baselines":{"patient_baseline":null}},{"title":"sweating","records":[{"severity":1,"recorded_at":"2026-02-06T11:14:39.036Z"},{"severity":6,"recorded_at":"2026-02-06T11:12:05.141Z"},{"severity":5,"recorded_at":"2026-02-06T11:05:49.613Z"}],"baselines":{"patient_baseline":null}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"},{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"},{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"},{"blood_pressure":"120/80","heart_rate":"70","oxygen_level":"98","body_temp":"98.6","blood_sugar":"100"}],"activities":[{"_id":{"$oid":"66e2761ae288f29d07a1d094"},"attendees":[],"facility_id":{"$oid":"66b4cce3b672e092b873cace"},"name":"Breakfast","from_date":{"$date":"2024-09-13T00:00:00.000Z"},"from_time":"10:00","to_time":"10:30","description":"The attitude of gratitude is the highest Lunch.","location":"Canteen","createdAt":{"$date":"2024-09-12T05:03:22.594Z"},"updatedAt":{"$date":"2024-09-12T05:03:22.604Z"},"__v":0,"image":"8187733396.png"}]}</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-02-09T13:54:18.913Z</v>
+      </c>
+      <c r="B25" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D25">
+        <v>36</v>
+      </c>
+      <c r="G25" t="str">
+        <v>John Doe has shown improvement in symptoms related to Alcohol Withdrawal, with notable reductions in confusion and sweating over the past week.</v>
+      </c>
+      <c r="H25" t="str">
+        <v>MEDIUM: Initial symptoms of confusion and sweating were above baseline but have improved; stay vigilant.</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Blood Pressure has remained stable with minor fluctuations, averaging 120/80. | Heart Rate is within normal range, averaging 70 bpm. | SpO2 levels are consistently healthy, averaging 98%. | Body Temperature has been normal, averaging 98.5°F. | Blood Sugar levels show minor variations but remain generally stable.</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Regular morning activities, such as breakfast and walks, contribute to stabilizing symptoms and vitals. | Light exercise appears beneficial in maintaining a steady heart rate.</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Continue daily morning walks to maintain physical and mental well-being. | Ensure balanced meals, especially at breakfast, to help maintain energy levels.</v>
+      </c>
+      <c r="L25" t="str">
+        <v>The patient's recovery from Alcohol Withdrawal is progressing well. Continued observation and support are recommended.</v>
+      </c>
+      <c r="M25" t="str">
+        <v>Maintain regular check-ins with the care team. | Continue daily monitoring of vitals and symptoms. | Schedule a follow-up appointment in two weeks to review progress.</v>
+      </c>
+      <c r="N25">
+        <v>2423</v>
+      </c>
+      <c r="O25">
+        <v>309</v>
+      </c>
+      <c r="P25">
+        <v>2732</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>gpt-4o</v>
+      </c>
+      <c r="R25" t="str">
+        <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"118/78"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"122/82"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"120/80"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"121/79"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"119/81"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"120/80"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"123/81"}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"68"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"72"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"70"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"71"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"69"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"70"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"97"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"99"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"97"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"98.4"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98.6"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98.5"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"98.6"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"98.4"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98.5"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"95"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"102"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"105"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"99"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"100"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update health records and model configurations. Replaced deprecated models in index.js with 'gpt-5' and commented out older models. Modified output.json to reflect a simplified structure for model responses, enhancing compatibility with the latest updates.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R25"/>
+  <dimension ref="A1:R29"/>
   <cols>
     <col min="1" max="1" width="25.83203125" customWidth="1"/>
     <col min="2" max="2" width="15.83203125" customWidth="1"/>
@@ -1658,9 +1658,209 @@
         <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"118/78"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"122/82"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"120/80"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"121/79"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"119/81"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"120/80"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"123/81"}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"68"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"72"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"70"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"71"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"69"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"70"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"97"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"99"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"97"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"98.4"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98.6"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98.5"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"98.6"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"98.4"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98.5"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"95"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"102"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"105"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"99"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"100"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-02-09T13:54:23.799Z</v>
+      </c>
+      <c r="B26" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D26">
+        <v>36</v>
+      </c>
+      <c r="G26" t="str">
+        <v>John Doe has shown improvement in his health after recovering from Alcohol Withdrawal. Most vital signs are stable, but there are occasional spikes in symptoms like confusion and sweating.</v>
+      </c>
+      <c r="H26" t="str">
+        <v>MEDIUM: Occasional confusion and sweating recorded. Monitor for any worsening symptoms.</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Blood Pressure is mostly in the normal range, fluctuating between 118/78 and 123/81. | Heart Rate is stable, ranging from 68 to 73 beats per minute. | SpO2 levels remain healthy at 97-99%. | Body Temperature is consistently around normal at 98.4-98.6°F. | Blood Sugar levels are slightly elevated at times but mostly within normal limits (95-105 mg/dL).</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Daily activities including regular meals and light exercise contribute to stable vitals. | Increased sweating and confusion often correlate with higher stress or irregular sleep.</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Maintain a consistent sleep schedule to help reduce confusion. | Incorporate more hydrating foods and regular exercise to alleviate sweating symptoms. | Monitor blood sugar levels by eating smaller, balanced meals throughout the day.</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Continue monitoring for any return of severe withdrawal symptoms. | Encourage patient to communicate any sudden changes in their condition.</v>
+      </c>
+      <c r="M26" t="str">
+        <v>Schedule a follow-up appointment to reassess vitals and symptoms. | Consider a consultation with a nutritionist for tailored dietary recommendations.</v>
+      </c>
+      <c r="N26">
+        <v>2423</v>
+      </c>
+      <c r="O26">
+        <v>353</v>
+      </c>
+      <c r="P26">
+        <v>2776</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+      <c r="R26" t="str">
+        <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"118/78"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"122/82"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"120/80"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"121/79"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"119/81"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"120/80"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"123/81"}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"68"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"72"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"70"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"71"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"69"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"70"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"97"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"99"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"97"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"98.4"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98.6"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98.5"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"98.6"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"98.4"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98.5"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"95"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"102"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"105"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"99"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"100"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-02-09T13:54:34.476Z</v>
+      </c>
+      <c r="B27" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D27">
+        <v>36</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Continuous management and monitoring reveal stable vital signs with minor fluctuations in symptom severity following alcohol withdrawal.</v>
+      </c>
+      <c r="H27" t="str">
+        <v>MEDIUM: Symptoms of confusion and sweating have shown fluctuations but are on a downward trend. Monitor for any unexpected spikes.</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Stable blood pressure with slight variations within the normal range. | Heart rate appears consistent, with minor fluctuations observed. | Oxygen saturation levels remain within the normal range. | Body temperature stays within normal limits. | Blood sugar shows slight variations but requires attention to dietary intake.</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Symptom intensity mildly correlates with missing regular meals or increased physical activity. | Daily activities like walks and light exercise positively associate with better vital sign stability.</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Maintain regular meal times, especially a healthy breakfast to stabilize blood sugar levels. | Moderate, regular exercise like morning walks can aid in maintaining stable health indicators. | Ensure sufficient hydration and a balanced diet to help manage symptoms and stabilize vitals.</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Patient shows good compliance to the prescribed routine, beneficial effects on health noticeable. | Continue monitoring blood sugar closely in relation to meal timings and content.</v>
+      </c>
+      <c r="M27" t="str">
+        <v>Schedule a follow-up consultation next month to review progress and adjust care plan as necessary. | Consider nutritional counseling to optimize diet and further stabilize blood sugar levels.</v>
+      </c>
+      <c r="N27">
+        <v>2366</v>
+      </c>
+      <c r="O27">
+        <v>331</v>
+      </c>
+      <c r="P27">
+        <v>2697</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>gpt-4-turbo</v>
+      </c>
+      <c r="R27" t="str">
+        <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"118/78"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"122/82"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"120/80"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"121/79"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"119/81"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"120/80"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"123/81"}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"68"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"72"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"70"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"71"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"69"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"70"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"97"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"99"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"97"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"98.4"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98.6"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98.5"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"98.6"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"98.4"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98.5"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"95"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"102"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"105"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"99"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"100"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-02-09T13:54:37.831Z</v>
+      </c>
+      <c r="B28" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D28">
+        <v>36</v>
+      </c>
+      <c r="G28" t="str">
+        <v>John Doe's health overview</v>
+      </c>
+      <c r="H28" t="str">
+        <v>HIGH: Alcohol Withdrawal symptoms like confusion and sweating at concerning levels. Immediate medical attention required.</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Blood Pressure within normal range, Heart Rate slightly elevated, SpO2 levels are good, Body Temperature normal, Blood Sugar slightly high.</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Morning walks positively impact vitals, regular meals maintain stable blood sugar levels.</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Increase hydration, reduce alcohol consumption, consider consulting a healthcare professional.</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Patient's vitals show improvements, continue monitoring closely.</v>
+      </c>
+      <c r="M28" t="str">
+        <v>Urgent medical evaluation recommended, follow-up appointment with a specialist.</v>
+      </c>
+      <c r="N28">
+        <v>2366</v>
+      </c>
+      <c r="O28">
+        <v>174</v>
+      </c>
+      <c r="P28">
+        <v>2540</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>gpt-3.5-turbo</v>
+      </c>
+      <c r="R28" t="str">
+        <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"118/78"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"122/82"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"120/80"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"121/79"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"119/81"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"120/80"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"123/81"}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"68"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"72"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"70"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"71"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"69"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"70"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"97"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"99"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"97"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"98.4"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98.6"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98.5"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"98.6"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"98.4"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98.5"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"95"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"102"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"105"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"99"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"100"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-02-09T14:24:40.587Z</v>
+      </c>
+      <c r="B29" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D29">
+        <v>36</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Vitals are stable and in normal ranges. Withdrawal-related symptoms are improving through the week. No urgent alerts found.</v>
+      </c>
+      <c r="H29" t="str">
+        <v/>
+      </c>
+      <c r="I29" t="str">
+        <v>Blood pressure averaged ~120/80 mmHg (range 118/78–123/81); stable and normal. | Heart rate averaged ~70 bpm (range 68–73); steady resting range. | SpO2 stayed 97–99%; normal oxygen levels. | Body temperature 98.4–98.6 F; no fever. | Morning blood sugar ranged 95–105 mg/dL; a few readings slightly above ideal, often taken soon after breakfast which can raise values a little.</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Confusion scores trended down (from 6 to 2 over the week). | Sweating scores trended down (from 6 to 2 over the week). | Vitals were usually taken around 8:10–8:25; breakfast often happened just before, which may nudge glucose up. | Light activity (walks/exercise) did not raise heart rate and symptoms stayed mild afterward. | Lunch and dinner times were irregular on some days; more regular meals may support steadier energy and glucose.</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Continue alcohol-free routine and supports. | Have regular meals (breakfast within an hour of waking, plus lunch and dinner) with protein and fiber; limit sugary drinks. | Drink water regularly through the day. | Do 20–30 minutes of easy activity (like a walk) most days. | Check a true fasting glucose (8+ hours without food) on 1–2 mornings next week for a clearer trend. | Use brief breathing or mindfulness breaks to reduce stress, which may help sweating and focus. | Keep a steady sleep schedule (consistent bedtime and wake time).</v>
+      </c>
+      <c r="L29" t="str">
+        <v>No urgent concerns today; vitals are stable and symptoms are improving. | Slightly higher morning glucose may be due to readings taken soon after eating; a fasting check will clarify. | Please reach out if confusion returns or any new concerning symptoms appear.</v>
+      </c>
+      <c r="M29" t="str">
+        <v>Log vitals at the same time each morning, preferably before breakfast for clearer fasting readings. | Add meal and activity logs more consistently this week. | Maintain alcohol recovery supports and routine. | Schedule a routine check-in within 2–4 weeks to review progress and fasting glucose. | Seek care sooner if any red flags occur: confusion suddenly worse, severe shaking, chest pain, shortness of breath, SpO2 &lt;94%, fever ≥100.4 F, repeated BP &gt;140/90, or resting HR &gt;100.</v>
+      </c>
+      <c r="N29">
+        <v>2422</v>
+      </c>
+      <c r="O29">
+        <v>3613</v>
+      </c>
+      <c r="P29">
+        <v>6035</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>gpt-5</v>
+      </c>
+      <c r="R29" t="str">
+        <v>{"conditions":{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}],"baselines":{"patient_baseline":8}}]},"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"118/78"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"122/82"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"120/80"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"121/79"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"119/81"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"120/80"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"123/81"}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"68"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"72"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"70"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"71"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"69"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"70"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"97"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"99"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"97"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"98.4"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98.6"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98.5"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"98.6"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"98.4"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98.5"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"95"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"102"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"105"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"99"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"100"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update health records to reflect patient improvement post-alcohol withdrawal. Revised overall summary, health alerts, and next steps for clarity. Adjusted vital signs and daily patterns to enhance monitoring and guidance. Updated token usage metrics accordingly.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -397,25 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R40"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="30.83203125" customWidth="1"/>
-    <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="60.83203125" customWidth="1"/>
-    <col min="9" max="9" width="60.83203125" customWidth="1"/>
-    <col min="10" max="10" width="60.83203125" customWidth="1"/>
-    <col min="11" max="11" width="60.83203125" customWidth="1"/>
-    <col min="12" max="12" width="60.83203125" customWidth="1"/>
-    <col min="13" max="13" width="60.83203125" customWidth="1"/>
-    <col min="14" max="14" width="15.83203125" customWidth="1"/>
-    <col min="15" max="15" width="18.83203125" customWidth="1"/>
-    <col min="16" max="16" width="15.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:R41"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -483,7 +465,7 @@
       <c r="C2" t="str">
         <v>Male</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="str">
         <v>36</v>
       </c>
       <c r="E2" t="str">
@@ -513,13 +495,13 @@
       <c r="M2" t="str">
         <v>Schedule a follow-up consultation with the healthcare provider within 24 hours. | Monitor symptoms closely and use prescribed inhalers if applicable. | Seek immediate emergency assistance if unable to talk, eat, or breathe properly.</v>
       </c>
-      <c r="N2">
+      <c r="N2" t="str">
         <v>1048</v>
       </c>
-      <c r="O2">
+      <c r="O2" t="str">
         <v>376</v>
       </c>
-      <c r="P2">
+      <c r="P2" t="str">
         <v>1424</v>
       </c>
     </row>
@@ -533,7 +515,7 @@
       <c r="C3" t="str">
         <v>Male</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="str">
         <v>36</v>
       </c>
       <c r="E3" t="str">
@@ -563,13 +545,13 @@
       <c r="M3" t="str">
         <v>Schedule an urgent follow-up appointment with the respiratory specialist. | Consider an emergency visit if breathing becomes severely impaired. | Ensure patient has access to prescribed inhalers and emergency medications as directed by their healthcare provider. | Continue tracking symptom scores daily to identify any escalation.</v>
       </c>
-      <c r="N3">
+      <c r="N3" t="str">
         <v>1048</v>
       </c>
-      <c r="O3">
+      <c r="O3" t="str">
         <v>398</v>
       </c>
-      <c r="P3">
+      <c r="P3" t="str">
         <v>1446</v>
       </c>
     </row>
@@ -583,7 +565,7 @@
       <c r="C4" t="str">
         <v>Male</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="str">
         <v>36</v>
       </c>
       <c r="E4" t="str">
@@ -613,13 +595,13 @@
       <c r="M4" t="str">
         <v>Schedule an urgent consultation with a healthcare provider. | Monitor symptom changes closely and seek immediate help if breathing worsens. | Keep emergency inhalers accessible at all times. | Plan for a follow-up appointment to reassess condition and treatment.</v>
       </c>
-      <c r="N4">
+      <c r="N4" t="str">
         <v>1048</v>
       </c>
-      <c r="O4">
+      <c r="O4" t="str">
         <v>419</v>
       </c>
-      <c r="P4">
+      <c r="P4" t="str">
         <v>1467</v>
       </c>
     </row>
@@ -633,7 +615,7 @@
       <c r="C5" t="str">
         <v>Male</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="str">
         <v>36</v>
       </c>
       <c r="E5" t="str">
@@ -663,13 +645,13 @@
       <c r="M5" t="str">
         <v>Schedule urgent consultation with respiratory specialist. | Consider in-person evaluation to assess lung function. | Monitor symptoms closely and seek emergency care if breathing worsens.</v>
       </c>
-      <c r="N5">
+      <c r="N5" t="str">
         <v>1048</v>
       </c>
-      <c r="O5">
+      <c r="O5" t="str">
         <v>342</v>
       </c>
-      <c r="P5">
+      <c r="P5" t="str">
         <v>1390</v>
       </c>
     </row>
@@ -683,7 +665,7 @@
       <c r="C6" t="str">
         <v>Male</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="str">
         <v>36</v>
       </c>
       <c r="E6" t="str">
@@ -713,13 +695,13 @@
       <c r="M6" t="str">
         <v>Schedule an urgent consultation with the pulmonologist or asthma specialist. | Monitor symptoms closely with daily logs for any changes. | Ensure access to prescribed inhalers and emergency asthma action plan.</v>
       </c>
-      <c r="N6">
+      <c r="N6" t="str">
         <v>1048</v>
       </c>
-      <c r="O6">
+      <c r="O6" t="str">
         <v>350</v>
       </c>
-      <c r="P6">
+      <c r="P6" t="str">
         <v>1398</v>
       </c>
     </row>
@@ -733,7 +715,7 @@
       <c r="C7" t="str">
         <v>Male</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="str">
         <v>36</v>
       </c>
       <c r="E7" t="str">
@@ -763,13 +745,13 @@
       <c r="M7" t="str">
         <v>Schedule an urgent consultation with the healthcare provider. | Monitor symptoms closely and seek emergency care if breathing worsens. | Consider pulmonary function testing to assess lung status.</v>
       </c>
-      <c r="N7">
+      <c r="N7" t="str">
         <v>1048</v>
       </c>
-      <c r="O7">
+      <c r="O7" t="str">
         <v>331</v>
       </c>
-      <c r="P7">
+      <c r="P7" t="str">
         <v>1379</v>
       </c>
     </row>
@@ -783,7 +765,7 @@
       <c r="C8" t="str">
         <v>Male</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="str">
         <v>36</v>
       </c>
       <c r="E8" t="str">
@@ -813,13 +795,13 @@
       <c r="M8" t="str">
         <v>Schedule an urgent consultation with the respiratory specialist. | Consider emergency care if symptoms such as inability to talk or eat worsen. | Regularly track symptoms and vital signs to update the care team.</v>
       </c>
-      <c r="N8">
+      <c r="N8" t="str">
         <v>1048</v>
       </c>
-      <c r="O8">
+      <c r="O8" t="str">
         <v>367</v>
       </c>
-      <c r="P8">
+      <c r="P8" t="str">
         <v>1415</v>
       </c>
     </row>
@@ -833,7 +815,7 @@
       <c r="C9" t="str">
         <v>Male</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="str">
         <v>36</v>
       </c>
       <c r="E9" t="str">
@@ -863,13 +845,13 @@
       <c r="M9" t="str">
         <v>Schedule an urgent consultation with the healthcare provider for asthma management. | Consider emergency evaluation if breathing difficulties increase or oxygen levels drop. | Follow up regularly to adjust care plans based on symptom progression.</v>
       </c>
-      <c r="N9">
+      <c r="N9" t="str">
         <v>1048</v>
       </c>
-      <c r="O9">
+      <c r="O9" t="str">
         <v>342</v>
       </c>
-      <c r="P9">
+      <c r="P9" t="str">
         <v>1390</v>
       </c>
     </row>
@@ -883,7 +865,7 @@
       <c r="C10" t="str">
         <v>Male</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="str">
         <v>36</v>
       </c>
       <c r="E10" t="str">
@@ -913,13 +895,13 @@
       <c r="M10" t="str">
         <v>Seek urgent consultation with a healthcare provider to assess current episode. | Consider scheduling a follow-up appointment for asthma management adjustment. | Prepare an emergency action plan including medication review and trigger avoidance.</v>
       </c>
-      <c r="N10">
+      <c r="N10" t="str">
         <v>1048</v>
       </c>
-      <c r="O10">
+      <c r="O10" t="str">
         <v>368</v>
       </c>
-      <c r="P10">
+      <c r="P10" t="str">
         <v>1416</v>
       </c>
     </row>
@@ -933,7 +915,7 @@
       <c r="C11" t="str">
         <v>Male</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="str">
         <v>36</v>
       </c>
       <c r="E11" t="str">
@@ -963,13 +945,13 @@
       <c r="M11" t="str">
         <v>Schedule a follow-up consultation with a pulmonologist or asthma specialist as soon as possible. | Consider immediate evaluation at emergency care if symptoms such as inability to talk or eat persist or worsen. | Maintain a symptom diary to track changes and report to care team regularly.</v>
       </c>
-      <c r="N11">
+      <c r="N11" t="str">
         <v>1048</v>
       </c>
-      <c r="O11">
+      <c r="O11" t="str">
         <v>413</v>
       </c>
-      <c r="P11">
+      <c r="P11" t="str">
         <v>1461</v>
       </c>
     </row>
@@ -983,7 +965,7 @@
       <c r="C12" t="str">
         <v>Male</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="str">
         <v>36</v>
       </c>
       <c r="E12" t="str">
@@ -1013,13 +995,13 @@
       <c r="M12" t="str">
         <v>Schedule urgent consultation with pulmonologist or emergency care provider. | Monitor breathing patterns and symptom severity throughout the day. | Prepare for possible immediate treatment based on symptom progression.</v>
       </c>
-      <c r="N12">
+      <c r="N12" t="str">
         <v>1048</v>
       </c>
-      <c r="O12">
+      <c r="O12" t="str">
         <v>352</v>
       </c>
-      <c r="P12">
+      <c r="P12" t="str">
         <v>1400</v>
       </c>
     </row>
@@ -1033,7 +1015,7 @@
       <c r="C13" t="str">
         <v>Male</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="str">
         <v>36</v>
       </c>
       <c r="E13" t="str">
@@ -1063,13 +1045,13 @@
       <c r="M13" t="str">
         <v>Schedule an urgent consultation with your healthcare provider to reassess asthma management. | Consider visiting emergency care if symptoms like inability to talk or severe breathlessness persist or worsen. | Monitor symptoms and vitals regularly and maintain communication with your care team.</v>
       </c>
-      <c r="N13">
+      <c r="N13" t="str">
         <v>1048</v>
       </c>
-      <c r="O13">
+      <c r="O13" t="str">
         <v>389</v>
       </c>
-      <c r="P13">
+      <c r="P13" t="str">
         <v>1437</v>
       </c>
     </row>
@@ -1083,7 +1065,7 @@
       <c r="C14" t="str">
         <v>Male</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="str">
         <v>36</v>
       </c>
       <c r="E14" t="str">
@@ -1113,13 +1095,13 @@
       <c r="M14" t="str">
         <v>Schedule an immediate follow-up appointment with your asthma specialist. | Consider visiting an emergency facility if symptoms such as inability to talk or eat worsen. | Continue monitoring vitals and symptom severity closely at home.</v>
       </c>
-      <c r="N14">
+      <c r="N14" t="str">
         <v>1048</v>
       </c>
-      <c r="O14">
+      <c r="O14" t="str">
         <v>386</v>
       </c>
-      <c r="P14">
+      <c r="P14" t="str">
         <v>1434</v>
       </c>
     </row>
@@ -1133,7 +1115,7 @@
       <c r="C15" t="str">
         <v>Male</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="str">
         <v>36</v>
       </c>
       <c r="E15" t="str">
@@ -1163,13 +1145,13 @@
       <c r="M15" t="str">
         <v>Schedule an urgent consultation with a healthcare provider or asthma specialist. | Consider visiting the emergency room if symptoms worsen, especially inability to speak or eat, or worsening breathing difficulty. | Monitor symptoms closely and maintain regular vital sign checks. | Avoid known asthma triggers and prepare for possible lab tests or inhaler adjustments as directed by a healthcare professional.</v>
       </c>
-      <c r="N15">
+      <c r="N15" t="str">
         <v>1056</v>
       </c>
-      <c r="O15">
+      <c r="O15" t="str">
         <v>391</v>
       </c>
-      <c r="P15">
+      <c r="P15" t="str">
         <v>1447</v>
       </c>
     </row>
@@ -1183,7 +1165,7 @@
       <c r="C16" t="str">
         <v>Male</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="str">
         <v>36</v>
       </c>
       <c r="E16" t="str">
@@ -1213,13 +1195,13 @@
       <c r="M16" t="str">
         <v>Urgent evaluation by respiratory specialist is recommended. | Continuous monitoring of oxygen saturation and respiratory status. | Consider referral to emergency care if symptoms fail to improve or worsen. | Educate patient on recognizing early warning signs of severe asthma exacerbations.</v>
       </c>
-      <c r="N16">
+      <c r="N16" t="str">
         <v>1138</v>
       </c>
-      <c r="O16">
+      <c r="O16" t="str">
         <v>407</v>
       </c>
-      <c r="P16">
+      <c r="P16" t="str">
         <v>1545</v>
       </c>
     </row>
@@ -1233,7 +1215,7 @@
       <c r="C17" t="str">
         <v>Male</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="str">
         <v>36</v>
       </c>
       <c r="E17" t="str">
@@ -1263,13 +1245,13 @@
       <c r="M17" t="str">
         <v>Schedule a follow-up consultation with your healthcare provider and review asthma action plan.</v>
       </c>
-      <c r="N17">
+      <c r="N17" t="str">
         <v>1048</v>
       </c>
-      <c r="O17">
+      <c r="O17" t="str">
         <v>236</v>
       </c>
-      <c r="P17">
+      <c r="P17" t="str">
         <v>1284</v>
       </c>
       <c r="Q17" t="str">
@@ -1286,7 +1268,7 @@
       <c r="C18" t="str">
         <v>Male</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="str">
         <v>36</v>
       </c>
       <c r="G18" t="str">
@@ -1310,13 +1292,13 @@
       <c r="M18" t="str">
         <v>Schedule a follow-up appointment with a healthcare provider. | Keep a daily log of any symptoms or changes in health. | Engage in scheduled activities and try to maintain a structured routine.</v>
       </c>
-      <c r="N18">
+      <c r="N18" t="str">
         <v>1079</v>
       </c>
-      <c r="O18">
+      <c r="O18" t="str">
         <v>290</v>
       </c>
-      <c r="P18">
+      <c r="P18" t="str">
         <v>1369</v>
       </c>
       <c r="Q18" t="str">
@@ -1333,7 +1315,7 @@
       <c r="C19" t="str">
         <v>Male</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="str">
         <v>36</v>
       </c>
       <c r="G19" t="str">
@@ -1357,13 +1339,13 @@
       <c r="M19" t="str">
         <v>Schedule a follow-up appointment to further assess the episodes of confusion. | Monitor daily activities and symptoms closely.</v>
       </c>
-      <c r="N19">
+      <c r="N19" t="str">
         <v>1079</v>
       </c>
-      <c r="O19">
+      <c r="O19" t="str">
         <v>261</v>
       </c>
-      <c r="P19">
+      <c r="P19" t="str">
         <v>1340</v>
       </c>
       <c r="Q19" t="str">
@@ -1380,7 +1362,7 @@
       <c r="C20" t="str">
         <v>Male</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="str">
         <v>36</v>
       </c>
       <c r="G20" t="str">
@@ -1404,13 +1386,13 @@
       <c r="M20" t="str">
         <v>Schedule a follow-up appointment in two weeks. | Monitor symptoms closely and seek help if they worsen.</v>
       </c>
-      <c r="N20">
+      <c r="N20" t="str">
         <v>1079</v>
       </c>
-      <c r="O20">
+      <c r="O20" t="str">
         <v>204</v>
       </c>
-      <c r="P20">
+      <c r="P20" t="str">
         <v>1283</v>
       </c>
       <c r="Q20" t="str">
@@ -1427,7 +1409,7 @@
       <c r="C21" t="str">
         <v>Male</v>
       </c>
-      <c r="D21">
+      <c r="D21" t="str">
         <v>36</v>
       </c>
       <c r="G21" t="str">
@@ -1451,13 +1433,13 @@
       <c r="M21" t="str">
         <v>Keep a daily log of symptoms and vital signs for further assessment. | Schedule a follow-up appointment with the healthcare provider next week.</v>
       </c>
-      <c r="N21">
+      <c r="N21" t="str">
         <v>1079</v>
       </c>
-      <c r="O21">
+      <c r="O21" t="str">
         <v>220</v>
       </c>
-      <c r="P21">
+      <c r="P21" t="str">
         <v>1299</v>
       </c>
       <c r="Q21" t="str">
@@ -1474,7 +1456,7 @@
       <c r="C22" t="str">
         <v>Male</v>
       </c>
-      <c r="D22">
+      <c r="D22" t="str">
         <v>36</v>
       </c>
       <c r="G22" t="str">
@@ -1498,13 +1480,13 @@
       <c r="M22" t="str">
         <v>Schedule a follow-up appointment for ongoing assessment.</v>
       </c>
-      <c r="N22">
+      <c r="N22" t="str">
         <v>1079</v>
       </c>
-      <c r="O22">
+      <c r="O22" t="str">
         <v>203</v>
       </c>
-      <c r="P22">
+      <c r="P22" t="str">
         <v>1282</v>
       </c>
       <c r="Q22" t="str">
@@ -1521,7 +1503,7 @@
       <c r="C23" t="str">
         <v>Male</v>
       </c>
-      <c r="D23">
+      <c r="D23" t="str">
         <v>36</v>
       </c>
       <c r="G23" t="str">
@@ -1545,13 +1527,13 @@
       <c r="M23" t="str">
         <v>Schedule a follow-up appointment with the healthcare provider in the next month. | Maintain a daily log of symptoms and vital signs to discuss in the next visit.</v>
       </c>
-      <c r="N23">
+      <c r="N23" t="str">
         <v>1079</v>
       </c>
-      <c r="O23">
+      <c r="O23" t="str">
         <v>273</v>
       </c>
-      <c r="P23">
+      <c r="P23" t="str">
         <v>1352</v>
       </c>
       <c r="Q23" t="str">
@@ -1568,7 +1550,7 @@
       <c r="C24" t="str">
         <v>Male</v>
       </c>
-      <c r="D24">
+      <c r="D24" t="str">
         <v>36</v>
       </c>
       <c r="G24" t="str">
@@ -1592,13 +1574,13 @@
       <c r="M24" t="str">
         <v>Schedule a follow-up appointment to review progress and address any remaining concerns.</v>
       </c>
-      <c r="N24">
+      <c r="N24" t="str">
         <v>771</v>
       </c>
-      <c r="O24">
+      <c r="O24" t="str">
         <v>214</v>
       </c>
-      <c r="P24">
+      <c r="P24" t="str">
         <v>985</v>
       </c>
       <c r="Q24" t="str">
@@ -1618,7 +1600,7 @@
       <c r="C25" t="str">
         <v>Male</v>
       </c>
-      <c r="D25">
+      <c r="D25" t="str">
         <v>36</v>
       </c>
       <c r="G25" t="str">
@@ -1642,13 +1624,13 @@
       <c r="M25" t="str">
         <v>Maintain regular check-ins with the care team. | Continue daily monitoring of vitals and symptoms. | Schedule a follow-up appointment in two weeks to review progress.</v>
       </c>
-      <c r="N25">
+      <c r="N25" t="str">
         <v>2423</v>
       </c>
-      <c r="O25">
+      <c r="O25" t="str">
         <v>309</v>
       </c>
-      <c r="P25">
+      <c r="P25" t="str">
         <v>2732</v>
       </c>
       <c r="Q25" t="str">
@@ -1668,7 +1650,7 @@
       <c r="C26" t="str">
         <v>Male</v>
       </c>
-      <c r="D26">
+      <c r="D26" t="str">
         <v>36</v>
       </c>
       <c r="G26" t="str">
@@ -1692,13 +1674,13 @@
       <c r="M26" t="str">
         <v>Schedule a follow-up appointment to reassess vitals and symptoms. | Consider a consultation with a nutritionist for tailored dietary recommendations.</v>
       </c>
-      <c r="N26">
+      <c r="N26" t="str">
         <v>2423</v>
       </c>
-      <c r="O26">
+      <c r="O26" t="str">
         <v>353</v>
       </c>
-      <c r="P26">
+      <c r="P26" t="str">
         <v>2776</v>
       </c>
       <c r="Q26" t="str">
@@ -1718,7 +1700,7 @@
       <c r="C27" t="str">
         <v>Male</v>
       </c>
-      <c r="D27">
+      <c r="D27" t="str">
         <v>36</v>
       </c>
       <c r="G27" t="str">
@@ -1742,13 +1724,13 @@
       <c r="M27" t="str">
         <v>Schedule a follow-up consultation next month to review progress and adjust care plan as necessary. | Consider nutritional counseling to optimize diet and further stabilize blood sugar levels.</v>
       </c>
-      <c r="N27">
+      <c r="N27" t="str">
         <v>2366</v>
       </c>
-      <c r="O27">
+      <c r="O27" t="str">
         <v>331</v>
       </c>
-      <c r="P27">
+      <c r="P27" t="str">
         <v>2697</v>
       </c>
       <c r="Q27" t="str">
@@ -1768,7 +1750,7 @@
       <c r="C28" t="str">
         <v>Male</v>
       </c>
-      <c r="D28">
+      <c r="D28" t="str">
         <v>36</v>
       </c>
       <c r="G28" t="str">
@@ -1792,13 +1774,13 @@
       <c r="M28" t="str">
         <v>Urgent medical evaluation recommended, follow-up appointment with a specialist.</v>
       </c>
-      <c r="N28">
+      <c r="N28" t="str">
         <v>2366</v>
       </c>
-      <c r="O28">
+      <c r="O28" t="str">
         <v>174</v>
       </c>
-      <c r="P28">
+      <c r="P28" t="str">
         <v>2540</v>
       </c>
       <c r="Q28" t="str">
@@ -1818,7 +1800,7 @@
       <c r="C29" t="str">
         <v>Male</v>
       </c>
-      <c r="D29">
+      <c r="D29" t="str">
         <v>36</v>
       </c>
       <c r="G29" t="str">
@@ -1842,13 +1824,13 @@
       <c r="M29" t="str">
         <v>Log vitals at the same time each morning, preferably before breakfast for clearer fasting readings. | Add meal and activity logs more consistently this week. | Maintain alcohol recovery supports and routine. | Schedule a routine check-in within 2–4 weeks to review progress and fasting glucose. | Seek care sooner if any red flags occur: confusion suddenly worse, severe shaking, chest pain, shortness of breath, SpO2 &lt;94%, fever ≥100.4 F, repeated BP &gt;140/90, or resting HR &gt;100.</v>
       </c>
-      <c r="N29">
+      <c r="N29" t="str">
         <v>2422</v>
       </c>
-      <c r="O29">
+      <c r="O29" t="str">
         <v>3613</v>
       </c>
-      <c r="P29">
+      <c r="P29" t="str">
         <v>6035</v>
       </c>
       <c r="Q29" t="str">
@@ -1868,7 +1850,7 @@
       <c r="C30" t="str">
         <v>Male</v>
       </c>
-      <c r="D30">
+      <c r="D30" t="str">
         <v>36</v>
       </c>
       <c r="E30" t="str">
@@ -1898,13 +1880,13 @@
       <c r="M30" t="str">
         <v>If shortness of breath is severe, new, or occurs with chest pain, blue lips, fainting, or SpO2 at 92% or lower, call emergency services now. | If shortness of breath returns or lasts more than a few minutes, arrange same-day or next-day care. | Schedule a primary care visit in the next 1–2 weeks to review breathing and attention concerns. | Record any new breathing episodes with time, activity, and SpO2 if available. | Continue daily vitals at about the same time each morning for trend tracking. | Set reminders for important tasks and appointments to reduce the impact of forgetfulness.</v>
       </c>
-      <c r="N30">
+      <c r="N30" t="str">
         <v>2353</v>
       </c>
-      <c r="O30">
+      <c r="O30" t="str">
         <v>3503</v>
       </c>
-      <c r="P30">
+      <c r="P30" t="str">
         <v>5856</v>
       </c>
       <c r="Q30" t="str">
@@ -1924,7 +1906,7 @@
       <c r="C31" t="str">
         <v>Male</v>
       </c>
-      <c r="D31">
+      <c r="D31" t="str">
         <v>36</v>
       </c>
       <c r="E31" t="str">
@@ -1954,13 +1936,13 @@
       <c r="M31" t="str">
         <v>If shortness of breath is severe, new, or occurs with chest pain, blue lips, fainting, or SpO2 at 92% or lower, call emergency services now. | If shortness of breath returns or lasts more than a few minutes, arrange same-day or next-day care. | Schedule a primary care visit in the next 1–2 weeks to review breathing and attention concerns. | Record any new breathing episodes with time, activity, and SpO2 if available. | Continue daily vitals at about the same time each morning for trend tracking. | Set reminders for important tasks and appointments to reduce the impact of forgetfulness.</v>
       </c>
-      <c r="N31">
+      <c r="N31" t="str">
         <v>2353</v>
       </c>
-      <c r="O31">
+      <c r="O31" t="str">
         <v>3503</v>
       </c>
-      <c r="P31">
+      <c r="P31" t="str">
         <v>5856</v>
       </c>
       <c r="Q31" t="str">
@@ -1980,7 +1962,7 @@
       <c r="C32" t="str">
         <v>Male</v>
       </c>
-      <c r="D32">
+      <c r="D32" t="str">
         <v>36</v>
       </c>
       <c r="E32" t="str">
@@ -2010,13 +1992,13 @@
       <c r="M32" t="str">
         <v>Schedule a follow-up appointment with a healthcare provider to discuss shortness of breath. | Consider a cognitive assessment regarding ADHD symptoms.</v>
       </c>
-      <c r="N32">
+      <c r="N32" t="str">
         <v>2354</v>
       </c>
-      <c r="O32">
+      <c r="O32" t="str">
         <v>340</v>
       </c>
-      <c r="P32">
+      <c r="P32" t="str">
         <v>2694</v>
       </c>
       <c r="Q32" t="str">
@@ -2036,7 +2018,7 @@
       <c r="C33" t="str">
         <v>Male</v>
       </c>
-      <c r="D33">
+      <c r="D33" t="str">
         <v>36</v>
       </c>
       <c r="E33" t="str">
@@ -2066,13 +2048,13 @@
       <c r="M33" t="str">
         <v>Schedule a follow-up appointment with a healthcare provider to discuss shortness of breath. | Consider a cognitive assessment regarding ADHD symptoms.</v>
       </c>
-      <c r="N33">
+      <c r="N33" t="str">
         <v>2354</v>
       </c>
-      <c r="O33">
+      <c r="O33" t="str">
         <v>340</v>
       </c>
-      <c r="P33">
+      <c r="P33" t="str">
         <v>2694</v>
       </c>
       <c r="Q33" t="str">
@@ -2092,7 +2074,7 @@
       <c r="C34" t="str">
         <v>Male</v>
       </c>
-      <c r="D34">
+      <c r="D34" t="str">
         <v>36</v>
       </c>
       <c r="E34" t="str">
@@ -2122,13 +2104,13 @@
       <c r="M34" t="str">
         <v>Schedule an appointment with a healthcare provider to discuss shortness of breath and its management. | Follow up on blood sugar monitoring and consider dietary adjustments.</v>
       </c>
-      <c r="N34">
+      <c r="N34" t="str">
         <v>2354</v>
       </c>
-      <c r="O34">
+      <c r="O34" t="str">
         <v>407</v>
       </c>
-      <c r="P34">
+      <c r="P34" t="str">
         <v>2761</v>
       </c>
       <c r="Q34" t="str">
@@ -2148,7 +2130,7 @@
       <c r="C35" t="str">
         <v>Male</v>
       </c>
-      <c r="D35">
+      <c r="D35" t="str">
         <v>36</v>
       </c>
       <c r="E35" t="str">
@@ -2178,13 +2160,13 @@
       <c r="M35" t="str">
         <v>Schedule an appointment with a healthcare provider to discuss shortness of breath and its management. | Follow up on blood sugar monitoring and consider dietary adjustments.</v>
       </c>
-      <c r="N35">
+      <c r="N35" t="str">
         <v>2354</v>
       </c>
-      <c r="O35">
+      <c r="O35" t="str">
         <v>407</v>
       </c>
-      <c r="P35">
+      <c r="P35" t="str">
         <v>2761</v>
       </c>
       <c r="Q35" t="str">
@@ -2204,7 +2186,7 @@
       <c r="C36" t="str">
         <v>Male</v>
       </c>
-      <c r="D36">
+      <c r="D36" t="str">
         <v>36</v>
       </c>
       <c r="E36" t="str">
@@ -2234,13 +2216,13 @@
       <c r="M36" t="str">
         <v>Schedule a medical consultation to discuss shortness of breath management. | Implement strategies for improved daily activity adherence, such as setting up alarms or reminders.</v>
       </c>
-      <c r="N36">
+      <c r="N36" t="str">
         <v>2479</v>
       </c>
-      <c r="O36">
+      <c r="O36" t="str">
         <v>316</v>
       </c>
-      <c r="P36">
+      <c r="P36" t="str">
         <v>2795</v>
       </c>
       <c r="Q36" t="str">
@@ -2260,7 +2242,7 @@
       <c r="C37" t="str">
         <v>Male</v>
       </c>
-      <c r="D37">
+      <c r="D37" t="str">
         <v>36</v>
       </c>
       <c r="E37" t="str">
@@ -2290,13 +2272,13 @@
       <c r="M37" t="str">
         <v>Schedule a medical consultation to discuss shortness of breath management. | Implement strategies for improved daily activity adherence, such as setting up alarms or reminders.</v>
       </c>
-      <c r="N37">
+      <c r="N37" t="str">
         <v>2479</v>
       </c>
-      <c r="O37">
+      <c r="O37" t="str">
         <v>316</v>
       </c>
-      <c r="P37">
+      <c r="P37" t="str">
         <v>2795</v>
       </c>
       <c r="Q37" t="str">
@@ -2316,7 +2298,7 @@
       <c r="C38" t="str">
         <v>Male</v>
       </c>
-      <c r="D38">
+      <c r="D38" t="str">
         <v>36</v>
       </c>
       <c r="E38" t="str">
@@ -2346,13 +2328,13 @@
       <c r="M38" t="str">
         <v>Continue monitoring vital signs daily. | Schedule a follow-up appointment with your care team in one month. | Keep a diary of any unusual symptoms for future discussions with your doctor.</v>
       </c>
-      <c r="N38">
+      <c r="N38" t="str">
         <v>2406</v>
       </c>
-      <c r="O38">
+      <c r="O38" t="str">
         <v>359</v>
       </c>
-      <c r="P38">
+      <c r="P38" t="str">
         <v>2765</v>
       </c>
       <c r="Q38" t="str">
@@ -2372,7 +2354,7 @@
       <c r="C39" t="str">
         <v>Male</v>
       </c>
-      <c r="D39">
+      <c r="D39" t="str">
         <v>36</v>
       </c>
       <c r="E39" t="str">
@@ -2402,13 +2384,13 @@
       <c r="M39" t="str">
         <v>Schedule an appointment with a healthcare provider to discuss shortness of breath. | Conduct a follow-up assessment of ADHD symptoms with the care team. | Implement the recommended lifestyle changes and monitor progress.</v>
       </c>
-      <c r="N39">
+      <c r="N39" t="str">
         <v>2479</v>
       </c>
-      <c r="O39">
+      <c r="O39" t="str">
         <v>413</v>
       </c>
-      <c r="P39">
+      <c r="P39" t="str">
         <v>2892</v>
       </c>
       <c r="Q39" t="str">
@@ -2428,7 +2410,7 @@
       <c r="C40" t="str">
         <v>Male</v>
       </c>
-      <c r="D40">
+      <c r="D40" t="str">
         <v>36</v>
       </c>
       <c r="E40" t="str">
@@ -2458,13 +2440,13 @@
       <c r="M40" t="str">
         <v>Schedule an appointment with a healthcare provider to discuss shortness of breath. | Conduct a follow-up assessment of ADHD symptoms with the care team. | Implement the recommended lifestyle changes and monitor progress.</v>
       </c>
-      <c r="N40">
+      <c r="N40" t="str">
         <v>2479</v>
       </c>
-      <c r="O40">
+      <c r="O40" t="str">
         <v>413</v>
       </c>
-      <c r="P40">
+      <c r="P40" t="str">
         <v>2892</v>
       </c>
       <c r="Q40" t="str">
@@ -2474,9 +2456,65 @@
         <v>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","status":"suspected","symptom_lookup_id":"56f51f54-0b28-4e3a-b5ca-1344f2f2cc4a","symptom_title":"short of breath","symptoms":[{"records":[{"severity":6,"recorded_at":"2026-02-12T11:22:02.375Z"},{"severity":7,"recorded_at":"2026-02-11T09:18:17.203Z"},{"severity":8,"recorded_at":"2026-02-10T08:18:17.203Z"},{"severity":10,"recorded_at":"2026-02-09T07:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-08T11:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-07T06:30:15.500Z"}],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","status":"suspected","symptom_lookup_id":"cc50560b-a35e-4315-9856-7c693335dbb0","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[{"severity":7,"recorded_at":"2026-02-12T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-11T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-10T07:35:35.042Z"},{"severity":4,"recorded_at":"2026-02-09T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-08T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-07T07:35:35.042Z"},{"severity":7,"recorded_at":"2026-02-06T07:35:35.042Z"}],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"118/78"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"122/82"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"120/80"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"121/79"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"119/81"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"120/80"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"123/81"}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"68"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"72"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"70"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"71"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"69"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"70"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"97"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"99"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"97"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"98.4"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"98.6"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98.5"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"98.6"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"98.4"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"98.5"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"timestamp":"2026-02-03T08:15:00.000Z","value":"95"},{"timestamp":"2026-02-04T08:20:00.000Z","value":"102"},{"timestamp":"2026-02-05T08:10:00.000Z","value":"98"},{"timestamp":"2026-02-06T08:25:00.000Z","value":"105"},{"timestamp":"2026-02-07T08:30:00.000Z","value":"99"},{"timestamp":"2026-02-08T08:18:00.000Z","value":"100"},{"timestamp":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2026-02-12T08:16:21.058Z</v>
+      </c>
+      <c r="B41" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D41" t="str">
+        <v>36</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Alcohol Withdrawal</v>
+      </c>
+      <c r="F41" t="str">
+        <v>6985cb0d41eeb53a74254efe</v>
+      </c>
+      <c r="G41" t="str">
+        <v>John Doe has shown improvement after recovering from alcohol withdrawal. Most vital signs are stable, but monitoring continues.</v>
+      </c>
+      <c r="H41" t="str">
+        <v>LOW: Mild confusion and sweating were noted but are improving.</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Blood Pressure: Stable around 120/80 mmHg. | Heart Rate: Ranging from 68 to 73 bpm, consistent. | SpO2: Levels are between 97% and 99%, indicating good oxygenation. | Body Temperature: Normal, between 98.4°F and 98.6°F. | Blood Sugar: Mostly within normal range, fluctuating slightly.</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Regular meals and light exercise contribute positively to overall well-being. | Increased sweating linked to stress or anxiety; maintaining hydration recommended.</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Incorporate more fruits and vegetables into daily meals. | Practice relaxation techniques to manage stress and reduce sweating. | Stay hydrated, especially during activities.</v>
+      </c>
+      <c r="L41" t="str">
+        <v>Continue monitoring symptoms of confusion and sweating. | Follow up in one month to reassess health status.</v>
+      </c>
+      <c r="M41" t="str">
+        <v>Schedule a follow-up appointment with your healthcare provider. | Consider joining a support group for ongoing recovery.</v>
+      </c>
+      <c r="N41" t="str">
+        <v>2538</v>
+      </c>
+      <c r="O41" t="str">
+        <v>302</v>
+      </c>
+      <c r="P41" t="str">
+        <v>2840</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+      <c r="R41" t="str">
+        <v>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-04T08:20:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-05T08:10:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-06T08:25:00.000Z","value":{"systolic":121,"diastolic":79}},{"recorded_at":"2026-02-07T08:30:00.000Z","value":{"systolic":119,"diastolic":81}},{"recorded_at":"2026-02-08T08:18:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-09T08:22:00.000Z","value":{"systolic":123,"diastolic":81}}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"68"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"72"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"70"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"71"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"69"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"70"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"97"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"99"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"97"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"98.4"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98.6"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98.5"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"98.6"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"98.4"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98.5"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"95"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"102"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"105"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"99"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"100"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R41"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor health record management by updating condition normalization in index.js. Revised output.json to reflect a detailed health summary, including new symptoms and vital signs monitoring. Removed unused PDF generation code and adjusted package dependencies accordingly.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -397,7 +397,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R43"/>
+  <cols>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="30.83203125" customWidth="1"/>
+    <col min="7" max="7" width="50.83203125" customWidth="1"/>
+    <col min="8" max="8" width="60.83203125" customWidth="1"/>
+    <col min="9" max="9" width="60.83203125" customWidth="1"/>
+    <col min="10" max="10" width="60.83203125" customWidth="1"/>
+    <col min="11" max="11" width="60.83203125" customWidth="1"/>
+    <col min="12" max="12" width="60.83203125" customWidth="1"/>
+    <col min="13" max="13" width="60.83203125" customWidth="1"/>
+    <col min="14" max="14" width="15.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2512,9 +2530,121 @@
         <v>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-04T08:20:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-05T08:10:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-06T08:25:00.000Z","value":{"systolic":121,"diastolic":79}},{"recorded_at":"2026-02-07T08:30:00.000Z","value":{"systolic":119,"diastolic":81}},{"recorded_at":"2026-02-08T08:18:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-09T08:22:00.000Z","value":{"systolic":123,"diastolic":81}}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"68"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"72"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"70"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"71"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"69"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"70"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"97"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"99"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"97"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"98.4"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98.6"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98.5"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"98.6"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"98.4"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98.5"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"95"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"102"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"105"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"99"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"100"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2026-02-12T08:18:18.891Z</v>
+      </c>
+      <c r="B42" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D42">
+        <v>36</v>
+      </c>
+      <c r="E42" t="str">
+        <v>short of breath</v>
+      </c>
+      <c r="F42" t="str">
+        <v>6985cdf941eeb53a74254f5f</v>
+      </c>
+      <c r="G42" t="str">
+        <v>John Doe, a 36-year-old male, exhibits symptoms of shortness of breath and suspected ADHD-related forgetfulness. Monitoring of vital signs shows consistent readings, but attention to shortness of breath is advised.</v>
+      </c>
+      <c r="H42" t="str">
+        <v>HIGH: Shortness of breath severity has reached an alarming level. Immediate assessment is recommended.</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Blood Pressure: Stable, consistently around 120/80 mmHg. | Heart Rate: Generally stable ranging from 68 to 73 bpm. | SpO2: Remained steady between 97% and 99%. | Body Temperature: Consistent normal range between 98.4°F and 98.6°F. | Blood Sugar: Minor fluctuations observed, mostly within normal range.</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Routine meals occurring regularly with breakfast being the most frequent activity. | Activity levels include light exercise and morning walks which may help improve overall well-being.</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Engage in a breathing exercise regimen to alleviate shortness of breath. | Maintain a consistent eating schedule to support blood sugar levels. | Consider mindfulness activities to help manage ADHD symptoms.</v>
+      </c>
+      <c r="L42" t="str">
+        <v>Monitor shortness of breath severity and frequency closely. | Evaluate possible triggers for ADHD symptoms in daily activities.</v>
+      </c>
+      <c r="M42" t="str">
+        <v>Schedule a follow-up appointment for a thorough respiratory evaluation. | Consider a consultation with a mental health professional regarding ADHD.</v>
+      </c>
+      <c r="N42">
+        <v>2611</v>
+      </c>
+      <c r="O42">
+        <v>341</v>
+      </c>
+      <c r="P42">
+        <v>2952</v>
+      </c>
+      <c r="Q42" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+      <c r="R42" t="str">
+        <v>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","status":"suspected","symptom_lookup_id":"56f51f54-0b28-4e3a-b5ca-1344f2f2cc4a","symptom_title":"short of breath","symptoms":[{"records":[{"severity":6,"recorded_at":"2026-02-12T11:22:02.375Z"},{"severity":7,"recorded_at":"2026-02-11T09:18:17.203Z"},{"severity":8,"recorded_at":"2026-02-10T08:18:17.203Z"},{"severity":10,"recorded_at":"2026-02-09T07:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-08T11:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-07T06:30:15.500Z"}],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","status":"suspected","symptom_lookup_id":"cc50560b-a35e-4315-9856-7c693335dbb0","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[{"severity":7,"recorded_at":"2026-02-12T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-11T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-10T07:35:35.042Z"},{"severity":4,"recorded_at":"2026-02-09T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-08T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-07T07:35:35.042Z"},{"severity":7,"recorded_at":"2026-02-06T07:35:35.042Z"}],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-04T08:20:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-05T08:10:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-06T08:25:00.000Z","value":{"systolic":121,"diastolic":79}},{"recorded_at":"2026-02-07T08:30:00.000Z","value":{"systolic":119,"diastolic":81}},{"recorded_at":"2026-02-08T08:18:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-09T08:22:00.000Z","value":{"systolic":123,"diastolic":81}}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"68"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"72"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"70"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"71"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"69"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"70"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"97"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"99"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"97"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"98.4"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98.6"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98.5"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"98.6"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"98.4"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98.5"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"95"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"102"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"105"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"99"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"100"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2026-02-12T08:18:18.891Z</v>
+      </c>
+      <c r="B43" t="str">
+        <v>John Doe</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Male</v>
+      </c>
+      <c r="D43">
+        <v>36</v>
+      </c>
+      <c r="E43" t="str">
+        <v>ADHD-is forgetful in daily activities.(0-4)</v>
+      </c>
+      <c r="F43" t="str">
+        <v>698d82c7bb05e0b7c13a1f34</v>
+      </c>
+      <c r="G43" t="str">
+        <v>John Doe, a 36-year-old male, exhibits symptoms of shortness of breath and suspected ADHD-related forgetfulness. Monitoring of vital signs shows consistent readings, but attention to shortness of breath is advised.</v>
+      </c>
+      <c r="H43" t="str">
+        <v>HIGH: Shortness of breath severity has reached an alarming level. Immediate assessment is recommended.</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Blood Pressure: Stable, consistently around 120/80 mmHg. | Heart Rate: Generally stable ranging from 68 to 73 bpm. | SpO2: Remained steady between 97% and 99%. | Body Temperature: Consistent normal range between 98.4°F and 98.6°F. | Blood Sugar: Minor fluctuations observed, mostly within normal range.</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Routine meals occurring regularly with breakfast being the most frequent activity. | Activity levels include light exercise and morning walks which may help improve overall well-being.</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Engage in a breathing exercise regimen to alleviate shortness of breath. | Maintain a consistent eating schedule to support blood sugar levels. | Consider mindfulness activities to help manage ADHD symptoms.</v>
+      </c>
+      <c r="L43" t="str">
+        <v>Monitor shortness of breath severity and frequency closely. | Evaluate possible triggers for ADHD symptoms in daily activities.</v>
+      </c>
+      <c r="M43" t="str">
+        <v>Schedule a follow-up appointment for a thorough respiratory evaluation. | Consider a consultation with a mental health professional regarding ADHD.</v>
+      </c>
+      <c r="N43">
+        <v>2611</v>
+      </c>
+      <c r="O43">
+        <v>341</v>
+      </c>
+      <c r="P43">
+        <v>2952</v>
+      </c>
+      <c r="Q43" t="str">
+        <v>gpt-4o-mini</v>
+      </c>
+      <c r="R43" t="str">
+        <v>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","status":"suspected","symptom_lookup_id":"56f51f54-0b28-4e3a-b5ca-1344f2f2cc4a","symptom_title":"short of breath","symptoms":[{"records":[{"severity":6,"recorded_at":"2026-02-12T11:22:02.375Z"},{"severity":7,"recorded_at":"2026-02-11T09:18:17.203Z"},{"severity":8,"recorded_at":"2026-02-10T08:18:17.203Z"},{"severity":10,"recorded_at":"2026-02-09T07:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-08T11:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-07T06:30:15.500Z"}],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","status":"suspected","symptom_lookup_id":"cc50560b-a35e-4315-9856-7c693335dbb0","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[{"severity":7,"recorded_at":"2026-02-12T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-11T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-10T07:35:35.042Z"},{"severity":4,"recorded_at":"2026-02-09T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-08T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-07T07:35:35.042Z"},{"severity":7,"recorded_at":"2026-02-06T07:35:35.042Z"}],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-04T08:20:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-05T08:10:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-06T08:25:00.000Z","value":{"systolic":121,"diastolic":79}},{"recorded_at":"2026-02-07T08:30:00.000Z","value":{"systolic":119,"diastolic":81}},{"recorded_at":"2026-02-08T08:18:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-09T08:22:00.000Z","value":{"systolic":123,"diastolic":81}}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"68"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"72"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"70"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"71"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"69"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"70"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"97"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"99"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"97"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"98.4"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98.6"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98.5"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"98.6"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"98.4"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98.5"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"95"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"102"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"105"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"99"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"100"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update health records and model configuration. Changed model in index.js to 'gpt-5' for improved performance. Revised output.json to provide a more detailed and actionable health summary, including updated health alerts, vital signs, daily patterns, and care team notes. Enhanced token usage metrics for better tracking.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="676" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="412">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1199,6 +1199,54 @@
   </si>
   <si>
     <t>Schedule an appointment with the healthcare provider for evaluation of respiratory issues. | Review ADHD management plan.</t>
+  </si>
+  <si>
+    <t>2026-02-12T08:23:45.627Z</t>
+  </si>
+  <si>
+    <t>John Doe is a 36-year-old male experiencing symptoms of shortness of breath and forgetfulness associated with suspected ADHD. Monitoring vital signs shows generally stable readings but highlights the need for further attention to breathing difficulties.</t>
+  </si>
+  <si>
+    <t>HIGH: Severe shortness of breath detected. Recommend urgent medical evaluation.</t>
+  </si>
+  <si>
+    <t>Blood pressure remains stable with values around 120/80. | Heart rate averages 70 beats per minute, which is within normal range. | SpO2 levels are good, consistently above 97%. | Body temperature is normal, averaging 98.5°F. | Blood sugar levels are generally stable but show some fluctuations, especially with a peak at 105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular meal times and light exercise are integrated into the daily routine. | Shortness of breath severity was higher on days with increased activity.</t>
+  </si>
+  <si>
+    <t>Incorporate breathing exercises into daily routine to help manage shortness of breath. | Maintain a balanced diet, focusing on low-sugar foods to stabilize blood sugar levels.</t>
+  </si>
+  <si>
+    <t>Monitor severity of shortness of breath closely. | Consider further assessment for ADHD-related symptoms.</t>
+  </si>
+  <si>
+    <t>Schedule an appointment with a healthcare provider for breathing evaluation. | Discuss cognitive strategies for managing forgetfulness.</t>
+  </si>
+  <si>
+    <t>2026-02-12T10:06:16.924Z</t>
+  </si>
+  <si>
+    <t>Vitals are stable and in normal ranges. Shortness of breath spiked on Feb 9 and has improved but is still present. Attention/forgetfulness remains moderate to high. Monitor closely and arrange follow-up.</t>
+  </si>
+  <si>
+    <t>HIGH: Severe shortness of breath reported on Feb 9 with ongoing moderate episodes. Seek urgent care now if breathing is severe, happens at rest, gets worse, or comes with chest pain, fainting, blue/gray lips or face, confusion, or SpO2 under 92%. | MEDIUM: Repeated shortness of breath over several days despite normal vitals. Needs same‑week medical review.</t>
+  </si>
+  <si>
+    <t>Blood pressure 119–123 / 79–81 mmHg: stable and normal. | Heart rate 68–73 bpm: steady resting range. | SpO2 97–99%: normal oxygen levels during recorded checks. | Body temperature 98.4–98.6°F: no fever pattern. | Blood sugar 95–105 mg/dL: near‑normal; keep noting whether readings are fasting or after meals.</t>
+  </si>
+  <si>
+    <t>Shortness of breath often logged in the morning to late morning; peak on Feb 9, then gradual improvement. | No clear link between recorded walks/light exercise and worse breathing on logged days. | Regular breakfasts noted; no consistent impact on blood sugar or vitals seen. | Symptoms may be influenced by morning factors (cold air, allergens, rush/stress). Track context with each entry.</t>
+  </si>
+  <si>
+    <t>During episodes, use slow deep breaths and pursed‑lip breathing (inhale through nose 2 counts, exhale through pursed lips 4 counts). | Warm up before activity, pace yourself, and avoid smoke, strong scents, and very cold air. Use a scarf over the mouth in cold weather. | Track triggers with each symptom: time, activity, location, allergens, stress, and meal timing. | If available, check and log SpO2 during symptoms. | Stay hydrated and avoid very large meals right before exertion. | For forgetfulness: use phone reminders and checklists, keep items in fixed spots, and set a simple daily routine. | Aim for a steady sleep schedule (7–9 hours) to support energy and focus. | Plan short, frequent movement breaks rather than long, intense sessions.</t>
+  </si>
+  <si>
+    <t>Vitals appear normal; breathing symptoms remain the main concern given the severe peak and persistence. | Recommend clinical assessment to evaluate lungs/airways and heart as appropriate. | Consider spirometry and objective breathing assessment if symptoms continue. | Review environmental/allergen exposures and recent illnesses. | Clarify context of glucose readings (fasting vs post‑meal) at next visit.</t>
+  </si>
+  <si>
+    <t>Book a same‑week appointment with your primary care clinician to review shortness of breath. | Go to urgent care or call emergency services now if severe breathing returns, or if there is chest pain, fainting, blue lips/face, confusion, or SpO2 under 92%. | Log each breathing episode with time, activity, environment, and SpO2 if available. | Continue daily vitals; add readings during or soon after symptoms when safe. | Discuss attention/forgetfulness at the next visit and ask about simple screening and support strategies. | Reassess symptoms and vitals trends in 1–2 weeks or sooner if they worsen.</t>
   </si>
 </sst>
 </file>
@@ -1575,7 +1623,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P49"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -3757,6 +3805,206 @@
         <v>2911</v>
       </c>
     </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>396</v>
+      </c>
+      <c r="B46" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46">
+        <v>36</v>
+      </c>
+      <c r="E46" t="s">
+        <v>302</v>
+      </c>
+      <c r="F46" t="s">
+        <v>303</v>
+      </c>
+      <c r="G46" t="s">
+        <v>397</v>
+      </c>
+      <c r="H46" t="s">
+        <v>398</v>
+      </c>
+      <c r="I46" t="s">
+        <v>399</v>
+      </c>
+      <c r="J46" t="s">
+        <v>400</v>
+      </c>
+      <c r="K46" t="s">
+        <v>401</v>
+      </c>
+      <c r="L46" t="s">
+        <v>402</v>
+      </c>
+      <c r="M46" t="s">
+        <v>403</v>
+      </c>
+      <c r="N46">
+        <v>2611</v>
+      </c>
+      <c r="O46">
+        <v>325</v>
+      </c>
+      <c r="P46">
+        <v>2936</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>396</v>
+      </c>
+      <c r="B47" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47">
+        <v>36</v>
+      </c>
+      <c r="E47" t="s">
+        <v>314</v>
+      </c>
+      <c r="F47" t="s">
+        <v>315</v>
+      </c>
+      <c r="G47" t="s">
+        <v>397</v>
+      </c>
+      <c r="H47" t="s">
+        <v>398</v>
+      </c>
+      <c r="I47" t="s">
+        <v>399</v>
+      </c>
+      <c r="J47" t="s">
+        <v>400</v>
+      </c>
+      <c r="K47" t="s">
+        <v>401</v>
+      </c>
+      <c r="L47" t="s">
+        <v>402</v>
+      </c>
+      <c r="M47" t="s">
+        <v>403</v>
+      </c>
+      <c r="N47">
+        <v>2611</v>
+      </c>
+      <c r="O47">
+        <v>325</v>
+      </c>
+      <c r="P47">
+        <v>2936</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>404</v>
+      </c>
+      <c r="B48" t="s">
+        <v>17</v>
+      </c>
+      <c r="C48" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48">
+        <v>36</v>
+      </c>
+      <c r="E48" t="s">
+        <v>302</v>
+      </c>
+      <c r="F48" t="s">
+        <v>303</v>
+      </c>
+      <c r="G48" t="s">
+        <v>405</v>
+      </c>
+      <c r="H48" t="s">
+        <v>406</v>
+      </c>
+      <c r="I48" t="s">
+        <v>407</v>
+      </c>
+      <c r="J48" t="s">
+        <v>408</v>
+      </c>
+      <c r="K48" t="s">
+        <v>409</v>
+      </c>
+      <c r="L48" t="s">
+        <v>410</v>
+      </c>
+      <c r="M48" t="s">
+        <v>411</v>
+      </c>
+      <c r="N48">
+        <v>2610</v>
+      </c>
+      <c r="O48">
+        <v>3104</v>
+      </c>
+      <c r="P48">
+        <v>5714</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>404</v>
+      </c>
+      <c r="B49" t="s">
+        <v>17</v>
+      </c>
+      <c r="C49" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49">
+        <v>36</v>
+      </c>
+      <c r="E49" t="s">
+        <v>314</v>
+      </c>
+      <c r="F49" t="s">
+        <v>315</v>
+      </c>
+      <c r="G49" t="s">
+        <v>405</v>
+      </c>
+      <c r="H49" t="s">
+        <v>406</v>
+      </c>
+      <c r="I49" t="s">
+        <v>407</v>
+      </c>
+      <c r="J49" t="s">
+        <v>408</v>
+      </c>
+      <c r="K49" t="s">
+        <v>409</v>
+      </c>
+      <c r="L49" t="s">
+        <v>410</v>
+      </c>
+      <c r="M49" t="s">
+        <v>411</v>
+      </c>
+      <c r="N49">
+        <v>2610</v>
+      </c>
+      <c r="O49">
+        <v>3104</v>
+      </c>
+      <c r="P49">
+        <v>5714</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Integrate PDF report generation in index.js and update health_records.xlsx. Enhanced output.json with refined health summaries, alerts, and recommendations for improved patient monitoring. Updated package.json and package-lock.json to include new dependencies for PDF generation.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="482">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1385,6 +1385,78 @@
   </si>
   <si>
     <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"lookup_id":"BLOOD_PRESSURE","vital_name":"Blood Pressure","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-04T08:20:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-05T08:10:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-06T08:25:00.000Z","value":{"systolic":121,"diastolic":79}},{"recorded_at":"2026-02-07T08:30:00.000Z","value":{"systolic":119,"diastolic":81}},{"recorded_at":"2026-02-08T08:18:00.000Z","value":{"systolic":120,"diastolic":80}},{"recorded_at":"2026-02-09T08:22:00.000Z","value":{"systolic":123,"diastolic":81}}]},{"lookup_id":"HEART_RATE","vital_name":"Heart Rate","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"68"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"72"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"70"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"71"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"69"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"70"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"73"}]},{"lookup_id":"SPO2","vital_name":"SpO2","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"97"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"99"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"97"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98"}]},{"lookup_id":"BODY_TEMPERATURE","vital_name":"Body Temperature","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"98.4"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"98.6"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98.5"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"98.6"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"98.4"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"98.5"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"98.6"}]},{"lookup_id":"BLOOD_SUGAR","vital_name":"Blood Sugar","records":[{"recorded_at":"2026-02-03T08:15:00.000Z","value":"95"},{"recorded_at":"2026-02-04T08:20:00.000Z","value":"102"},{"recorded_at":"2026-02-05T08:10:00.000Z","value":"98"},{"recorded_at":"2026-02-06T08:25:00.000Z","value":"105"},{"recorded_at":"2026-02-07T08:30:00.000Z","value":"99"},{"recorded_at":"2026-02-08T08:18:00.000Z","value":"100"},{"recorded_at":"2026-02-09T08:22:00.000Z","value":"103"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
+  </si>
+  <si>
+    <t>2026-02-13T09:52:07.023Z</t>
+  </si>
+  <si>
+    <t>John Doe has recovered from Alcohol Withdrawal. Vitals show stable conditions but monitor for any unusual symptoms.</t>
+  </si>
+  <si>
+    <t>LOW: No critical alerts found.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable around 120/80. | Heart Rate: Average around 70 beats per minute. | SpO2: Consistently above 97%. | Body Temperature: Normal range around 98.4°F. | Blood Sugar: Fluctuating, mostly within normal limits.</t>
+  </si>
+  <si>
+    <t>Regular meals and light exercise contribute positively to overall health. | Temperature and blood pressure readings are consistent throughout the week.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet rich in fruits and vegetables. | Stay hydrated and limit caffeine intake. | Include regular physical activity, such as daily walks.</t>
+  </si>
+  <si>
+    <t>Continue to monitor vital signs regularly. | Follow-up on any recurrence of withdrawal symptoms.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment in one month. | Consider daily journaling of symptoms and mood.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:01:52.063Z</t>
+  </si>
+  <si>
+    <t>John Doe has recently recovered from Alcohol Withdrawal. His vital signs are stable with normal ranges observed over the past week. No critical health alerts are present.</t>
+  </si>
+  <si>
+    <t>LOW: Mild sweating and confusion recorded; continue monitoring symptoms.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable (systolic 119-123, diastolic 79-81) | Heart Rate: Consistent (68-73 bpm) | SpO2: Good (97-99%) | Body Temperature: Normal (98.4-98.6°F) | Blood Sugar: Slight fluctuation (95-105 mg/dL)</t>
+  </si>
+  <si>
+    <t>Regular breakfast intake noted, contributing to stable energy levels. | Incorporation of light exercises like morning walks seems to improve overall well-being. | Variability in lunch and dinner times may influence post-meal blood sugar levels.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet focusing on whole foods to support recovery. | Stay hydrated and manage stress through relaxation techniques. | Continue daily walks to promote cardiovascular health.</t>
+  </si>
+  <si>
+    <t>Patient is recovering well post-treatment for Alcohol Withdrawal. | Continued monitoring of vitals and symptoms recommended. | Encourage participation in regular follow-up appointments.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with the healthcare provider. | Monitor any resurgence of symptoms like confusion or excessive sweating. | Engage in regular activity and maintain healthy nutrition.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:10:07.807Z</t>
+  </si>
+  <si>
+    <t>John Doe is a 36-year-old male who has successfully overcome Alcohol Withdrawal and currently shows stable vital signs.</t>
+  </si>
+  <si>
+    <t>LOW: Mild confusion and sweating have been recorded but are decreasing over time.</t>
+  </si>
+  <si>
+    <t>Blood pressure remains stable with readings around 120/80 mmHg. | Heart rate is consistent, averaging around 70 bpm. | SpO2 levels are healthy at approximately 98%. | Body temperature is normal, fluctuating slightly around 98.4°F to 98.6°F. | Blood sugar levels are within a reasonable range, peaking at 105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular meals are observed, primarily consisting of breakfast, lunch, and dinner. | Morning walks and light exercise contribute positively to overall health.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet with fruits and vegetables. | Stay hydrated and continue daily physical activity to improve wellness. | Monitor stress levels and practice relaxation techniques.</t>
+  </si>
+  <si>
+    <t>Continued monitoring of mental and physical health is recommended post-recovery. | Focus on developing a consistent routine to ensure ongoing well-being.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with the healthcare provider in one month. | Consider joining a support group for ongoing recovery support.</t>
   </si>
 </sst>
 </file>
@@ -1761,7 +1833,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -4501,6 +4573,174 @@
         <v>457</v>
       </c>
     </row>
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>458</v>
+      </c>
+      <c r="B55" t="s">
+        <v>19</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55">
+        <v>36</v>
+      </c>
+      <c r="E55" t="s">
+        <v>356</v>
+      </c>
+      <c r="F55" t="s">
+        <v>357</v>
+      </c>
+      <c r="G55" t="s">
+        <v>459</v>
+      </c>
+      <c r="H55" t="s">
+        <v>460</v>
+      </c>
+      <c r="I55" t="s">
+        <v>461</v>
+      </c>
+      <c r="J55" t="s">
+        <v>462</v>
+      </c>
+      <c r="K55" t="s">
+        <v>463</v>
+      </c>
+      <c r="L55" t="s">
+        <v>464</v>
+      </c>
+      <c r="M55" t="s">
+        <v>465</v>
+      </c>
+      <c r="N55">
+        <v>2538</v>
+      </c>
+      <c r="O55">
+        <v>268</v>
+      </c>
+      <c r="P55">
+        <v>2806</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>34</v>
+      </c>
+      <c r="R55" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>466</v>
+      </c>
+      <c r="B56" t="s">
+        <v>19</v>
+      </c>
+      <c r="C56" t="s">
+        <v>20</v>
+      </c>
+      <c r="D56">
+        <v>36</v>
+      </c>
+      <c r="E56" t="s">
+        <v>356</v>
+      </c>
+      <c r="F56" t="s">
+        <v>357</v>
+      </c>
+      <c r="G56" t="s">
+        <v>467</v>
+      </c>
+      <c r="H56" t="s">
+        <v>468</v>
+      </c>
+      <c r="I56" t="s">
+        <v>469</v>
+      </c>
+      <c r="J56" t="s">
+        <v>470</v>
+      </c>
+      <c r="K56" t="s">
+        <v>471</v>
+      </c>
+      <c r="L56" t="s">
+        <v>472</v>
+      </c>
+      <c r="M56" t="s">
+        <v>473</v>
+      </c>
+      <c r="N56">
+        <v>2538</v>
+      </c>
+      <c r="O56">
+        <v>353</v>
+      </c>
+      <c r="P56">
+        <v>2891</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>34</v>
+      </c>
+      <c r="R56" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>474</v>
+      </c>
+      <c r="B57" t="s">
+        <v>19</v>
+      </c>
+      <c r="C57" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57">
+        <v>36</v>
+      </c>
+      <c r="E57" t="s">
+        <v>356</v>
+      </c>
+      <c r="F57" t="s">
+        <v>357</v>
+      </c>
+      <c r="G57" t="s">
+        <v>475</v>
+      </c>
+      <c r="H57" t="s">
+        <v>476</v>
+      </c>
+      <c r="I57" t="s">
+        <v>477</v>
+      </c>
+      <c r="J57" t="s">
+        <v>478</v>
+      </c>
+      <c r="K57" t="s">
+        <v>479</v>
+      </c>
+      <c r="L57" t="s">
+        <v>480</v>
+      </c>
+      <c r="M57" t="s">
+        <v>481</v>
+      </c>
+      <c r="N57">
+        <v>2538</v>
+      </c>
+      <c r="O57">
+        <v>318</v>
+      </c>
+      <c r="P57">
+        <v>2856</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>34</v>
+      </c>
+      <c r="R57" t="s">
+        <v>457</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update health records and output.json with refined summaries and alerts for better patient monitoring. Adjusted PDF report formatting for improved readability and spacing. Enhanced vital signs and daily patterns descriptions to reflect ongoing recovery challenges.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="482">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="490">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1457,6 +1457,30 @@
   </si>
   <si>
     <t>Schedule a follow-up appointment with the healthcare provider in one month. | Consider joining a support group for ongoing recovery support.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:19:50.486Z</t>
+  </si>
+  <si>
+    <t>John Doe is recovering from Alcohol Withdrawal. His vital signs show stable readings, but symptoms like confusion and sweating still occasionally occur.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Confusion and sweating levels indicate ongoing recovery challenges. Monitor these symptoms closely.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: stable between 119-123/79-81 mmHg. | Heart Rate: averages 70 bpm with minor fluctuations. | SpO2: consistent at 97-99%. | Body Temperature: remains within normal range (98.4-98.6°F). | Blood Sugar: fluctuates slightly between 95-105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular breakfast and afternoon meals contribute to stable blood sugar levels. | Morning walks and light exercise have a positive effect on heart rate. | Increased levels of sweating correlate with higher severity of confusion symptoms.</t>
+  </si>
+  <si>
+    <t>Maintain a consistent meal schedule to help regulate blood sugar levels. | Incorporate more light exercises to boost overall wellness. | Stay hydrated to manage sweating and support recovery.</t>
+  </si>
+  <si>
+    <t>Continue monitoring symptoms of confusion and sweating. | Encourage John to maintain a consistent routine for meals and activities.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with the healthcare provider. | Consider a consultation with a nutritionist to fine-tune dietary habits. | Monitor vital signs at home and report any significant changes.</t>
   </si>
 </sst>
 </file>
@@ -1833,7 +1857,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R58"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -4741,6 +4765,62 @@
         <v>457</v>
       </c>
     </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>482</v>
+      </c>
+      <c r="B58" t="s">
+        <v>19</v>
+      </c>
+      <c r="C58" t="s">
+        <v>20</v>
+      </c>
+      <c r="D58">
+        <v>36</v>
+      </c>
+      <c r="E58" t="s">
+        <v>356</v>
+      </c>
+      <c r="F58" t="s">
+        <v>357</v>
+      </c>
+      <c r="G58" t="s">
+        <v>483</v>
+      </c>
+      <c r="H58" t="s">
+        <v>484</v>
+      </c>
+      <c r="I58" t="s">
+        <v>485</v>
+      </c>
+      <c r="J58" t="s">
+        <v>486</v>
+      </c>
+      <c r="K58" t="s">
+        <v>487</v>
+      </c>
+      <c r="L58" t="s">
+        <v>488</v>
+      </c>
+      <c r="M58" t="s">
+        <v>489</v>
+      </c>
+      <c r="N58">
+        <v>2538</v>
+      </c>
+      <c r="O58">
+        <v>346</v>
+      </c>
+      <c r="P58">
+        <v>2884</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>34</v>
+      </c>
+      <c r="R58" t="s">
+        <v>457</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update index.html for improved styling and layout consistency, including adjustments to font sizes, margins, and colors. Revise output.json to reflect updated patient health summaries and remove unnecessary health alerts. Replace PDF generation logic in pdfReport.js with Puppeteer for enhanced report rendering. Update package.json and package-lock.json to include Puppeteer as a dependency.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="529">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1481,6 +1481,123 @@
   </si>
   <si>
     <t>Schedule a follow-up appointment with the healthcare provider. | Consider a consultation with a nutritionist to fine-tune dietary habits. | Monitor vital signs at home and report any significant changes.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:45:34.331Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has successfully recovered from Alcohol Withdrawal. His vital signs indicate stable health with consistent readings.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Blood Pressure readings are stable, ranging from 119/79 to 123/81. | Heart Rate is consistent, varying between 68 to 73 bpm. | SpO2 levels are within normal range, between 97% to 99%. | Body Temperature is stable, hovering around 98.4°F to 98.6°F. | Blood Sugar levels fluctuate slightly, with readings from 95 to 105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular meals and daily physical activities such as morning walks are positively influencing vital signs. | Stress levels indicated by confusion and sweating were higher in the initial days of withdrawal but have shown improvement with routine.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet with consistent meal times to help stabilize blood sugar levels. | Engage in regular light exercise to promote cardiovascular health. | Consider mindfulness or relaxation techniques to manage stress.</t>
+  </si>
+  <si>
+    <t>Monitor any resurgence of withdrawal symptoms; continue encouraging daily routine. | Reassess vital signs weekly to ensure ongoing stability after recovery.</t>
+  </si>
+  <si>
+    <t>Continue current lifestyle and monitor symptoms daily. | Schedule a follow-up consultation in two weeks to review health progress.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:50:57.525Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has successfully cured his Alcohol Withdrawal condition. Alertness and physical symptoms have improved over time. Vitals are generally stable.</t>
+  </si>
+  <si>
+    <t>LOW: Continue to monitor mild confusion and sweating symptoms. If they worsen, consult a healthcare provider.</t>
+  </si>
+  <si>
+    <t>Blood Pressure is within normal ranges with slight variations. | Heart Rate fluctuates but remains at healthy levels. | Oxygen Saturation (SpO2) is stable at 97%-99%. | Body Temperature remains steady at approximately 98.5°F. | Blood Sugar readings show slight increases but are within acceptable limits.</t>
+  </si>
+  <si>
+    <t>Regular breakfast habits with light exercise and morning walks correlate with lower symptom severity. | Daily fluctuations in heart rate and blood pressure are minimally impacted by activity levels.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet, focusing on whole grains and lean proteins. | Stay hydrated and avoid excessive caffeine intake. | Incorporate mindfulness or relaxation techniques to manage stress.</t>
+  </si>
+  <si>
+    <t>John has shown good recovery from Alcohol Withdrawal. Ongoing support and monitoring are recommended.</t>
+  </si>
+  <si>
+    <t>Continue regular follow-up appointments with the care team. | Monitor symptoms closely and report any sudden changes. | Consider scheduling a consultation if confusion or sweating intensifies.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:51:31.622Z</t>
+  </si>
+  <si>
+    <t>John Doe has successfully recovered from Alcohol Withdrawal and is experiencing decreased symptoms. His vital signs are stable with no urgent concerns.</t>
+  </si>
+  <si>
+    <t>LOW: Mild confusion was noted on some days but is improving.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Consistently within normal range, averaging 120/80 mmHg. | Heart Rate: Maintained between 68-73 bpm. | SpO2: Steady at 97-99%. | Body Temperature: Stable around 98.5°F. | Blood Sugar: Minor variations observed, with levels ranging from 95 to 105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular meal times appear to correlate with stable blood sugar levels. | Consistent morning walks and exercises are linked to improved heart rate and blood pressure.</t>
+  </si>
+  <si>
+    <t>Continue with regular meal times to further stabilize blood sugar. | Incorporate more light exercises into daily routine for cardiovascular benefits. | Maintain hydration throughout the day.</t>
+  </si>
+  <si>
+    <t>Monitor any returning symptoms of confusion and make adjustments as needed. | Encourage continued engagement in physical activity to support recovery.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with your healthcare provider in two weeks. | Keep a daily log of symptoms and activities to share during your next visit.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:53:01.550Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, is recovering from Alcohol Withdrawal. Most symptoms have improved, but some instances of confusion and sweating were noted.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Monitor any recurring symptoms of confusion and sweating</t>
+  </si>
+  <si>
+    <t>Blood Pressure remains stable with values mostly around 120/80. | Heart Rate is consistent, averaging around 70 beats per minute. | SpO2 levels are healthy, staying between 97% to 99%. | Body Temperature is normal, consistently around 98.4°F to 98.6°F. | Blood Sugar levels range from 95 to 105 mg/dL, which is acceptable.</t>
+  </si>
+  <si>
+    <t>Regular meal timings and light exercises, like morning walks, contribute to stable vital signs. | The inclusion of breakfast appears to align with more consistent energy levels.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet rich in fruits and vegetables for better recovery. | Incorporate regular light exercise, such as walks, to enhance overall well-being.</t>
+  </si>
+  <si>
+    <t>Continue monitoring symptoms, especially any re-emergence of confusion or severe sweating. | Keep an eye on blood sugar levels and maintain hydration.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment to assess ongoing symptoms and recovery. | Consider a consult with a nutritionist for tailored dietary advice.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:53:32.364Z</t>
+  </si>
+  <si>
+    <t>John Doe has shown improvement after recovering from Alcohol Withdrawal. Most vital signs are within normal ranges, indicating stable health.</t>
+  </si>
+  <si>
+    <t>Blood Pressure is stable, average reading of 120/80. | Heart Rate remains steady, averaging around 70 beats per minute. | SpO2 is consistently above 97%, indicating good oxygen levels. | Body Temperature is normal, averaging around 98.5°F. | Blood Sugar levels are mostly within normal limits but show slight variations.</t>
+  </si>
+  <si>
+    <t>Regular meals and morning walks support overall health. | Increased sweating and confusion were noted during Alcohol Withdrawal recovery days. | Stable vital signs indicate a positive response to daily routines.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet with regular meals to keep blood sugar levels stable. | Stay physically active with regular walks or light exercises. | Ensure consistent hydration, especially during physical activities.</t>
+  </si>
+  <si>
+    <t>Continued monitoring of mental health is essential after Alcohol Withdrawal. | Maintain follow-up visits to monitor essential vitals specifically during recovery.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with the healthcare provider. | Continue to track daily activities and symptoms for any changes. | Explore support groups for long-term recovery from Alcohol dependency.</t>
   </si>
 </sst>
 </file>
@@ -1857,7 +1974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R58"/>
+  <dimension ref="A1:R63"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -4821,6 +4938,286 @@
         <v>457</v>
       </c>
     </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>490</v>
+      </c>
+      <c r="B59" t="s">
+        <v>19</v>
+      </c>
+      <c r="C59" t="s">
+        <v>20</v>
+      </c>
+      <c r="D59">
+        <v>36</v>
+      </c>
+      <c r="E59" t="s">
+        <v>356</v>
+      </c>
+      <c r="F59" t="s">
+        <v>357</v>
+      </c>
+      <c r="G59" t="s">
+        <v>491</v>
+      </c>
+      <c r="H59" t="s">
+        <v>492</v>
+      </c>
+      <c r="I59" t="s">
+        <v>493</v>
+      </c>
+      <c r="J59" t="s">
+        <v>494</v>
+      </c>
+      <c r="K59" t="s">
+        <v>495</v>
+      </c>
+      <c r="L59" t="s">
+        <v>496</v>
+      </c>
+      <c r="M59" t="s">
+        <v>497</v>
+      </c>
+      <c r="N59">
+        <v>2538</v>
+      </c>
+      <c r="O59">
+        <v>318</v>
+      </c>
+      <c r="P59">
+        <v>2856</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>34</v>
+      </c>
+      <c r="R59" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>498</v>
+      </c>
+      <c r="B60" t="s">
+        <v>19</v>
+      </c>
+      <c r="C60" t="s">
+        <v>20</v>
+      </c>
+      <c r="D60">
+        <v>36</v>
+      </c>
+      <c r="E60" t="s">
+        <v>356</v>
+      </c>
+      <c r="F60" t="s">
+        <v>357</v>
+      </c>
+      <c r="G60" t="s">
+        <v>499</v>
+      </c>
+      <c r="H60" t="s">
+        <v>500</v>
+      </c>
+      <c r="I60" t="s">
+        <v>501</v>
+      </c>
+      <c r="J60" t="s">
+        <v>502</v>
+      </c>
+      <c r="K60" t="s">
+        <v>503</v>
+      </c>
+      <c r="L60" t="s">
+        <v>504</v>
+      </c>
+      <c r="M60" t="s">
+        <v>505</v>
+      </c>
+      <c r="N60">
+        <v>2538</v>
+      </c>
+      <c r="O60">
+        <v>326</v>
+      </c>
+      <c r="P60">
+        <v>2864</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>34</v>
+      </c>
+      <c r="R60" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>506</v>
+      </c>
+      <c r="B61" t="s">
+        <v>19</v>
+      </c>
+      <c r="C61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D61">
+        <v>36</v>
+      </c>
+      <c r="E61" t="s">
+        <v>356</v>
+      </c>
+      <c r="F61" t="s">
+        <v>357</v>
+      </c>
+      <c r="G61" t="s">
+        <v>507</v>
+      </c>
+      <c r="H61" t="s">
+        <v>508</v>
+      </c>
+      <c r="I61" t="s">
+        <v>509</v>
+      </c>
+      <c r="J61" t="s">
+        <v>510</v>
+      </c>
+      <c r="K61" t="s">
+        <v>511</v>
+      </c>
+      <c r="L61" t="s">
+        <v>512</v>
+      </c>
+      <c r="M61" t="s">
+        <v>513</v>
+      </c>
+      <c r="N61">
+        <v>2538</v>
+      </c>
+      <c r="O61">
+        <v>322</v>
+      </c>
+      <c r="P61">
+        <v>2860</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>34</v>
+      </c>
+      <c r="R61" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>514</v>
+      </c>
+      <c r="B62" t="s">
+        <v>19</v>
+      </c>
+      <c r="C62" t="s">
+        <v>20</v>
+      </c>
+      <c r="D62">
+        <v>36</v>
+      </c>
+      <c r="E62" t="s">
+        <v>356</v>
+      </c>
+      <c r="F62" t="s">
+        <v>357</v>
+      </c>
+      <c r="G62" t="s">
+        <v>515</v>
+      </c>
+      <c r="H62" t="s">
+        <v>516</v>
+      </c>
+      <c r="I62" t="s">
+        <v>517</v>
+      </c>
+      <c r="J62" t="s">
+        <v>518</v>
+      </c>
+      <c r="K62" t="s">
+        <v>519</v>
+      </c>
+      <c r="L62" t="s">
+        <v>520</v>
+      </c>
+      <c r="M62" t="s">
+        <v>521</v>
+      </c>
+      <c r="N62">
+        <v>2538</v>
+      </c>
+      <c r="O62">
+        <v>333</v>
+      </c>
+      <c r="P62">
+        <v>2871</v>
+      </c>
+      <c r="Q62" t="s">
+        <v>34</v>
+      </c>
+      <c r="R62" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>522</v>
+      </c>
+      <c r="B63" t="s">
+        <v>19</v>
+      </c>
+      <c r="C63" t="s">
+        <v>20</v>
+      </c>
+      <c r="D63">
+        <v>36</v>
+      </c>
+      <c r="E63" t="s">
+        <v>356</v>
+      </c>
+      <c r="F63" t="s">
+        <v>357</v>
+      </c>
+      <c r="G63" t="s">
+        <v>523</v>
+      </c>
+      <c r="H63" t="s">
+        <v>492</v>
+      </c>
+      <c r="I63" t="s">
+        <v>524</v>
+      </c>
+      <c r="J63" t="s">
+        <v>525</v>
+      </c>
+      <c r="K63" t="s">
+        <v>526</v>
+      </c>
+      <c r="L63" t="s">
+        <v>527</v>
+      </c>
+      <c r="M63" t="s">
+        <v>528</v>
+      </c>
+      <c r="N63">
+        <v>2538</v>
+      </c>
+      <c r="O63">
+        <v>301</v>
+      </c>
+      <c r="P63">
+        <v>2839</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>34</v>
+      </c>
+      <c r="R63" t="s">
+        <v>457</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update index.html for enhanced styling and layout, including adjustments to section titles and content presentation. Revise output.json to reflect updated patient health summaries and alerts, ensuring clarity in monitoring. Minor adjustments made to pdfReport.js for consistent styling in report generation.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="529">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="560">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1598,6 +1598,99 @@
   </si>
   <si>
     <t>Schedule a follow-up appointment with the healthcare provider. | Continue to track daily activities and symptoms for any changes. | Explore support groups for long-term recovery from Alcohol dependency.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:57:03.439Z</t>
+  </si>
+  <si>
+    <t>John Doe is showing a stable health status after recovering from Alcohol Withdrawal. Vitals are consistently within normal ranges, but monitoring is advised due to past symptoms.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable at around 120/80 mmHg. | Heart Rate: Consistent average around 70 bpm. | SpO2: Remains healthy at approximately 98%. | Body Temperature: Normal range between 98.4°F and 98.6°F. | Blood Sugar: Values are fluctuating but generally within normal limits.</t>
+  </si>
+  <si>
+    <t>Regular meals and light exercise contribute to stable vital signs. | Incorporating morning walks has shown positive effects on mood and overall health.</t>
+  </si>
+  <si>
+    <t>Maintain hydration by drinking plenty of water throughout the day. | Incorporate more fruits and vegetables into your meals for added nutrients. | Continue regular light exercise for cardiovascular health.</t>
+  </si>
+  <si>
+    <t>Patient is encouraged to keep monitoring symptoms and vitals regularly. | Continue with regular follow-ups to ensure recovery is maintained.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with your healthcare provider. | Monitor daily activities and symptoms closely. | Consider keeping a food and activity diary to share with the care team.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:58:26.235Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has shown improvements from his previously cured condition of Alcohol Withdrawal. His vital signs are mostly stable, but some symptoms related to the condition were recorded.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Mild symptoms of sweating and confusion were reported, indicating potential ongoing issues.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable, averaging around 120/80. | Heart Rate: Consistently between 68 and 73 bpm. | SpO2 Level: Remained above 97%, indicating good oxygen saturation. | Body Temperature: Stable around 98.5°F. | Blood Sugar: A few slight variations, with average levels around 100 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular meals and light exercises seem to correlate with better vitals. | Mild fluctuations in blood sugar related to dietary intake.</t>
+  </si>
+  <si>
+    <t>Maintain consistent meal times to help stabilize blood sugar levels. | Incorporate more light exercises during the day to aid overall health.</t>
+  </si>
+  <si>
+    <t>Continue monitoring symptoms and maintain a healthy routine. Recommend regular follow-ups for ongoing support.</t>
+  </si>
+  <si>
+    <t>Schedule an appointment with a healthcare provider for routine check-ups. | Monitor symptoms closely and report if they worsen.</t>
+  </si>
+  <si>
+    <t>2026-02-13T10:59:21.621Z</t>
+  </si>
+  <si>
+    <t>John Doe has successfully recovered from Alcohol Withdrawal. His vital signs are stable with some fluctuations noted in blood sugar levels. Continued monitoring and healthy habits are essential.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Blood sugar levels have shown some fluctuations, reaching a high of 105 mg/dL. Regular monitoring is recommended.</t>
+  </si>
+  <si>
+    <t>Blood Pressure is stable averaging around 120/80 mmHg. | Heart Rate is consistent with an average around 70 beats per minute. | SpO2 levels are healthy, consistently around 97-99%. | Body Temperature remains within normal limits, averaging approximately 98.5°F.</t>
+  </si>
+  <si>
+    <t>A regular breakfast routine appears to help stabilize blood sugar levels. | Morning walks contribute positively to overall well-being and heart rate stability.</t>
+  </si>
+  <si>
+    <t>Maintain a consistent meal schedule to support stable blood sugar levels. | Incorporate more fruits and vegetables into your diet for better nutrient balance. | Consider light exercises in the evening to promote relaxation and overall health.</t>
+  </si>
+  <si>
+    <t>Patient shows good recovery progress. Continuous lifestyle management is crucial to prevent relapse. | Monitor blood sugar levels and recommend follow-up consultation if fluctuations continue.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment to review blood sugar levels. | Continue daily monitoring of vitals and symptoms. | Adhere to lifestyle changes suggested for better health management.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:00:24.616Z</t>
+  </si>
+  <si>
+    <t>John Doe has shown recovery from Alcohol Withdrawal, with notable fluctuations in symptoms like confusion and sweating. Vitals remain stable with normal blood pressure and heart rate.</t>
+  </si>
+  <si>
+    <t>LOW: Monitor for any returning symptoms of confusion or sweating.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable around 120/80 mmHg | Heart Rate: Average around 70 bpm | SpO2: Maintained at 97-99% | Body Temperature: Consistently around 98.4°F-98.6°F | Blood Sugar: Varies from 95-105 mg/dL, requiring monitoring.</t>
+  </si>
+  <si>
+    <t>Routine meals and regular light exercise positively impacted heart rate and overall well-being. | Engaging in morning walks contributed to improved mental clarity.</t>
+  </si>
+  <si>
+    <t>Maintain a consistent meal schedule to stabilize blood sugar levels. | Incorporate daily walks for enhanced physical and mental health. | Stay hydrated and consider mindfulness practices to manage stress.</t>
+  </si>
+  <si>
+    <t>Continue observing symptoms closely and encourage patient engagement in physical activities. | Consider regular follow-ups to monitor recovery progress.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up consultation to discuss any recurring symptoms. | Continue tracking vital signs daily.</t>
   </si>
 </sst>
 </file>
@@ -1974,7 +2067,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R63"/>
+  <dimension ref="A1:R67"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -5218,6 +5311,230 @@
         <v>457</v>
       </c>
     </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>529</v>
+      </c>
+      <c r="B64" t="s">
+        <v>19</v>
+      </c>
+      <c r="C64" t="s">
+        <v>20</v>
+      </c>
+      <c r="D64">
+        <v>36</v>
+      </c>
+      <c r="E64" t="s">
+        <v>356</v>
+      </c>
+      <c r="F64" t="s">
+        <v>357</v>
+      </c>
+      <c r="G64" t="s">
+        <v>530</v>
+      </c>
+      <c r="H64" t="s">
+        <v>492</v>
+      </c>
+      <c r="I64" t="s">
+        <v>531</v>
+      </c>
+      <c r="J64" t="s">
+        <v>532</v>
+      </c>
+      <c r="K64" t="s">
+        <v>533</v>
+      </c>
+      <c r="L64" t="s">
+        <v>534</v>
+      </c>
+      <c r="M64" t="s">
+        <v>535</v>
+      </c>
+      <c r="N64">
+        <v>2538</v>
+      </c>
+      <c r="O64">
+        <v>299</v>
+      </c>
+      <c r="P64">
+        <v>2837</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>34</v>
+      </c>
+      <c r="R64" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="65" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>536</v>
+      </c>
+      <c r="B65" t="s">
+        <v>19</v>
+      </c>
+      <c r="C65" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65">
+        <v>36</v>
+      </c>
+      <c r="E65" t="s">
+        <v>356</v>
+      </c>
+      <c r="F65" t="s">
+        <v>357</v>
+      </c>
+      <c r="G65" t="s">
+        <v>537</v>
+      </c>
+      <c r="H65" t="s">
+        <v>538</v>
+      </c>
+      <c r="I65" t="s">
+        <v>539</v>
+      </c>
+      <c r="J65" t="s">
+        <v>540</v>
+      </c>
+      <c r="K65" t="s">
+        <v>541</v>
+      </c>
+      <c r="L65" t="s">
+        <v>542</v>
+      </c>
+      <c r="M65" t="s">
+        <v>543</v>
+      </c>
+      <c r="N65">
+        <v>2538</v>
+      </c>
+      <c r="O65">
+        <v>312</v>
+      </c>
+      <c r="P65">
+        <v>2850</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>34</v>
+      </c>
+      <c r="R65" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="66" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>544</v>
+      </c>
+      <c r="B66" t="s">
+        <v>19</v>
+      </c>
+      <c r="C66" t="s">
+        <v>20</v>
+      </c>
+      <c r="D66">
+        <v>36</v>
+      </c>
+      <c r="E66" t="s">
+        <v>356</v>
+      </c>
+      <c r="F66" t="s">
+        <v>357</v>
+      </c>
+      <c r="G66" t="s">
+        <v>545</v>
+      </c>
+      <c r="H66" t="s">
+        <v>546</v>
+      </c>
+      <c r="I66" t="s">
+        <v>547</v>
+      </c>
+      <c r="J66" t="s">
+        <v>548</v>
+      </c>
+      <c r="K66" t="s">
+        <v>549</v>
+      </c>
+      <c r="L66" t="s">
+        <v>550</v>
+      </c>
+      <c r="M66" t="s">
+        <v>551</v>
+      </c>
+      <c r="N66">
+        <v>2538</v>
+      </c>
+      <c r="O66">
+        <v>339</v>
+      </c>
+      <c r="P66">
+        <v>2877</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>34</v>
+      </c>
+      <c r="R66" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="67" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>552</v>
+      </c>
+      <c r="B67" t="s">
+        <v>19</v>
+      </c>
+      <c r="C67" t="s">
+        <v>20</v>
+      </c>
+      <c r="D67">
+        <v>36</v>
+      </c>
+      <c r="E67" t="s">
+        <v>356</v>
+      </c>
+      <c r="F67" t="s">
+        <v>357</v>
+      </c>
+      <c r="G67" t="s">
+        <v>553</v>
+      </c>
+      <c r="H67" t="s">
+        <v>554</v>
+      </c>
+      <c r="I67" t="s">
+        <v>555</v>
+      </c>
+      <c r="J67" t="s">
+        <v>556</v>
+      </c>
+      <c r="K67" t="s">
+        <v>557</v>
+      </c>
+      <c r="L67" t="s">
+        <v>558</v>
+      </c>
+      <c r="M67" t="s">
+        <v>559</v>
+      </c>
+      <c r="N67">
+        <v>2538</v>
+      </c>
+      <c r="O67">
+        <v>309</v>
+      </c>
+      <c r="P67">
+        <v>2847</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>34</v>
+      </c>
+      <c r="R67" t="s">
+        <v>457</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Revise output.json to provide a more detailed patient health summary, including updated vital signs, health alerts, and care recommendations. Update health_records.xlsx to reflect recent changes in health data management.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1042" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="639">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1691,6 +1691,243 @@
   </si>
   <si>
     <t>Schedule a follow-up consultation to discuss any recurring symptoms. | Continue tracking vital signs daily.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:05:44.550Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has successfully overcome Alcohol Withdrawal. While he is currently stable, monitoring of his health conditions and lifestyle is recommended.</t>
+  </si>
+  <si>
+    <t>LOW: Mild confusion and sweating were recorded, generally improving over the observation period.</t>
+  </si>
+  <si>
+    <t>Blood pressure readings are within normal limits, consistently around 120/80. | Heart rate is stable, ranging from 68 to 73 bpm. | SpO2 levels are normal, consistently above 97%. | Body temperature is within a healthy range, averaging around 98.5°F. | Blood sugar levels fluctuate but remain mostly within a normal range.</t>
+  </si>
+  <si>
+    <t>Breakfast is regularly consumed, usually in the morning. | Engaging in physical activities such as morning walks and light exercise positively impacts overall well-being.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet with regular meals to stabilize blood sugar levels. | Incorporate daily physical activities to enhance mood and physical health. | Stay hydrated and manage stress through mindfulness practices.</t>
+  </si>
+  <si>
+    <t>Continued support and monitoring are needed post-recovery to reinforce healthy habits. | Encourage regular follow-ups to track any re-emergence of symptoms.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with a healthcare provider. | Continue to log daily activities and health symptoms. | Consider joining a support group for ongoing motivation and assistance.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:11:48.619Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has successfully recovered from Alcohol Withdrawal. His vital signs are stable, and there are some noted fluctuations in his symptoms which require monitoring.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Confusion levels have varied in severity. Monitor mental clarity and report any significant changes. | LOW: Sweating episodes were frequent but are decreasing. Continue to stay hydrated.</t>
+  </si>
+  <si>
+    <t>Blood pressure remains within normal ranges with slight increases noted on some days. | Heart rate is stable, averaging around 70 beats per minute. | SpO2 levels are consistently good, averaging around 98%. | Body temperature is stable, averaging about 98.5°F. | Blood sugar levels are slightly fluctuating but remain generally acceptable.</t>
+  </si>
+  <si>
+    <t>Regular meals and light exercise seem to positively correlate with stable vital signs. | Days with both breakfast and light exercise have lower heart rates.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet to support stability in blood sugar levels. | Incorporate more regular physical activities to improve overall health. | Stay hydrated, especially during hot weather or after exercise.</t>
+  </si>
+  <si>
+    <t>Continue monitoring confusion and sweating patterns closely. | Patient shows signs of improved health after previous condition.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment in two weeks to reassess the situation. | Consider consulting a specialist if symptoms of confusion persist.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:37:09.732Z</t>
+  </si>
+  <si>
+    <t>John Doe's health shows stable vital signs following recovery from Alcohol Withdrawal. While no critical alerts are indicated, mild symptoms were recorded during the recovery phase.</t>
+  </si>
+  <si>
+    <t>LOW: Mild confusion and sweating were reported; symptoms are decreasing over time.</t>
+  </si>
+  <si>
+    <t>Blood Pressure is stable around 120/80 mmHg. | Heart Rate is normal, averaging between 68-73 bpm. | SpO2 levels are healthy at 97-99%. | Body Temperature remains within normal limits, around 98.4-98.6°F. | Blood Sugar is fluctuating slightly but stays within acceptable ranges.</t>
+  </si>
+  <si>
+    <t>Regular meal timings observed with consistent breakfast intake. | Physical activity is maintained with daily walks and light exercises.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet with regular meal times. | Incorporate more physical activity throughout the day.</t>
+  </si>
+  <si>
+    <t>Continue monitoring symptoms related to past Alcohol Withdrawal. Advise follow-up if symptoms persist.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up consultation in one month. | Monitor daily activities and symptoms.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:37:57.755Z</t>
+  </si>
+  <si>
+    <t>John Doe has shown improvement in symptoms related to Alcohol Withdrawal and is now cured. Vital signs indicate stable health with no immediate concerns.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable at around 120/80 mmHg. | Heart Rate: Average around 70 bpm. | SpO2: Consistently above 97%. | Body Temperature: Normal range around 98.5°F. | Blood Sugar: Slightly elevated but within manageable limits.</t>
+  </si>
+  <si>
+    <t>Regular meals and moderate exercise appear to contribute to stable vitals. | Improvement in symptoms correlates with adherence to a structured routine.</t>
+  </si>
+  <si>
+    <t>Continue regular healthy meals, including fruits and vegetables. | Stay hydrated and limit consumption of alcohol and sugary drinks. | Incorporate daily light exercise to maintain cardiovascular health.</t>
+  </si>
+  <si>
+    <t>Patient has shown significant improvement and is advised to maintain current lifestyle. | Continued monitoring of blood sugar levels is recommended.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment in one month to review ongoing health. | Monitor symptoms closely and seek assistance if any concerns arise.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:40:00.211Z</t>
+  </si>
+  <si>
+    <t>John Doe has successfully recovered from alcohol withdrawal. His vital signs are stable, showing no critical issues requiring urgent attention.</t>
+  </si>
+  <si>
+    <t>LOW: Mild fluctuations in heart rate and blood sugar levels have been observed.</t>
+  </si>
+  <si>
+    <t>Blood pressure remains stable in the normal range with a systolic average of 120 mmHg and a diastolic average of 80 mmHg. | Heart rate is within the normal range, averaging around 70 beats per minute. | SpO2 levels are consistently above 97%, indicating good oxygen saturation. | Body temperature remains stable, ranging from 98.4°F to 98.6°F. | Blood sugar levels fluctuate mildly but remain within acceptable limits.</t>
+  </si>
+  <si>
+    <t>Consistent breakfast timing contributes to stable blood sugar levels throughout the day. | Engaging in morning walks appears to positively impact heart rate and overall mood.</t>
+  </si>
+  <si>
+    <t>Consider continuing regular morning walks to maintain cardiovascular health. | Stay hydrated and include a balanced diet to help stabilize blood sugar levels.</t>
+  </si>
+  <si>
+    <t>John is on the right track with his recovery. Continue to monitor vitals closely.</t>
+  </si>
+  <si>
+    <t>Schedule regular check-ins with the healthcare team to monitor recovery progress. | Maintain daily activity logs to help identify patterns in health and wellness.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:40:37.129Z</t>
+  </si>
+  <si>
+    <t>John Doe is 36 years old and has recently recovered from Alcohol Withdrawal. His vital signs are stable, but there is a history of symptoms like confusion and sweating that were recently recorded.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Monitor for any recurring symptoms related to Alcohol Withdrawal.</t>
+  </si>
+  <si>
+    <t>Blood Pressure is within normal range, averaging around 120/80 mmHg. | Heart Rate is consistent at around 70 beats per minute. | SpO2 levels are stable, averaging 98%. | Body Temperature is normal, averaging approximately 98.5°F. | Blood Sugar levels are slightly variable, ranging from 95 to 105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular meal times, with consistent breakfast and lunch routines. | Incorporation of light exercise and morning walks on some days. | Slight increases in blood sugar observed after meals.</t>
+  </si>
+  <si>
+    <t>Consider reducing sugar intake to stabilize blood sugar levels. | Maintain hydration throughout the day. | Continue engaging in daily physical activity to support heart health.</t>
+  </si>
+  <si>
+    <t>Monitor the patient for signs of withdrawal symptoms. | Ensure regular follow-ups to assess mental health.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment in one month. | Consider discussing any recurring symptoms with the healthcare provider.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:41:49.825Z</t>
+  </si>
+  <si>
+    <t>Patient John Doe has recently completed treatment for Alcohol Withdrawal and is currently stable with normal vital signs.</t>
+  </si>
+  <si>
+    <t>LOW: No critical health alerts detected. Continue monitoring.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable and within normal range. | Heart Rate: Consistently normal. | SpO2: Levels are satisfactory. | Body Temperature: Normal range maintained. | Blood Sugar: Fluctuations within acceptable limits.</t>
+  </si>
+  <si>
+    <t>Regular meal times observed with healthy choices. | Engaged in physical activities like morning walks and light exercises. | Consistently maintained hydration levels.</t>
+  </si>
+  <si>
+    <t>Keep a balanced diet including fruits and vegetables. | Stay hydrated and maintain regular physical activities. | Limit alcohol consumption and avoid stress.</t>
+  </si>
+  <si>
+    <t>Continue encouraging the patient to adhere to healthy habits. | Monitor any upcoming visits for potential follow-ups.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment in two weeks. | Maintain a daily log of symptoms and lifestyle changes. | Consider joining a support group for long-term recovery.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:42:35.840Z</t>
+  </si>
+  <si>
+    <t>John Doe is currently in a stable condition after recovering from alcohol withdrawal. Vitals show normal ranges, but some symptoms such as confusion and sweating were noted during recovery.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Monitor confusion and sweating symptoms as they previously peaked in severity. Continued observation is advised.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable within normal range (120/80). | Heart Rate: Average around 70 bpm, within normal limits. | SpO2: Consistently above 97%, indicating good oxygenation. | Body Temperature: Normal range between 98.4°F and 98.6°F. | Blood Sugar: Fluctuations between 95 and 105 mg/dL, generally stable.</t>
+  </si>
+  <si>
+    <t>Regular meals and light exercises positively impact energy levels and vitals. | Melting ice cream syndrome observed during afternoon hours, correlating with increased sweating.</t>
+  </si>
+  <si>
+    <t>Maintain consistent meal times to help stabilize blood sugar levels. | Incorporate relaxation techniques to manage stress and reduce confusion.</t>
+  </si>
+  <si>
+    <t>Patient is responding well to recovery protocols; encourage adherence to follow-up appointments.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment to assess ongoing symptoms. | Continue monitoring vitals daily and keep a symptom diary.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:43:32.169Z</t>
+  </si>
+  <si>
+    <t>John Doe has successfully overcome Alcohol Withdrawal. His vital signs are mostly stable, but there are indications of occasional confusion and sweating.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Occasional confusion and sweating were noted; monitor for recurrence.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable around 120/80 mmHg, slight increase observed last reading. | Heart Rate: Normal, averaging around 70 bpm. | SpO2: Maintained at 97-99%, within normal range. | Body Temperature: Consistent around 98.4°F - 98.6°F. | Blood Sugar: Fluctuating but generally within acceptable levels.</t>
+  </si>
+  <si>
+    <t>Regular meals including breakfast and lunch appear to coincide with stable blood sugar levels. | Activity levels such as morning walks and light exercise contribute positively to overall vitality.</t>
+  </si>
+  <si>
+    <t>Continue regular physical activity such as walks to maintain health. | Stay hydrated and follow a balanced diet, focusing on fruits and vegetables.</t>
+  </si>
+  <si>
+    <t>Patient has shown improvement in symptoms related to alcohol withdrawal. Continue monitoring.</t>
+  </si>
+  <si>
+    <t>Keep a diary of symptoms, noting any days of increased confusion or sweating. | Schedule a follow-up appointment in two weeks to reassess condition.</t>
+  </si>
+  <si>
+    <t>2026-02-13T11:54:18.770Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, is experiencing shortness of breath with increasing severity over the past week. Monitoring of vital signs shows stable blood pressure and heart rate, but attention is needed for management of respiratory symptoms.</t>
+  </si>
+  <si>
+    <t>HIGH: Shortness of breath has been reported with increasing severity. Immediate consultation is recommended.</t>
+  </si>
+  <si>
+    <t>Blood Pressure: Stable with values around 120/80 mmHg. | Heart Rate: Consistent around 70 bpm. | SpO2: Normal at 97-99%. | Body Temperature: Normal range 98.4-98.6°F. | Blood Sugar: Slight fluctuations noted, with a peak of 105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Regular meals and morning activity have been noted, correlated with stable blood pressure and heart rate. | Shortness of breath symptoms appear more pronounced after physical activities.</t>
+  </si>
+  <si>
+    <t>Consider relaxing activities like deep breathing exercises or yoga to help with shortness of breath. | Maintain a consistent eating schedule and stay hydrated.</t>
+  </si>
+  <si>
+    <t>Monitoring of respiratory symptoms is essential. Recommend follow-up with a healthcare provider immediately if symptoms worsen.</t>
+  </si>
+  <si>
+    <t>Schedule a consultation with a healthcare provider regarding respiratory symptoms. | Continue monitoring vital signs daily and keep a record of any changes.</t>
   </si>
 </sst>
 </file>
@@ -2067,7 +2304,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R67"/>
+  <dimension ref="A1:R78"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -5535,6 +5772,622 @@
         <v>457</v>
       </c>
     </row>
+    <row r="68" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>560</v>
+      </c>
+      <c r="B68" t="s">
+        <v>19</v>
+      </c>
+      <c r="C68" t="s">
+        <v>20</v>
+      </c>
+      <c r="D68">
+        <v>36</v>
+      </c>
+      <c r="E68" t="s">
+        <v>356</v>
+      </c>
+      <c r="F68" t="s">
+        <v>357</v>
+      </c>
+      <c r="G68" t="s">
+        <v>561</v>
+      </c>
+      <c r="H68" t="s">
+        <v>562</v>
+      </c>
+      <c r="I68" t="s">
+        <v>563</v>
+      </c>
+      <c r="J68" t="s">
+        <v>564</v>
+      </c>
+      <c r="K68" t="s">
+        <v>565</v>
+      </c>
+      <c r="L68" t="s">
+        <v>566</v>
+      </c>
+      <c r="M68" t="s">
+        <v>567</v>
+      </c>
+      <c r="N68">
+        <v>2538</v>
+      </c>
+      <c r="O68">
+        <v>345</v>
+      </c>
+      <c r="P68">
+        <v>2883</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>34</v>
+      </c>
+      <c r="R68" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="69" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>568</v>
+      </c>
+      <c r="B69" t="s">
+        <v>19</v>
+      </c>
+      <c r="C69" t="s">
+        <v>20</v>
+      </c>
+      <c r="D69">
+        <v>36</v>
+      </c>
+      <c r="E69" t="s">
+        <v>356</v>
+      </c>
+      <c r="F69" t="s">
+        <v>357</v>
+      </c>
+      <c r="G69" t="s">
+        <v>569</v>
+      </c>
+      <c r="H69" t="s">
+        <v>570</v>
+      </c>
+      <c r="I69" t="s">
+        <v>571</v>
+      </c>
+      <c r="J69" t="s">
+        <v>572</v>
+      </c>
+      <c r="K69" t="s">
+        <v>573</v>
+      </c>
+      <c r="L69" t="s">
+        <v>574</v>
+      </c>
+      <c r="M69" t="s">
+        <v>575</v>
+      </c>
+      <c r="N69">
+        <v>2538</v>
+      </c>
+      <c r="O69">
+        <v>356</v>
+      </c>
+      <c r="P69">
+        <v>2894</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>34</v>
+      </c>
+      <c r="R69" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="70" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>576</v>
+      </c>
+      <c r="B70" t="s">
+        <v>19</v>
+      </c>
+      <c r="C70" t="s">
+        <v>20</v>
+      </c>
+      <c r="D70">
+        <v>36</v>
+      </c>
+      <c r="E70" t="s">
+        <v>356</v>
+      </c>
+      <c r="F70" t="s">
+        <v>357</v>
+      </c>
+      <c r="G70" t="s">
+        <v>577</v>
+      </c>
+      <c r="H70" t="s">
+        <v>578</v>
+      </c>
+      <c r="I70" t="s">
+        <v>579</v>
+      </c>
+      <c r="J70" t="s">
+        <v>580</v>
+      </c>
+      <c r="K70" t="s">
+        <v>581</v>
+      </c>
+      <c r="L70" t="s">
+        <v>582</v>
+      </c>
+      <c r="M70" t="s">
+        <v>583</v>
+      </c>
+      <c r="N70">
+        <v>2538</v>
+      </c>
+      <c r="O70">
+        <v>282</v>
+      </c>
+      <c r="P70">
+        <v>2820</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>34</v>
+      </c>
+      <c r="R70" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="71" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>584</v>
+      </c>
+      <c r="B71" t="s">
+        <v>19</v>
+      </c>
+      <c r="C71" t="s">
+        <v>20</v>
+      </c>
+      <c r="D71">
+        <v>36</v>
+      </c>
+      <c r="E71" t="s">
+        <v>356</v>
+      </c>
+      <c r="F71" t="s">
+        <v>357</v>
+      </c>
+      <c r="G71" t="s">
+        <v>585</v>
+      </c>
+      <c r="H71" t="s">
+        <v>492</v>
+      </c>
+      <c r="I71" t="s">
+        <v>586</v>
+      </c>
+      <c r="J71" t="s">
+        <v>587</v>
+      </c>
+      <c r="K71" t="s">
+        <v>588</v>
+      </c>
+      <c r="L71" t="s">
+        <v>589</v>
+      </c>
+      <c r="M71" t="s">
+        <v>590</v>
+      </c>
+      <c r="N71">
+        <v>2538</v>
+      </c>
+      <c r="O71">
+        <v>273</v>
+      </c>
+      <c r="P71">
+        <v>2811</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>34</v>
+      </c>
+      <c r="R71" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="72" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>591</v>
+      </c>
+      <c r="B72" t="s">
+        <v>19</v>
+      </c>
+      <c r="C72" t="s">
+        <v>20</v>
+      </c>
+      <c r="D72">
+        <v>36</v>
+      </c>
+      <c r="E72" t="s">
+        <v>356</v>
+      </c>
+      <c r="F72" t="s">
+        <v>357</v>
+      </c>
+      <c r="G72" t="s">
+        <v>592</v>
+      </c>
+      <c r="H72" t="s">
+        <v>593</v>
+      </c>
+      <c r="I72" t="s">
+        <v>594</v>
+      </c>
+      <c r="J72" t="s">
+        <v>595</v>
+      </c>
+      <c r="K72" t="s">
+        <v>596</v>
+      </c>
+      <c r="L72" t="s">
+        <v>597</v>
+      </c>
+      <c r="M72" t="s">
+        <v>598</v>
+      </c>
+      <c r="N72">
+        <v>2538</v>
+      </c>
+      <c r="O72">
+        <v>323</v>
+      </c>
+      <c r="P72">
+        <v>2861</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>34</v>
+      </c>
+      <c r="R72" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>599</v>
+      </c>
+      <c r="B73" t="s">
+        <v>19</v>
+      </c>
+      <c r="C73" t="s">
+        <v>20</v>
+      </c>
+      <c r="D73">
+        <v>36</v>
+      </c>
+      <c r="E73" t="s">
+        <v>356</v>
+      </c>
+      <c r="F73" t="s">
+        <v>357</v>
+      </c>
+      <c r="G73" t="s">
+        <v>600</v>
+      </c>
+      <c r="H73" t="s">
+        <v>601</v>
+      </c>
+      <c r="I73" t="s">
+        <v>602</v>
+      </c>
+      <c r="J73" t="s">
+        <v>603</v>
+      </c>
+      <c r="K73" t="s">
+        <v>604</v>
+      </c>
+      <c r="L73" t="s">
+        <v>605</v>
+      </c>
+      <c r="M73" t="s">
+        <v>606</v>
+      </c>
+      <c r="N73">
+        <v>2538</v>
+      </c>
+      <c r="O73">
+        <v>322</v>
+      </c>
+      <c r="P73">
+        <v>2860</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>34</v>
+      </c>
+      <c r="R73" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="74" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>607</v>
+      </c>
+      <c r="B74" t="s">
+        <v>19</v>
+      </c>
+      <c r="C74" t="s">
+        <v>20</v>
+      </c>
+      <c r="D74">
+        <v>36</v>
+      </c>
+      <c r="E74" t="s">
+        <v>356</v>
+      </c>
+      <c r="F74" t="s">
+        <v>357</v>
+      </c>
+      <c r="G74" t="s">
+        <v>608</v>
+      </c>
+      <c r="H74" t="s">
+        <v>609</v>
+      </c>
+      <c r="I74" t="s">
+        <v>610</v>
+      </c>
+      <c r="J74" t="s">
+        <v>611</v>
+      </c>
+      <c r="K74" t="s">
+        <v>612</v>
+      </c>
+      <c r="L74" t="s">
+        <v>613</v>
+      </c>
+      <c r="M74" t="s">
+        <v>614</v>
+      </c>
+      <c r="N74">
+        <v>2538</v>
+      </c>
+      <c r="O74">
+        <v>277</v>
+      </c>
+      <c r="P74">
+        <v>2815</v>
+      </c>
+      <c r="Q74" t="s">
+        <v>34</v>
+      </c>
+      <c r="R74" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="75" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>615</v>
+      </c>
+      <c r="B75" t="s">
+        <v>19</v>
+      </c>
+      <c r="C75" t="s">
+        <v>20</v>
+      </c>
+      <c r="D75">
+        <v>36</v>
+      </c>
+      <c r="E75" t="s">
+        <v>356</v>
+      </c>
+      <c r="F75" t="s">
+        <v>357</v>
+      </c>
+      <c r="G75" t="s">
+        <v>616</v>
+      </c>
+      <c r="H75" t="s">
+        <v>617</v>
+      </c>
+      <c r="I75" t="s">
+        <v>618</v>
+      </c>
+      <c r="J75" t="s">
+        <v>619</v>
+      </c>
+      <c r="K75" t="s">
+        <v>620</v>
+      </c>
+      <c r="L75" t="s">
+        <v>621</v>
+      </c>
+      <c r="M75" t="s">
+        <v>622</v>
+      </c>
+      <c r="N75">
+        <v>2538</v>
+      </c>
+      <c r="O75">
+        <v>318</v>
+      </c>
+      <c r="P75">
+        <v>2856</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>34</v>
+      </c>
+      <c r="R75" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="76" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>623</v>
+      </c>
+      <c r="B76" t="s">
+        <v>19</v>
+      </c>
+      <c r="C76" t="s">
+        <v>20</v>
+      </c>
+      <c r="D76">
+        <v>36</v>
+      </c>
+      <c r="E76" t="s">
+        <v>356</v>
+      </c>
+      <c r="F76" t="s">
+        <v>357</v>
+      </c>
+      <c r="G76" t="s">
+        <v>624</v>
+      </c>
+      <c r="H76" t="s">
+        <v>625</v>
+      </c>
+      <c r="I76" t="s">
+        <v>626</v>
+      </c>
+      <c r="J76" t="s">
+        <v>627</v>
+      </c>
+      <c r="K76" t="s">
+        <v>628</v>
+      </c>
+      <c r="L76" t="s">
+        <v>629</v>
+      </c>
+      <c r="M76" t="s">
+        <v>630</v>
+      </c>
+      <c r="N76">
+        <v>2538</v>
+      </c>
+      <c r="O76">
+        <v>309</v>
+      </c>
+      <c r="P76">
+        <v>2847</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>34</v>
+      </c>
+      <c r="R76" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="77" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>631</v>
+      </c>
+      <c r="B77" t="s">
+        <v>19</v>
+      </c>
+      <c r="C77" t="s">
+        <v>20</v>
+      </c>
+      <c r="D77">
+        <v>36</v>
+      </c>
+      <c r="E77" t="s">
+        <v>310</v>
+      </c>
+      <c r="F77" t="s">
+        <v>311</v>
+      </c>
+      <c r="G77" t="s">
+        <v>632</v>
+      </c>
+      <c r="H77" t="s">
+        <v>633</v>
+      </c>
+      <c r="I77" t="s">
+        <v>634</v>
+      </c>
+      <c r="J77" t="s">
+        <v>635</v>
+      </c>
+      <c r="K77" t="s">
+        <v>636</v>
+      </c>
+      <c r="L77" t="s">
+        <v>637</v>
+      </c>
+      <c r="M77" t="s">
+        <v>638</v>
+      </c>
+      <c r="N77">
+        <v>2611</v>
+      </c>
+      <c r="O77">
+        <v>328</v>
+      </c>
+      <c r="P77">
+        <v>2939</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>34</v>
+      </c>
+      <c r="R77" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="78" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>631</v>
+      </c>
+      <c r="B78" t="s">
+        <v>19</v>
+      </c>
+      <c r="C78" t="s">
+        <v>20</v>
+      </c>
+      <c r="D78">
+        <v>36</v>
+      </c>
+      <c r="E78" t="s">
+        <v>322</v>
+      </c>
+      <c r="F78" t="s">
+        <v>323</v>
+      </c>
+      <c r="G78" t="s">
+        <v>632</v>
+      </c>
+      <c r="H78" t="s">
+        <v>633</v>
+      </c>
+      <c r="I78" t="s">
+        <v>634</v>
+      </c>
+      <c r="J78" t="s">
+        <v>635</v>
+      </c>
+      <c r="K78" t="s">
+        <v>636</v>
+      </c>
+      <c r="L78" t="s">
+        <v>637</v>
+      </c>
+      <c r="M78" t="s">
+        <v>638</v>
+      </c>
+      <c r="N78">
+        <v>2611</v>
+      </c>
+      <c r="O78">
+        <v>328</v>
+      </c>
+      <c r="P78">
+        <v>2939</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>34</v>
+      </c>
+      <c r="R78" t="s">
+        <v>448</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update output.json with revised patient health summaries, including changes to vital signs, health alerts, and care recommendations. Modify pdfReport.js to enhance condition information handling based on type. Update health_records.xlsx to reflect recent data changes.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1196" uniqueCount="639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="647">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1928,6 +1928,30 @@
   </si>
   <si>
     <t>Schedule a consultation with a healthcare provider regarding respiratory symptoms. | Continue monitoring vital signs daily and keep a record of any changes.</t>
+  </si>
+  <si>
+    <t>2026-02-13T13:50:10.787Z</t>
+  </si>
+  <si>
+    <t>John Doe has experienced occasional shortness of breath and signs of forgetfulness. His vital signs remain mostly stable, but some aspects show variability that may need attention.</t>
+  </si>
+  <si>
+    <t>HIGH: Shortness of breath severity has reached critical levels. Immediate evaluation is advised.</t>
+  </si>
+  <si>
+    <t>Blood pressure is generally stable, averaging 120/80 mmHg. | Heart rate fluctuates between 68 and 73 bpm. | SpO2 levels are consistently around 97-99%. | Body temperature remains normal at around 98.4-98.6°F. | Blood sugar levels show slight variability, peaking at 105 mg/dL.</t>
+  </si>
+  <si>
+    <t>Routine meals are consistent with breakfast being the most common activity. | Physical activity, such as morning walks, is integrated into the daily routine.</t>
+  </si>
+  <si>
+    <t>Consider deep breathing exercises to manage shortness of breath. | Increase physical activity, such as light exercises, to enhance overall fitness. | Establish reminders for daily activities to aid with forgetfulness.</t>
+  </si>
+  <si>
+    <t>Monitor the severity of symptoms daily and adjust activities accordingly. | Focus on maintaining a balanced diet and regular exercise.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with a healthcare provider to discuss shortness of breath. | Implement daily reminders for activities to support cognitive function. | Continue tracking vital signs and report any significant changes.</t>
   </si>
 </sst>
 </file>
@@ -2304,7 +2328,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R78"/>
+  <dimension ref="A1:R80"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -6388,6 +6412,118 @@
         <v>448</v>
       </c>
     </row>
+    <row r="79" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>639</v>
+      </c>
+      <c r="B79" t="s">
+        <v>19</v>
+      </c>
+      <c r="C79" t="s">
+        <v>20</v>
+      </c>
+      <c r="D79">
+        <v>36</v>
+      </c>
+      <c r="E79" t="s">
+        <v>310</v>
+      </c>
+      <c r="F79" t="s">
+        <v>311</v>
+      </c>
+      <c r="G79" t="s">
+        <v>640</v>
+      </c>
+      <c r="H79" t="s">
+        <v>641</v>
+      </c>
+      <c r="I79" t="s">
+        <v>642</v>
+      </c>
+      <c r="J79" t="s">
+        <v>643</v>
+      </c>
+      <c r="K79" t="s">
+        <v>644</v>
+      </c>
+      <c r="L79" t="s">
+        <v>645</v>
+      </c>
+      <c r="M79" t="s">
+        <v>646</v>
+      </c>
+      <c r="N79">
+        <v>2611</v>
+      </c>
+      <c r="O79">
+        <v>344</v>
+      </c>
+      <c r="P79">
+        <v>2955</v>
+      </c>
+      <c r="Q79" t="s">
+        <v>34</v>
+      </c>
+      <c r="R79" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="80" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>639</v>
+      </c>
+      <c r="B80" t="s">
+        <v>19</v>
+      </c>
+      <c r="C80" t="s">
+        <v>20</v>
+      </c>
+      <c r="D80">
+        <v>36</v>
+      </c>
+      <c r="E80" t="s">
+        <v>322</v>
+      </c>
+      <c r="F80" t="s">
+        <v>323</v>
+      </c>
+      <c r="G80" t="s">
+        <v>640</v>
+      </c>
+      <c r="H80" t="s">
+        <v>641</v>
+      </c>
+      <c r="I80" t="s">
+        <v>642</v>
+      </c>
+      <c r="J80" t="s">
+        <v>643</v>
+      </c>
+      <c r="K80" t="s">
+        <v>644</v>
+      </c>
+      <c r="L80" t="s">
+        <v>645</v>
+      </c>
+      <c r="M80" t="s">
+        <v>646</v>
+      </c>
+      <c r="N80">
+        <v>2611</v>
+      </c>
+      <c r="O80">
+        <v>344</v>
+      </c>
+      <c r="P80">
+        <v>2955</v>
+      </c>
+      <c r="Q80" t="s">
+        <v>34</v>
+      </c>
+      <c r="R80" t="s">
+        <v>448</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Implement payload hashing in index.js for improved data integrity. Update AiInsight schema to include unique payloadHash field, ensuring no duplicate insights are stored. Revise output.json with enhanced patient health summaries and recommendations. Update health_records.xlsx to reflect recent changes.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1224" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="656">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1952,6 +1952,33 @@
   </si>
   <si>
     <t>Schedule a follow-up appointment with a healthcare provider to discuss shortness of breath. | Implement daily reminders for activities to support cognitive function. | Continue tracking vital signs and report any significant changes.</t>
+  </si>
+  <si>
+    <t>2026-02-17T07:29:10.224Z</t>
+  </si>
+  <si>
+    <t>John Doe is currently experiencing some concerning symptoms, including shortness of breath and forgetfulness linked to ADHD. Vitals have remained stable but require monitoring.</t>
+  </si>
+  <si>
+    <t>HIGH: Shortness of breath severity levels have reached concerning heights. Immediate medical attention may be required.</t>
+  </si>
+  <si>
+    <t>Heart rate has ranged from 69 to 74 bpm. Blood pressure readings are well within normal limits, ranging from 117/77 to 122/82 mmHg. Oxygen saturation levels have remained healthy, ranging from 97% to 99%.</t>
+  </si>
+  <si>
+    <t>Regular meals and light exercise like morning walks are observed, which may positively affect overall health. | Increased forgetfulness has been noted which could correlate with activities and routine.</t>
+  </si>
+  <si>
+    <t>Maintain a consistent meal schedule to support cognitive function. | Incorporate more physical activities throughout the day to improve overall stamina. | Consider mindfulness or meditation practices to help with focus and attention.</t>
+  </si>
+  <si>
+    <t>Monitor John's symptoms closely, particularly noting any episodes of shortness of breath. | Engagement in cognitive exercises could be beneficial for managing ADHD symptoms.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment to discuss shortness of breath and possible further evaluation. | Record daily symptoms and activities to identify triggers and improve symptom management.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","status":"suspected","symptom_lookup_id":"56f51f54-0b28-4e3a-b5ca-1344f2f2cc4a","symptom_title":"short of breath","symptoms":[{"records":[{"severity":6,"recorded_at":"2026-02-12T11:22:02.375Z"},{"severity":7,"recorded_at":"2026-02-11T09:18:17.203Z"},{"severity":8,"recorded_at":"2026-02-10T08:18:17.203Z"},{"severity":10,"recorded_at":"2026-02-09T07:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-08T11:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-07T06:30:15.500Z"}],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","status":"suspected","symptom_lookup_id":"cc50560b-a35e-4315-9856-7c693335dbb0","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[{"severity":7,"recorded_at":"2026-02-12T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-11T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-10T07:35:35.042Z"},{"severity":4,"recorded_at":"2026-02-09T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-08T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-07T07:35:35.042Z"},{"severity":7,"recorded_at":"2026-02-06T07:35:35.042Z"}],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"record_id":"698d8b1dbb05e0b7c13a201a","recorded_at":"2026-02-11T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-11T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201b","vital_type":"HEART_RATE","value":74,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a201c","vital_type":"BLOOD_PRESSURE","value":{"systolic":122,"diastolic":82},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a201d","vital_type":"SPO2","value":97,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201c","recorded_at":"2026-02-12T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-12T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201e","vital_type":"HEART_RATE","value":72,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2021","vital_type":"BLOOD_PRESSURE","value":{"systolic":120,"diastolic":80},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2024","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201d","recorded_at":"2026-02-13T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-13T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201f","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2022","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2025","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2026","recorded_at":"2026-02-14T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-14T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2027","vital_type":"HEART_RATE","value":71,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2028","vital_type":"BLOOD_PRESSURE","value":{"systolic":119,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2029","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202a","recorded_at":"2026-02-15T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-15T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202b","vital_type":"HEART_RATE","value":69,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a202c","vital_type":"BLOOD_PRESSURE","value":{"systolic":117,"diastolic":77},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a202d","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202e","recorded_at":"2026-02-16T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-16T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202f","vital_type":"HEART_RATE","value":73,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2030","vital_type":"BLOOD_PRESSURE","value":{"systolic":121,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2031","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2032","recorded_at":"2026-02-17T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-17T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2033","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2034","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2035","vital_type":"SPO2","value":99,"unit":"%"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
   </si>
 </sst>
 </file>
@@ -2328,7 +2355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R80"/>
+  <dimension ref="A1:R82"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -6524,6 +6551,118 @@
         <v>448</v>
       </c>
     </row>
+    <row r="81" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>647</v>
+      </c>
+      <c r="B81" t="s">
+        <v>19</v>
+      </c>
+      <c r="C81" t="s">
+        <v>20</v>
+      </c>
+      <c r="D81">
+        <v>36</v>
+      </c>
+      <c r="E81" t="s">
+        <v>310</v>
+      </c>
+      <c r="F81" t="s">
+        <v>311</v>
+      </c>
+      <c r="G81" t="s">
+        <v>648</v>
+      </c>
+      <c r="H81" t="s">
+        <v>649</v>
+      </c>
+      <c r="I81" t="s">
+        <v>650</v>
+      </c>
+      <c r="J81" t="s">
+        <v>651</v>
+      </c>
+      <c r="K81" t="s">
+        <v>652</v>
+      </c>
+      <c r="L81" t="s">
+        <v>653</v>
+      </c>
+      <c r="M81" t="s">
+        <v>654</v>
+      </c>
+      <c r="N81">
+        <v>3169</v>
+      </c>
+      <c r="O81">
+        <v>321</v>
+      </c>
+      <c r="P81">
+        <v>3490</v>
+      </c>
+      <c r="Q81" t="s">
+        <v>34</v>
+      </c>
+      <c r="R81" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="82" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>647</v>
+      </c>
+      <c r="B82" t="s">
+        <v>19</v>
+      </c>
+      <c r="C82" t="s">
+        <v>20</v>
+      </c>
+      <c r="D82">
+        <v>36</v>
+      </c>
+      <c r="E82" t="s">
+        <v>322</v>
+      </c>
+      <c r="F82" t="s">
+        <v>323</v>
+      </c>
+      <c r="G82" t="s">
+        <v>648</v>
+      </c>
+      <c r="H82" t="s">
+        <v>649</v>
+      </c>
+      <c r="I82" t="s">
+        <v>650</v>
+      </c>
+      <c r="J82" t="s">
+        <v>651</v>
+      </c>
+      <c r="K82" t="s">
+        <v>652</v>
+      </c>
+      <c r="L82" t="s">
+        <v>653</v>
+      </c>
+      <c r="M82" t="s">
+        <v>654</v>
+      </c>
+      <c r="N82">
+        <v>3169</v>
+      </c>
+      <c r="O82">
+        <v>321</v>
+      </c>
+      <c r="P82">
+        <v>3490</v>
+      </c>
+      <c r="Q82" t="s">
+        <v>34</v>
+      </c>
+      <c r="R82" t="s">
+        <v>655</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Update patient health summaries in output.json for clarity and detail, including revised overall summary and health alerts. Adjust daily patterns and smart advice for better alignment with patient progress. Modify index.js to correct condition normalization and enhance logging for cache operations. Update health_records.xlsx to reflect recent changes.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="656">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="682">
   <si>
     <t>Timestamp</t>
   </si>
@@ -1979,6 +1979,84 @@
   </si>
   <si>
     <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","status":"suspected","symptom_lookup_id":"56f51f54-0b28-4e3a-b5ca-1344f2f2cc4a","symptom_title":"short of breath","symptoms":[{"records":[{"severity":6,"recorded_at":"2026-02-12T11:22:02.375Z"},{"severity":7,"recorded_at":"2026-02-11T09:18:17.203Z"},{"severity":8,"recorded_at":"2026-02-10T08:18:17.203Z"},{"severity":10,"recorded_at":"2026-02-09T07:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-08T11:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-07T06:30:15.500Z"}],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","status":"suspected","symptom_lookup_id":"cc50560b-a35e-4315-9856-7c693335dbb0","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[{"severity":7,"recorded_at":"2026-02-12T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-11T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-10T07:35:35.042Z"},{"severity":4,"recorded_at":"2026-02-09T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-08T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-07T07:35:35.042Z"},{"severity":7,"recorded_at":"2026-02-06T07:35:35.042Z"}],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"record_id":"698d8b1dbb05e0b7c13a201a","recorded_at":"2026-02-11T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-11T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201b","vital_type":"HEART_RATE","value":74,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a201c","vital_type":"BLOOD_PRESSURE","value":{"systolic":122,"diastolic":82},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a201d","vital_type":"SPO2","value":97,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201c","recorded_at":"2026-02-12T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-12T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201e","vital_type":"HEART_RATE","value":72,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2021","vital_type":"BLOOD_PRESSURE","value":{"systolic":120,"diastolic":80},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2024","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201d","recorded_at":"2026-02-13T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-13T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201f","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2022","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2025","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2026","recorded_at":"2026-02-14T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-14T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2027","vital_type":"HEART_RATE","value":71,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2028","vital_type":"BLOOD_PRESSURE","value":{"systolic":119,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2029","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202a","recorded_at":"2026-02-15T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-15T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202b","vital_type":"HEART_RATE","value":69,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a202c","vital_type":"BLOOD_PRESSURE","value":{"systolic":117,"diastolic":77},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a202d","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202e","recorded_at":"2026-02-16T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-16T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202f","vital_type":"HEART_RATE","value":73,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2030","vital_type":"BLOOD_PRESSURE","value":{"systolic":121,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2031","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2032","recorded_at":"2026-02-17T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-17T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2033","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2034","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2035","vital_type":"SPO2","value":99,"unit":"%"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
+  </si>
+  <si>
+    <t>2026-02-17T08:55:06.375Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has experienced increasing severity in symptoms like shortness of breath and forgetfulness linked to ADHD. His vital signs are mostly stable, but certain symptoms require attention.</t>
+  </si>
+  <si>
+    <t>HIGH: Shortness of breath severity is increasing! Immediate attention is suggested.</t>
+  </si>
+  <si>
+    <t>Heart rate ranged from 69 to 74 bpm, indicating a generally stable condition. | Blood pressure readings are within normal limits, highest being 122/82 mmHg. | Oxygen saturation levels are stable, mostly at 97% to 99%.</t>
+  </si>
+  <si>
+    <t>Routine activities like breakfast and walks are consistent, which may help manage symptoms. | There are fluctuations in forgetfulness severity during different times of the day.</t>
+  </si>
+  <si>
+    <t>Maintain a routine schedule to enhance memory and cognitive function. | Regular light exercises such as walking can improve respiratory function.</t>
+  </si>
+  <si>
+    <t>Monitor the patient's symptoms closely. | Consider a medication review for managing ADHD symptoms more effectively.</t>
+  </si>
+  <si>
+    <t>Schedule an appointment with a healthcare provider to discuss increasing severity of symptoms. | Consider implementing a daily planner to assist with memory issues.</t>
+  </si>
+  <si>
+    <t>2026-02-17T08:57:07.141Z</t>
+  </si>
+  <si>
+    <t>John Doe has successfully overcome alcohol withdrawal symptoms. Overall, vital signs appear stable.</t>
+  </si>
+  <si>
+    <t>LOW: Mild confusion and sweating symptoms reported but no urgent issues identified.</t>
+  </si>
+  <si>
+    <t>Heart rate ranges from 69 to 74 bpm, Blood pressure is stable between 117/77 to 122/82 mmHg, SPO2 levels consistently above 97%.</t>
+  </si>
+  <si>
+    <t>Routine activities, including regular meals and light exercise, contribute positively to vital signs.</t>
+  </si>
+  <si>
+    <t>Continue regular meals and light exercises, stay hydrated, and maintain a balanced diet.</t>
+  </si>
+  <si>
+    <t>Monitor any recurrence of symptoms and maintain regular follow-ups to ensure well-being.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with the care team in one month.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":5,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"record_id":"698d8b1dbb05e0b7c13a201a","recorded_at":"2026-02-11T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-11T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201b","vital_type":"HEART_RATE","value":74,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a201c","vital_type":"BLOOD_PRESSURE","value":{"systolic":122,"diastolic":82},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a201d","vital_type":"SPO2","value":97,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201c","recorded_at":"2026-02-12T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-12T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201e","vital_type":"HEART_RATE","value":72,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2021","vital_type":"BLOOD_PRESSURE","value":{"systolic":120,"diastolic":80},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2024","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201d","recorded_at":"2026-02-13T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-13T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201f","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2022","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2025","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2026","recorded_at":"2026-02-14T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-14T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2027","vital_type":"HEART_RATE","value":71,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2028","vital_type":"BLOOD_PRESSURE","value":{"systolic":119,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2029","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202a","recorded_at":"2026-02-15T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-15T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202b","vital_type":"HEART_RATE","value":69,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a202c","vital_type":"BLOOD_PRESSURE","value":{"systolic":117,"diastolic":77},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a202d","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202e","recorded_at":"2026-02-16T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-16T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202f","vital_type":"HEART_RATE","value":73,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2030","vital_type":"BLOOD_PRESSURE","value":{"systolic":121,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2031","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2032","recorded_at":"2026-02-17T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-17T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2033","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2034","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2035","vital_type":"SPO2","value":99,"unit":"%"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
+  </si>
+  <si>
+    <t>2026-02-17T09:00:33.892Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has successfully overcome alcohol withdrawal symptoms. While confusion and sweating were significant during his recovery, current vital signs indicate stability. Continued monitoring and support are essential for long-term health.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Monitor signs of confusion and sweating closely to ensure ongoing improvement.</t>
+  </si>
+  <si>
+    <t>Heart Rate: Ranged from 69 to 74 bpm, indicating stability. | Blood Pressure: Consistently within normal limits, ranging from 117/77 to 122/82 mmHg. | Oxygen Saturation: Maintained between 97% to 99%, suggesting healthy lung function.</t>
+  </si>
+  <si>
+    <t>Regular meal times and light exercise appear to correlate with stable vitals. | Increased sweating and confusion were observed prior to certain activities, indicating a possible reaction to stress or environmental factors.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet with a focus on hydration and nutrition to support recovery. | Incorporate a daily routine of light exercises, such as walking, to promote overall wellness.</t>
+  </si>
+  <si>
+    <t>Continue to monitor psychological and physical symptoms closely. Encourage regular check-ins. | Patient shows good progress, but vigilance is necessary for signs of relapse.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up consultation with the healthcare provider in one week. | Implement a daily log for symptoms and activities to discuss during the next appointment.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":7,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"record_id":"698d8b1dbb05e0b7c13a201a","recorded_at":"2026-02-11T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-11T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201b","vital_type":"HEART_RATE","value":74,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a201c","vital_type":"BLOOD_PRESSURE","value":{"systolic":122,"diastolic":82},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a201d","vital_type":"SPO2","value":97,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201c","recorded_at":"2026-02-12T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-12T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201e","vital_type":"HEART_RATE","value":72,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2021","vital_type":"BLOOD_PRESSURE","value":{"systolic":120,"diastolic":80},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2024","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201d","recorded_at":"2026-02-13T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-13T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201f","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2022","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2025","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2026","recorded_at":"2026-02-14T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-14T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2027","vital_type":"HEART_RATE","value":71,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2028","vital_type":"BLOOD_PRESSURE","value":{"systolic":119,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2029","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202a","recorded_at":"2026-02-15T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-15T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202b","vital_type":"HEART_RATE","value":69,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a202c","vital_type":"BLOOD_PRESSURE","value":{"systolic":117,"diastolic":77},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a202d","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202e","recorded_at":"2026-02-16T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-16T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202f","vital_type":"HEART_RATE","value":73,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2030","vital_type":"BLOOD_PRESSURE","value":{"systolic":121,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2031","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2032","recorded_at":"2026-02-17T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-17T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2033","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2034","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2035","vital_type":"SPO2","value":99,"unit":"%"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
   </si>
 </sst>
 </file>
@@ -2355,7 +2433,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R82"/>
+  <dimension ref="A1:R86"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -6663,6 +6741,230 @@
         <v>655</v>
       </c>
     </row>
+    <row r="83" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>656</v>
+      </c>
+      <c r="B83" t="s">
+        <v>19</v>
+      </c>
+      <c r="C83" t="s">
+        <v>20</v>
+      </c>
+      <c r="D83">
+        <v>36</v>
+      </c>
+      <c r="E83" t="s">
+        <v>310</v>
+      </c>
+      <c r="F83" t="s">
+        <v>311</v>
+      </c>
+      <c r="G83" t="s">
+        <v>657</v>
+      </c>
+      <c r="H83" t="s">
+        <v>658</v>
+      </c>
+      <c r="I83" t="s">
+        <v>659</v>
+      </c>
+      <c r="J83" t="s">
+        <v>660</v>
+      </c>
+      <c r="K83" t="s">
+        <v>661</v>
+      </c>
+      <c r="L83" t="s">
+        <v>662</v>
+      </c>
+      <c r="M83" t="s">
+        <v>663</v>
+      </c>
+      <c r="N83">
+        <v>3169</v>
+      </c>
+      <c r="O83">
+        <v>295</v>
+      </c>
+      <c r="P83">
+        <v>3464</v>
+      </c>
+      <c r="Q83" t="s">
+        <v>34</v>
+      </c>
+      <c r="R83" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="84" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>656</v>
+      </c>
+      <c r="B84" t="s">
+        <v>19</v>
+      </c>
+      <c r="C84" t="s">
+        <v>20</v>
+      </c>
+      <c r="D84">
+        <v>36</v>
+      </c>
+      <c r="E84" t="s">
+        <v>322</v>
+      </c>
+      <c r="F84" t="s">
+        <v>323</v>
+      </c>
+      <c r="G84" t="s">
+        <v>657</v>
+      </c>
+      <c r="H84" t="s">
+        <v>658</v>
+      </c>
+      <c r="I84" t="s">
+        <v>659</v>
+      </c>
+      <c r="J84" t="s">
+        <v>660</v>
+      </c>
+      <c r="K84" t="s">
+        <v>661</v>
+      </c>
+      <c r="L84" t="s">
+        <v>662</v>
+      </c>
+      <c r="M84" t="s">
+        <v>663</v>
+      </c>
+      <c r="N84">
+        <v>3169</v>
+      </c>
+      <c r="O84">
+        <v>295</v>
+      </c>
+      <c r="P84">
+        <v>3464</v>
+      </c>
+      <c r="Q84" t="s">
+        <v>34</v>
+      </c>
+      <c r="R84" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="85" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>664</v>
+      </c>
+      <c r="B85" t="s">
+        <v>19</v>
+      </c>
+      <c r="C85" t="s">
+        <v>20</v>
+      </c>
+      <c r="D85">
+        <v>36</v>
+      </c>
+      <c r="E85" t="s">
+        <v>356</v>
+      </c>
+      <c r="F85" t="s">
+        <v>357</v>
+      </c>
+      <c r="G85" t="s">
+        <v>665</v>
+      </c>
+      <c r="H85" t="s">
+        <v>666</v>
+      </c>
+      <c r="I85" t="s">
+        <v>667</v>
+      </c>
+      <c r="J85" t="s">
+        <v>668</v>
+      </c>
+      <c r="K85" t="s">
+        <v>669</v>
+      </c>
+      <c r="L85" t="s">
+        <v>670</v>
+      </c>
+      <c r="M85" t="s">
+        <v>671</v>
+      </c>
+      <c r="N85">
+        <v>3096</v>
+      </c>
+      <c r="O85">
+        <v>211</v>
+      </c>
+      <c r="P85">
+        <v>3307</v>
+      </c>
+      <c r="Q85" t="s">
+        <v>34</v>
+      </c>
+      <c r="R85" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>673</v>
+      </c>
+      <c r="B86" t="s">
+        <v>19</v>
+      </c>
+      <c r="C86" t="s">
+        <v>20</v>
+      </c>
+      <c r="D86">
+        <v>36</v>
+      </c>
+      <c r="E86" t="s">
+        <v>356</v>
+      </c>
+      <c r="F86" t="s">
+        <v>357</v>
+      </c>
+      <c r="G86" t="s">
+        <v>674</v>
+      </c>
+      <c r="H86" t="s">
+        <v>675</v>
+      </c>
+      <c r="I86" t="s">
+        <v>676</v>
+      </c>
+      <c r="J86" t="s">
+        <v>677</v>
+      </c>
+      <c r="K86" t="s">
+        <v>678</v>
+      </c>
+      <c r="L86" t="s">
+        <v>679</v>
+      </c>
+      <c r="M86" t="s">
+        <v>680</v>
+      </c>
+      <c r="N86">
+        <v>3096</v>
+      </c>
+      <c r="O86">
+        <v>340</v>
+      </c>
+      <c r="P86">
+        <v>3436</v>
+      </c>
+      <c r="Q86" t="s">
+        <v>34</v>
+      </c>
+      <c r="R86" t="s">
+        <v>681</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
Refactor condition handling in index.js by introducing a new sorting function and updating symptom records to use a simplified format for severity and timestamps. Revise overall health summary and alerts in output.json for improved clarity and urgency. Update health_records.xlsx to reflect the latest data changes.
</commit_message>
<xml_diff>
--- a/health_records.xlsx
+++ b/health_records.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1308" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1616" uniqueCount="799">
   <si>
     <t>Timestamp</t>
   </si>
@@ -2057,6 +2057,357 @@
   </si>
   <si>
     <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","status":"cured","disease_lookup_id":"e47e34b0-430a-4353-9935-7aa526d0686e","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[{"severity":7,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":6,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":4,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":5,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":3,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":4,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]},{"title":"sweating","records":[{"severity":6,"recorded_at":"2026-02-03T09:00:00.000Z"},{"severity":5,"recorded_at":"2026-02-04T09:15:00.000Z"},{"severity":5,"recorded_at":"2026-02-05T08:45:00.000Z"},{"severity":4,"recorded_at":"2026-02-06T09:30:00.000Z"},{"severity":4,"recorded_at":"2026-02-07T08:50:00.000Z"},{"severity":3,"recorded_at":"2026-02-08T09:10:00.000Z"},{"severity":2,"recorded_at":"2026-02-09T09:00:00.000Z"}]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"record_id":"698d8b1dbb05e0b7c13a201a","recorded_at":"2026-02-11T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-11T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201b","vital_type":"HEART_RATE","value":74,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a201c","vital_type":"BLOOD_PRESSURE","value":{"systolic":122,"diastolic":82},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a201d","vital_type":"SPO2","value":97,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201c","recorded_at":"2026-02-12T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-12T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201e","vital_type":"HEART_RATE","value":72,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2021","vital_type":"BLOOD_PRESSURE","value":{"systolic":120,"diastolic":80},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2024","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201d","recorded_at":"2026-02-13T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-13T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201f","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2022","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2025","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2026","recorded_at":"2026-02-14T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-14T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2027","vital_type":"HEART_RATE","value":71,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2028","vital_type":"BLOOD_PRESSURE","value":{"systolic":119,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2029","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202a","recorded_at":"2026-02-15T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-15T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202b","vital_type":"HEART_RATE","value":69,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a202c","vital_type":"BLOOD_PRESSURE","value":{"systolic":117,"diastolic":77},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a202d","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202e","recorded_at":"2026-02-16T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-16T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202f","vital_type":"HEART_RATE","value":73,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2030","vital_type":"BLOOD_PRESSURE","value":{"systolic":121,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2031","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2032","recorded_at":"2026-02-17T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-17T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2033","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2034","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2035","vital_type":"SPO2","value":99,"unit":"%"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:39:19.885Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has reported experiencing shortness of breath and forgetfulness in daily activities. His vital signs are generally stable, but he shows some fluctuation in heart rate.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Shortness of breath has been noted on multiple occasions; please monitor and consult a healthcare provider if it persists.</t>
+  </si>
+  <si>
+    <t>Heart Rate: Ranging from 69 to 74 bpm, generally stable. | Blood Pressure: Ranging from 117/77 to 122/82 mmHg, within normal limits. | Oxygen Saturation: Ranging from 97% to 99%, stable.</t>
+  </si>
+  <si>
+    <t>Breakfast is consistently consumed daily, followed by light activities like morning walks. | Activity appears to correlate with stable heart rate and blood pressure readings.</t>
+  </si>
+  <si>
+    <t>Consider reducing stress through mindfulness or relaxation techniques to help with forgetfulness. | Maintain regular meal patterns and hydration to support overall health.</t>
+  </si>
+  <si>
+    <t>Monitoring the patient’s shortness of breath is advised; maintain a log of symptoms.</t>
+  </si>
+  <si>
+    <t>Schedule a consultation with a healthcare provider to address the shortness of breath. | Continue regular monitoring of vitals and symptoms.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12T11:22:02.375Z"],[7,"2026-02-11T09:18:17.203Z"],[8,"2026-02-10T08:18:17.203Z"],[10,"2026-02-09T07:18:17.203Z"],[5,"2026-02-08T11:18:17.203Z"],[5,"2026-02-07T06:30:15.500Z"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[7,"2026-02-12T07:35:35.042Z"],[6,"2026-02-11T07:35:35.042Z"],[5,"2026-02-10T07:35:35.042Z"],[4,"2026-02-09T07:35:35.042Z"],[5,"2026-02-08T07:35:35.042Z"],[6,"2026-02-07T07:35:35.042Z"],[7,"2026-02-06T07:35:35.042Z"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"record_id":"698d8b1dbb05e0b7c13a201a","recorded_at":"2026-02-11T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-11T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201b","vital_type":"HEART_RATE","value":74,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a201c","vital_type":"BLOOD_PRESSURE","value":{"systolic":122,"diastolic":82},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a201d","vital_type":"SPO2","value":97,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201c","recorded_at":"2026-02-12T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-12T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201e","vital_type":"HEART_RATE","value":72,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2021","vital_type":"BLOOD_PRESSURE","value":{"systolic":120,"diastolic":80},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2024","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201d","recorded_at":"2026-02-13T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-13T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201f","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2022","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2025","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2026","recorded_at":"2026-02-14T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-14T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2027","vital_type":"HEART_RATE","value":71,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2028","vital_type":"BLOOD_PRESSURE","value":{"systolic":119,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2029","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202a","recorded_at":"2026-02-15T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-15T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202b","vital_type":"HEART_RATE","value":69,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a202c","vital_type":"BLOOD_PRESSURE","value":{"systolic":117,"diastolic":77},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a202d","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202e","recorded_at":"2026-02-16T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-16T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202f","vital_type":"HEART_RATE","value":73,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2030","vital_type":"BLOOD_PRESSURE","value":{"systolic":121,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2031","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2032","recorded_at":"2026-02-17T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-17T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2033","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2034","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2035","vital_type":"SPO2","value":99,"unit":"%"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:40:08.170Z</t>
+  </si>
+  <si>
+    <t>John Doe is experiencing shortness of breath and forgetfulness in daily activities. These symptoms have fluctuated in severity but show noticeable peaks that require careful monitoring.</t>
+  </si>
+  <si>
+    <t>HIGH: Severe shortness of breath recorded with a peak severity of 10 on February 9. Immediate medical attention recommended.</t>
+  </si>
+  <si>
+    <t>Heart rate averages between 69-74 bpm, which is within normal range. | Blood pressure readings are consistent: systolic between 117-122 mmHg and diastolic between 77-82 mmHg. | Oxygen saturation levels are stable, ranging from 97% to 99%.</t>
+  </si>
+  <si>
+    <t>Regular meal timings with breakfast occurring around the same time daily. | Incorporating morning walks may contribute positively to daily vitality and well-being.</t>
+  </si>
+  <si>
+    <t>Consider stress management techniques to improve focus and reduce forgetfulness, including mindfulness and regular breaks. | Maintain a balanced diet rich in fruits and vegetables to support overall health.</t>
+  </si>
+  <si>
+    <t>Continued monitoring of shortness of breath is essential. Follow up if symptoms worsen. | Encourage patient to document daily activities and symptoms for better management.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with a healthcare provider to discuss symptoms and potential treatments. | Consider keeping a daily log of symptoms and feelings to share with the care team.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","status":"suspected","symptom_lookup_id":"56f51f54-0b28-4e3a-b5ca-1344f2f2cc4a","symptom_title":"short of breath","symptoms":[{"records":[{"severity":6,"recorded_at":"2026-02-12T11:22:02.375Z"},{"severity":7,"recorded_at":"2026-02-11T09:18:17.203Z"},{"severity":8,"recorded_at":"2026-02-10T08:18:17.203Z"},{"severity":10,"recorded_at":"2026-02-09T07:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-08T11:18:17.203Z"},{"severity":5,"recorded_at":"2026-02-07T06:30:15.500Z"}],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","status":"suspected","symptom_lookup_id":"cc50560b-a35e-4315-9856-7c693335dbb0","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[{"severity":9,"recorded_at":"2026-02-12T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-11T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-10T07:35:35.042Z"},{"severity":4,"recorded_at":"2026-02-09T07:35:35.042Z"},{"severity":5,"recorded_at":"2026-02-08T07:35:35.042Z"},{"severity":6,"recorded_at":"2026-02-07T07:35:35.042Z"},{"severity":7,"recorded_at":"2026-02-06T07:35:35.042Z"}],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"record_id":"698d8b1dbb05e0b7c13a201a","recorded_at":"2026-02-11T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-11T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201b","vital_type":"HEART_RATE","value":74,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a201c","vital_type":"BLOOD_PRESSURE","value":{"systolic":122,"diastolic":82},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a201d","vital_type":"SPO2","value":97,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201c","recorded_at":"2026-02-12T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-12T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201e","vital_type":"HEART_RATE","value":72,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2021","vital_type":"BLOOD_PRESSURE","value":{"systolic":120,"diastolic":80},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2024","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a201d","recorded_at":"2026-02-13T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-13T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a201f","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2022","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2025","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2026","recorded_at":"2026-02-14T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-14T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2027","vital_type":"HEART_RATE","value":71,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2028","vital_type":"BLOOD_PRESSURE","value":{"systolic":119,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2029","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202a","recorded_at":"2026-02-15T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-15T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202b","vital_type":"HEART_RATE","value":69,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a202c","vital_type":"BLOOD_PRESSURE","value":{"systolic":117,"diastolic":77},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a202d","vital_type":"SPO2","value":99,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a202e","recorded_at":"2026-02-16T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-16T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a202f","vital_type":"HEART_RATE","value":73,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2030","vital_type":"BLOOD_PRESSURE","value":{"systolic":121,"diastolic":79},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2031","vital_type":"SPO2","value":98,"unit":"%"}]},{"record_id":"698d8b1dbb05e0b7c13a2032","recorded_at":"2026-02-17T08:11:09.381Z","recorded_by":{"role":"patient","lookup_id":"66834a2a-e734-4378-b3fe-d43cc817a4de"},"created_at":"2026-02-17T08:11:09.396Z","vitals":[{"vital_id":"698d8b1dbb05e0b7c13a2033","vital_type":"HEART_RATE","value":70,"unit":"bpm"},{"vital_id":"698d8b1dbb05e0b7c13a2034","vital_type":"BLOOD_PRESSURE","value":{"systolic":118,"diastolic":78},"unit":"mmHg"},{"vital_id":"698d8b1dbb05e0b7c13a2035","vital_type":"SPO2","value":99,"unit":"%"}]}],"activities":[{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-03T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-03T07:30:00.000Z"},"__v":0,"image":"8187733396.png"},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-03T09:00:00.000Z"},"updatedAt":{"$date":"2026-02-03T09:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-03T12:45:00.000Z"},"updatedAt":{"$date":"2026-02-03T12:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-04T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-04T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-04T18:30:00.000Z"},"updatedAt":{"$date":"2026-02-04T18:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-05T07:45:00.000Z"},"updatedAt":{"$date":"2026-02-05T07:45:00.000Z"},"__v":0,"image":null},{"activity_name":"Light Exercise","createdAt":{"$date":"2026-02-05T10:15:00.000Z"},"updatedAt":{"$date":"2026-02-05T10:15:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-06T08:20:00.000Z"},"updatedAt":{"$date":"2026-02-06T08:20:00.000Z"},"__v":0,"image":null},{"activity_name":"Lunch","createdAt":{"$date":"2026-02-06T13:00:00.000Z"},"updatedAt":{"$date":"2026-02-06T13:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-07T07:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T07:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Morning Walk","createdAt":{"$date":"2026-02-07T09:30:00.000Z"},"updatedAt":{"$date":"2026-02-07T09:30:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-08T08:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T08:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Dinner","createdAt":{"$date":"2026-02-08T19:00:00.000Z"},"updatedAt":{"$date":"2026-02-08T19:00:00.000Z"},"__v":0,"image":null},{"activity_name":"Breakfast","createdAt":{"$date":"2026-02-09T08:15:00.000Z"},"updatedAt":{"$date":"2026-02-09T08:15:00.000Z"},"__v":0,"image":null}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:42:38.908Z</t>
+  </si>
+  <si>
+    <t>John Doe is a 36-year-old male experiencing occasional shortness of breath and forgetfulness related to ADHD. His vitals are generally stable with normal heart rate and blood pressure readings.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Shortness of breath reported on multiple occasions. Consider further evaluation.</t>
+  </si>
+  <si>
+    <t>Heart Rate: Consistently within normal range, averaging around 71 beats per minute. | Blood Pressure: Generally stable, ranging from 117/77 to 122/82 mmHg. | SPO2: Oxygen saturation levels are good, consistently at 97% or higher.</t>
+  </si>
+  <si>
+    <t>Routine activities such as regular meals and light exercise appear to support stable vital signs. | Shortness of breath has been observed without a clear correlation to specific activities.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet rich in fruits, vegetables, and whole grains. | Incorporate regular light exercises to help manage weight and cardiovascular health. | Establish a structured daily routine to help improve focus and reduce forgetfulness.</t>
+  </si>
+  <si>
+    <t>Monitor the frequency of shortness of breath. | Consider discussing symptoms of forgetfulness with the care team for potential adjustments in management.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment to discuss shortness of breath. | Consider cognitive assessments for ADHD management. | Track daily activities and symptoms for better insights during the next visit.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12T11:22:02.375Z"],[7,"2026-02-11T09:18:17.203Z"],[8,"2026-02-10T08:18:17.203Z"],[10,"2026-02-09T07:18:17.203Z"],[5,"2026-02-08T11:18:17.203Z"],[5,"2026-02-07T06:30:15.500Z"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[7,"2026-02-12T07:35:35.042Z"],[6,"2026-02-11T07:35:35.042Z"],[5,"2026-02-10T07:35:35.042Z"],[4,"2026-02-09T07:35:35.042Z"],[5,"2026-02-08T07:35:35.042Z"],[6,"2026-02-07T07:35:35.042Z"],[7,"2026-02-06T07:35:35.042Z"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11T08:11:09.381Z","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12T08:11:09.381Z","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14T08:11:09.381Z","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15T08:11:09.381Z","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16T08:11:09.381Z","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03T07:30:00.000Z"},{"activity_name":"Morning Walk","createdAt":"2026-02-03T09:00:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-03T12:45:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-04T08:00:00.000Z"},{"activity_name":"Dinner","createdAt":"2026-02-04T18:30:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-05T07:45:00.000Z"},{"activity_name":"Light Exercise","createdAt":"2026-02-05T10:15:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-06T08:20:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-06T13:00:00.000Z"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:43:48.993Z</t>
+  </si>
+  <si>
+    <t>John Doe is experiencing shortness of breath occasionally and some forgetfulness, but vital signs are stable and within normal ranges.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Shortness of breath noted; consider further evaluation.</t>
+  </si>
+  <si>
+    <t>Heart rate is within normal limits (69-74 bpm). | Blood pressure readings are stable with a systolic range of 117-122 mmHg and diastolic range of 77-82 mmHg. | Oxygen saturation levels consistently high at 97-99%.</t>
+  </si>
+  <si>
+    <t>Consistent breakfast and lunch routine observed. | Light exercise included in daily activities may positively impact respiratory symptoms.</t>
+  </si>
+  <si>
+    <t>Maintain a regular exercise routine to improve lung capacity. | Consider mindfulness or relaxation techniques to help with forgetfulness.</t>
+  </si>
+  <si>
+    <t>Monitor shortness of breath; suggest a follow-up appointment if symptoms persist.</t>
+  </si>
+  <si>
+    <t>Schedule a consultation with a healthcare provider. | Keep a daily log of symptoms and activities for review.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12T11:22:02.375Z"],[7,"2026-02-11T09:18:17.203Z"],[8,"2026-02-10T08:18:17.203Z"],[10,"2026-02-09T07:18:17.203Z"],[5,"2026-02-08T11:18:17.203Z"],[5,"2026-02-07T06:30:15.500Z"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[7,"2026-02-12T07:35:35.042Z"],[6,"2026-02-11T07:35:35.042Z"],[5,"2026-02-10T07:35:35.042Z"],[10,"2026-02-09T07:35:35.042Z"],[5,"2026-02-08T07:35:35.042Z"],[6,"2026-02-07T07:35:35.042Z"],[7,"2026-02-06T07:35:35.042Z"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11T08:11:09.381Z","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12T08:11:09.381Z","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14T08:11:09.381Z","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15T08:11:09.381Z","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16T08:11:09.381Z","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03T07:30:00.000Z"},{"activity_name":"Morning Walk","createdAt":"2026-02-03T09:00:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-03T12:45:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-04T08:00:00.000Z"},{"activity_name":"Dinner","createdAt":"2026-02-04T18:30:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-05T07:45:00.000Z"},{"activity_name":"Light Exercise","createdAt":"2026-02-05T10:15:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-06T08:20:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-06T13:00:00.000Z"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:45:10.486Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has shown some fluctuations in vital signs and experiences shortness of breath and forgetfulness from ADHD. Continuous monitoring is advised.</t>
+  </si>
+  <si>
+    <t>HIGH: Shortness of breath reported frequently; further evaluation is needed.</t>
+  </si>
+  <si>
+    <t>Heart rate ranged from 69 to 74 bpm, considered normal. | Blood pressure readings were stable, with a range of 117/77 to 122/82 mmHg, indicating good cardiovascular health. | Oxygen saturation levels were between 97% and 99%, which are within normal limits.</t>
+  </si>
+  <si>
+    <t>Morning activities such as breakfast and walking are consistent. | Regular meal timings might correlate with stable vitals.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet rich in fruits, vegetables, and whole grains to support overall health. | Incorporate evening relaxation techniques to improve sleep quality and focus.</t>
+  </si>
+  <si>
+    <t>Monitor the frequency of shortness of breath; consider discussing this with a specialist. | Patient may benefit from cognitive behavioral strategies to manage ADHD symptoms.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment to assess shortness of breath. | Consider consultation with a respiratory specialist. | Continue tracking daily activities and symptoms for further insights.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12T11:22:02.375Z"],[7,"2026-02-11T09:18:17.203Z"],[8,"2026-02-10T08:18:17.203Z"],[10,"2026-02-09T07:18:17.203Z"],[5,"2026-02-08T11:18:17.203Z"],[5,"2026-02-07T06:30:15.500Z"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[10,"2026-02-12T07:35:35.042Z"],[6,"2026-02-11T07:35:35.042Z"],[5,"2026-02-10T07:35:35.042Z"],[10,"2026-02-09T07:35:35.042Z"],[5,"2026-02-08T07:35:35.042Z"],[6,"2026-02-07T07:35:35.042Z"],[7,"2026-02-06T07:35:35.042Z"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11T08:11:09.381Z","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12T08:11:09.381Z","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14T08:11:09.381Z","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15T08:11:09.381Z","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16T08:11:09.381Z","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03T07:30:00.000Z"},{"activity_name":"Morning Walk","createdAt":"2026-02-03T09:00:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-03T12:45:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-04T08:00:00.000Z"},{"activity_name":"Dinner","createdAt":"2026-02-04T18:30:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-05T07:45:00.000Z"},{"activity_name":"Light Exercise","createdAt":"2026-02-05T10:15:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-06T08:20:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-06T13:00:00.000Z"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:46:38.976Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, has reported symptoms of shortness of breath and forgetfulness related to ADHD. His vital signs over the past week show stable heart rates and blood pressure within normal ranges, but the frequency of symptoms requires monitoring.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Shortness of breath has been recorded with a maximum severity of 10. Attention to this symptom is advised. | LOW: Forgetfulness related to ADHD reported with a maximum severity of 10. Consider strategies to enhance daily memory.</t>
+  </si>
+  <si>
+    <t>Heart rate has ranged from 69 to 74 beats per minute, indicating good cardiovascular health. | Blood pressure readings are stable, with systolic values between 117-122 and diastolic values between 77-82. | Oxygen saturation levels are consistently high at 97 to 99%, reflecting good respiratory function.</t>
+  </si>
+  <si>
+    <t>Regular breakfast routines are established, contributing to stable energy levels. | Physical activity, including morning walks and light exercises, may correlate with lower heart rates.</t>
+  </si>
+  <si>
+    <t>Incorporate breathing exercises or meditation to help manage shortness of breath. | Use reminders or checklists to assist with memory and daily activities.</t>
+  </si>
+  <si>
+    <t>Continue monitoring symptoms and vitals closely. | Follow up on the shortness of breath and explore potential triggers.</t>
+  </si>
+  <si>
+    <t>Schedule an appointment with a healthcare provider to discuss symptoms and develop a management plan. | Consider a consultation with a mental health professional for ADHD-related concerns.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12T11:22:02.375Z"],[7,"2026-02-11T09:18:17.203Z"],[8,"2026-02-10T08:18:17.203Z"],[10,"2026-02-09T07:18:17.203Z"],[5,"2026-02-08T11:18:17.203Z"],[5,"2026-02-07T06:30:15.500Z"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[5,"2026-02-12T07:35:35.042Z"],[5,"2026-02-11T07:35:35.042Z"],[5,"2026-02-10T07:35:35.042Z"],[10,"2026-02-09T07:35:35.042Z"],[5,"2026-02-08T07:35:35.042Z"],[5,"2026-02-07T07:35:35.042Z"],[5,"2026-02-06T07:35:35.042Z"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11T08:11:09.381Z","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12T08:11:09.381Z","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14T08:11:09.381Z","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15T08:11:09.381Z","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16T08:11:09.381Z","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03T07:30:00.000Z"},{"activity_name":"Morning Walk","createdAt":"2026-02-03T09:00:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-03T12:45:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-04T08:00:00.000Z"},{"activity_name":"Dinner","createdAt":"2026-02-04T18:30:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-05T07:45:00.000Z"},{"activity_name":"Light Exercise","createdAt":"2026-02-05T10:15:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-06T08:20:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-06T13:00:00.000Z"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:48:04.070Z</t>
+  </si>
+  <si>
+    <t>John Doe is 36 years old and has been experiencing some symptoms related to shortness of breath and forgetfulness in daily activities. His vital signs show generally stable heart rate and blood pressure.</t>
+  </si>
+  <si>
+    <t>MEDIUM: John has reported shortness of breath. Monitor this symptom closely and consult a healthcare provider if it worsens.</t>
+  </si>
+  <si>
+    <t>Heart rate has been stable, averaging around 71 beats per minute. | Blood pressure is within normal range, averaging 119/78. | Oxygen saturation (SPO2) levels are healthy, mostly at 98-99%.</t>
+  </si>
+  <si>
+    <t>Daily activities include consistent meal times and a morning walk, which may contribute positively to overall health. | Forgetfulness may be linked to daily stressors or lack of routine.</t>
+  </si>
+  <si>
+    <t>Consider maintaining a regular sleep schedule to improve memory and focus. | Incorporate light exercises daily to help with breathing and overall stamina.</t>
+  </si>
+  <si>
+    <t>Monitor John's symptoms of shortness of breath and document any changes. | Support with medication for ADHD may be evaluated based on symptom severity.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with a healthcare provider to discuss symptoms. | Keep a daily log of activities and symptoms to identify patterns.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12T11:22:02.375Z"],[7,"2026-02-11T09:18:17.203Z"],[8,"2026-02-10T08:18:17.203Z"],[9,"2026-02-09T07:18:17.203Z"],[5,"2026-02-08T11:18:17.203Z"],[5,"2026-02-07T06:30:15.500Z"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[4,"2026-02-12T07:35:35.042Z"],[4,"2026-02-11T07:35:35.042Z"],[4,"2026-02-10T07:35:35.042Z"],[9,"2026-02-09T07:35:35.042Z"],[4,"2026-02-08T07:35:35.042Z"],[4,"2026-02-07T07:35:35.042Z"],[4,"2026-02-06T07:35:35.042Z"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11T08:11:09.381Z","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12T08:11:09.381Z","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14T08:11:09.381Z","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15T08:11:09.381Z","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16T08:11:09.381Z","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03T07:30:00.000Z"},{"activity_name":"Morning Walk","createdAt":"2026-02-03T09:00:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-03T12:45:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-04T08:00:00.000Z"},{"activity_name":"Dinner","createdAt":"2026-02-04T18:30:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-05T07:45:00.000Z"},{"activity_name":"Light Exercise","createdAt":"2026-02-05T10:15:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-06T08:20:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-06T13:00:00.000Z"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:49:14.881Z</t>
+  </si>
+  <si>
+    <t>John Doe has experienced some episodes of shortness of breath. His vitals appear stable with normal heart rate and blood pressure readings over the past week.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Frequent occurrences of shortness of breath noted; consider further evaluation.</t>
+  </si>
+  <si>
+    <t>Heart rate is stable, ranging from 69 to 74 bpm. | Blood pressure readings are within normal limits, with systolic values ranging from 117 to 122 mmHg and diastolic values from 77 to 82 mmHg. | Oxygen saturation levels are good, consistently above 97%.</t>
+  </si>
+  <si>
+    <t>Regular meal patterns observed with consistent breakfast timings. | Incorporation of light exercise appears to correlate with stable vital signs. | Morning walks contribute positively to overall well-being.</t>
+  </si>
+  <si>
+    <t>Maintain a balanced diet focusing on whole foods rich in nutrients. | Incorporate breathing exercises or relaxation techniques to manage episodes of shortness of breath. | Ensure adequate hydration and regular physical activity.</t>
+  </si>
+  <si>
+    <t>Monitor episodes of shortness of breath; may require follow-up with a specialist. | Continue logging daily activities and symptoms for better diagnosis.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with your healthcare provider. | Consider discussing breathing exercises with a healthcare professional. | Continue to track daily activities and any additional symptoms.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12 11:22:02"],[7,"2026-02-11 09:18:17"],[8,"2026-02-10 08:18:17"],[9,"2026-02-09 07:18:17"],[5,"2026-02-08 11:18:17"],[5,"2026-02-07 06:30:15"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[4,"2026-02-12 07:35:35"],[4,"2026-02-11 07:35:35"],[4,"2026-02-10 07:35:35"],[9,"2026-02-09 07:35:35"],[4,"2026-02-08 07:35:35"],[4,"2026-02-07 07:35:35"],[4,"2026-02-06 07:35:35"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11T08:11:09.381Z","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12T08:11:09.381Z","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14T08:11:09.381Z","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15T08:11:09.381Z","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16T08:11:09.381Z","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17T08:11:09.381Z","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03T07:30:00.000Z"},{"activity_name":"Morning Walk","createdAt":"2026-02-03T09:00:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-03T12:45:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-04T08:00:00.000Z"},{"activity_name":"Dinner","createdAt":"2026-02-04T18:30:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-05T07:45:00.000Z"},{"activity_name":"Light Exercise","createdAt":"2026-02-05T10:15:00.000Z"},{"activity_name":"Breakfast","createdAt":"2026-02-06T08:20:00.000Z"},{"activity_name":"Lunch","createdAt":"2026-02-06T13:00:00.000Z"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:50:53.397Z</t>
+  </si>
+  <si>
+    <t>Patient John Doe, a 36-year-old male, shows stable vital signs but reports shortness of breath and forgetfulness associated with ADHD symptoms. Ongoing monitoring and lifestyle adjustments are recommended.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Shortness of breath reported; monitor breathing patterns.</t>
+  </si>
+  <si>
+    <t>Heart rates between 69-74 bpm, blood pressure ranges from 117/77 to 122/82 mmHg, and oxygen saturation levels consistently above 97%.</t>
+  </si>
+  <si>
+    <t>Routine activities like breakfast, lunch, and light exercise may influence overall well-being.</t>
+  </si>
+  <si>
+    <t>Incorporate regular breathing exercises in your morning routine to help with shortness of breath. | Consider keeping a daily planner to manage forgetfulness better.</t>
+  </si>
+  <si>
+    <t>Monitor the patient's reported symptoms closely; consider follow-up consultations if breathing issues persist.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment to discuss shortness of breath. | Implement breathing exercises and track symptoms daily.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cdf941eeb53a74254f5f","type":"symptom","symptom_title":"short of breath","symptoms":[{"records":[[6,"2026-02-12 11:22:02"],[7,"2026-02-11 09:18:17"],[8,"2026-02-10 08:18:17"],[9,"2026-02-09 07:18:17"],[5,"2026-02-08 11:18:17"],[5,"2026-02-07 06:30:15"]],"title":"short of breath"}]},{"condition_id":"698d82c7bb05e0b7c13a1f34","type":"symptom","symptom_title":"ADHD-is forgetful in daily activities.(0-4)","symptoms":[{"records":[[4,"2026-02-12 07:35:35"],[4,"2026-02-11 07:35:35"],[4,"2026-02-10 07:35:35"],[9,"2026-02-09 07:35:35"],[4,"2026-02-08 07:35:35"],[4,"2026-02-07 07:35:35"],[4,"2026-02-06 07:35:35"]],"title":"ADHD-is forgetful in daily activities.(0-4)"}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11 08:11:09","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12 08:11:09","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13 08:11:09","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14 08:11:09","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15 08:11:09","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16 08:11:09","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17 08:11:09","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03 07:30:00"},{"activity_name":"Morning Walk","createdAt":"2026-02-03 09:00:00"},{"activity_name":"Lunch","createdAt":"2026-02-03 12:45:00"},{"activity_name":"Breakfast","createdAt":"2026-02-04 08:00:00"},{"activity_name":"Dinner","createdAt":"2026-02-04 18:30:00"},{"activity_name":"Breakfast","createdAt":"2026-02-05 07:45:00"},{"activity_name":"Light Exercise","createdAt":"2026-02-05 10:15:00"},{"activity_name":"Breakfast","createdAt":"2026-02-06 08:20:00"},{"activity_name":"Lunch","createdAt":"2026-02-06 13:00:00"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T08:51:35.348Z</t>
+  </si>
+  <si>
+    <t>John Doe is recovering from alcohol withdrawal. His vital signs are relatively stable but his symptoms of confusion and sweating have decreased over time.</t>
+  </si>
+  <si>
+    <t>MEDIUM: Monitor for continued symptoms of confusion and sweating as they may indicate fluctuating withdrawal effects.</t>
+  </si>
+  <si>
+    <t>Heart rate is stable, averaging around 71 bpm. | Blood pressure remains within normal ranges, with systolic around 119 mmHg and diastolic around 79 mmHg. | Oxygen saturation is consistently high at around 98-99%.</t>
+  </si>
+  <si>
+    <t>Daily routine includes regular meal times and light exercise which may positively impact overall recovery. | Increased symptoms observed on days with less physical activity.</t>
+  </si>
+  <si>
+    <t>Continue to maintain a balanced diet to support recovery. | Incorporate light physical activities such as walking to help reduce symptoms. | Stay hydrated and avoid caffeine for better sleep quality.</t>
+  </si>
+  <si>
+    <t>Continue monitoring symptom levels and consider scheduling regular check-ins for support. | Evaluate the effectiveness of daily activities in managing withdrawal symptoms.</t>
+  </si>
+  <si>
+    <t>Schedule a follow-up appointment with your healthcare provider. | Keep a daily log of symptoms and activities for better management insights. | Consider joining a support group to aid recovery.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[[7,"2026-02-03 09:00:00"],[6,"2026-02-04 09:15:00"],[4,"2026-02-05 08:45:00"],[5,"2026-02-06 09:30:00"],[3,"2026-02-07 08:50:00"],[4,"2026-02-08 09:10:00"],[2,"2026-02-09 09:00:00"]]},{"title":"sweating","records":[[6,"2026-02-03 09:00:00"],[5,"2026-02-04 09:15:00"],[5,"2026-02-05 08:45:00"],[4,"2026-02-06 09:30:00"],[4,"2026-02-07 08:50:00"],[3,"2026-02-08 09:10:00"],[2,"2026-02-09 09:00:00"]]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-11 08:11:09","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-12 08:11:09","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-13 08:11:09","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-14 08:11:09","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-15 08:11:09","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-16 08:11:09","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-17 08:11:09","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03 07:30:00"},{"activity_name":"Morning Walk","createdAt":"2026-02-03 09:00:00"},{"activity_name":"Lunch","createdAt":"2026-02-03 12:45:00"},{"activity_name":"Breakfast","createdAt":"2026-02-04 08:00:00"},{"activity_name":"Dinner","createdAt":"2026-02-04 18:30:00"},{"activity_name":"Breakfast","createdAt":"2026-02-05 07:45:00"},{"activity_name":"Light Exercise","createdAt":"2026-02-05 10:15:00"},{"activity_name":"Breakfast","createdAt":"2026-02-06 08:20:00"},{"activity_name":"Lunch","createdAt":"2026-02-06 13:00:00"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-20T10:06:39.290Z</t>
+  </si>
+  <si>
+    <t>John Doe is experiencing symptoms related to alcohol withdrawal. Monitoring is crucial.</t>
+  </si>
+  <si>
+    <t>HIGH: Confusion levels are concerning and should be assessed by a healthcare professional. | MEDIUM: Sweating levels indicate discomfort and potential hydration issues.</t>
+  </si>
+  <si>
+    <t>No vital signs were recorded, indicating a need for regular monitoring.</t>
+  </si>
+  <si>
+    <t>Breakfast is a consistent part of the morning routine. | Morning walks may positively influence mood and symptoms.</t>
+  </si>
+  <si>
+    <t>Consider a balanced diet with plenty of hydration to support recovery. | Regular light exercise may help improve overall well-being.</t>
+  </si>
+  <si>
+    <t>Patient's symptoms require careful observation, especially confusion and sweating.</t>
+  </si>
+  <si>
+    <t>Schedule an appointment with a healthcare provider. | Increase monitoring of symptoms and hydration.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[[7,"2026-02-03 09:00:00"],[6,"2026-02-04 09:15:00"],[4,"2026-02-05 08:45:00"],[5,"2026-02-06 09:30:00"],[3,"2026-02-07 08:50:00"],[4,"2026-02-08 09:10:00"],[2,"2026-02-09 09:00:00"]]},{"title":"sweating","records":[[6,"2026-02-03 09:00:00"],[5,"2026-02-04 09:15:00"],[5,"2026-02-05 08:45:00"],[4,"2026-02-06 09:30:00"],[4,"2026-02-07 08:50:00"],[3,"2026-02-08 09:10:00"],[2,"2026-02-09 09:00:00"]]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03 07:30:00"},{"activity_name":"Morning Walk","createdAt":"2026-02-03 09:00:00"},{"activity_name":"Lunch","createdAt":"2026-02-03 12:45:00"},{"activity_name":"Breakfast","createdAt":"2026-02-04 08:00:00"},{"activity_name":"Dinner","createdAt":"2026-02-04 18:30:00"},{"activity_name":"Breakfast","createdAt":"2026-02-05 07:45:00"},{"activity_name":"Light Exercise","createdAt":"2026-02-05 10:15:00"},{"activity_name":"Breakfast","createdAt":"2026-02-06 08:20:00"},{"activity_name":"Lunch","createdAt":"2026-02-06 13:00:00"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-24T07:02:28.164Z</t>
+  </si>
+  <si>
+    <t>John Doe, a 36-year-old male, is experiencing symptoms of alcohol withdrawal with episodes of confusion, sweating, anxiety, and disrupted sleep.</t>
+  </si>
+  <si>
+    <t>HIGH: The patient is displaying severe symptoms of alcohol withdrawal. Immediate medical attention is recommended.</t>
+  </si>
+  <si>
+    <t>Heart rate, blood pressure, and oxygen saturation are mostly within normal ranges, but there are instances of lower blood pressure readings.</t>
+  </si>
+  <si>
+    <t>Routine activities such as meals and exercise could be affecting the severity of withdrawal symptoms. Maintaining consistent meals may help stabilize mood.</t>
+  </si>
+  <si>
+    <t>Consider calming activities, such as meditation or calming teas, to help reduce anxiety. | Maintain a balanced diet with regular hydration to support recovery.</t>
+  </si>
+  <si>
+    <t>Monitor patient's vitals closely, especially heart rate and blood pressure. Schedule regular follow-ups to assess withdrawal symptoms and recovery progress.</t>
+  </si>
+  <si>
+    <t>Consult with a healthcare provider to evaluate the need for a support program for alcohol withdrawal. | Schedule follow-up appointments to monitor mental health and vitals.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[[7,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[6,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[5,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[6,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[5,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[4,"2026-02-19 18:00:00"],[3,"2026-02-19 20:00:00"],[4,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[5,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[4,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[5,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[4,"2026-02-21 12:00:00"],[3,"2026-02-21 14:00:00"],[4,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[4,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[4,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[3,"2026-02-23 14:00:00"],[2,"2026-02-23 16:00:00"],[3,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[3,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[3,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]},{"title":"sweating","records":[[6,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[5,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[4,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[5,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[4,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[3,"2026-02-19 18:00:00"],[4,"2026-02-19 20:00:00"],[3,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[4,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[3,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[4,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[3,"2026-02-21 12:00:00"],[4,"2026-02-21 14:00:00"],[3,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[3,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[3,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[2,"2026-02-23 14:00:00"],[3,"2026-02-23 16:00:00"],[2,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[2,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[2,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]},{"title":"anxiety","records":[[6,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[5,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[4,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[5,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[4,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[3,"2026-02-19 18:00:00"],[4,"2026-02-19 20:00:00"],[3,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[4,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[3,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[4,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[3,"2026-02-21 12:00:00"],[4,"2026-02-21 14:00:00"],[3,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[3,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[3,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[2,"2026-02-23 14:00:00"],[3,"2026-02-23 16:00:00"],[2,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[2,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[2,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]},{"title":"sleep","records":[[6,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[5,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[4,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[5,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[4,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[3,"2026-02-19 18:00:00"],[4,"2026-02-19 20:00:00"],[3,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[4,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[3,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[4,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[3,"2026-02-21 12:00:00"],[4,"2026-02-21 14:00:00"],[3,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[3,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[3,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[2,"2026-02-23 14:00:00"],[3,"2026-02-23 16:00:00"],[2,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[2,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[2,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-18 06:00:00","vitals":[["HEART_RATE",76],["BLOOD_PRESSURE",{"systolic":124,"diastolic":84}],["SPO2",96]]},{"recorded_at":"2026-02-18 08:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-18 10:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",97]]},{"recorded_at":"2026-02-18 12:00:00","vitals":[["HEART_RATE",75],["BLOOD_PRESSURE",{"systolic":123,"diastolic":83}],["SPO2",97]]},{"recorded_at":"2026-02-18 14:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",98]]},{"recorded_at":"2026-02-18 16:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-18 18:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",98]]},{"recorded_at":"2026-02-18 20:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-18 21:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",99]]},{"recorded_at":"2026-02-18 22:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-19 06:00:00","vitals":[["HEART_RATE",75],["BLOOD_PRESSURE",{"systolic":123,"diastolic":83}],["SPO2",97]]},{"recorded_at":"2026-02-19 08:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",97]]},{"recorded_at":"2026-02-19 10:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-19 12:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",98]]},{"recorded_at":"2026-02-19 14:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-19 16:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-19 18:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",99]]},{"recorded_at":"2026-02-19 20:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-19 21:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-19 22:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-20 06:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-20 08:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-20 10:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-20 12:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",98]]},{"recorded_at":"2026-02-20 14:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-20 16:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-20 18:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-20 20:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-20 21:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-20 22:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-21 06:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",98]]},{"recorded_at":"2026-02-21 08:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-21 10:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",98]]},{"recorded_at":"2026-02-21 12:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",99]]},{"recorded_at":"2026-02-21 14:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-21 16:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-21 18:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-21 20:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-21 21:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-21 22:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-22 06:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-22 08:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",98]]},{"recorded_at":"2026-02-22 10:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-22 12:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-22 14:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-22 16:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-22 18:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-22 20:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-22 21:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-22 22:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-23 06:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-23 08:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-23 10:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-23 12:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-23 14:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-23 16:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-23 18:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-23 20:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-23 21:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-23 22:00:00","vitals":[["HEART_RATE",65],["BLOOD_PRESSURE",{"systolic":113,"diastolic":73}],["SPO2",99]]},{"recorded_at":"2026-02-24 06:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-24 08:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-24 10:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-24 12:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-24 14:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-24 16:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-24 18:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-24 20:00:00","vitals":[["HEART_RATE",65],["BLOOD_PRESSURE",{"systolic":113,"diastolic":73}],["SPO2",99]]},{"recorded_at":"2026-02-24 21:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-24 22:00:00","vitals":[["HEART_RATE",64],["BLOOD_PRESSURE",{"systolic":112,"diastolic":72}],["SPO2",99]]}],"activities":[{"activity_name":"Breakfast","createdAt":"2026-02-03 07:30:00"},{"activity_name":"Morning Walk","createdAt":"2026-02-03 09:00:00"},{"activity_name":"Lunch","createdAt":"2026-02-03 12:45:00"},{"activity_name":"Breakfast","createdAt":"2026-02-04 08:00:00"},{"activity_name":"Dinner","createdAt":"2026-02-04 18:30:00"},{"activity_name":"Breakfast","createdAt":"2026-02-05 07:45:00"},{"activity_name":"Light Exercise","createdAt":"2026-02-05 10:15:00"},{"activity_name":"Breakfast","createdAt":"2026-02-06 08:20:00"},{"activity_name":"Lunch","createdAt":"2026-02-06 13:00:00"}]}</t>
+  </si>
+  <si>
+    <t>2026-02-24T07:04:46.727Z</t>
+  </si>
+  <si>
+    <t>John Doe is experiencing symptoms related to Alcohol Withdrawal, including confusion, sweating, anxiety, and sleep disturbances. Vitals are fluctuating but mostly within normal ranges.</t>
+  </si>
+  <si>
+    <t>HIGH: Symptoms of confusion and high anxiety indicate a need for immediate medical attention.</t>
+  </si>
+  <si>
+    <t>Heart rate is generally within normal limits but shows fluctuations, particularly during periods of anxiety. | Blood pressure readings are mostly stable, with some slight fluctuations. | Oxygen saturation is consistently above 95%, indicating good respiratory function.</t>
+  </si>
+  <si>
+    <t>Routine activities like meals and walks seem to correlate with improved mood and symptom management. | Increased symptoms of anxiety and confusion are noticeable during times without structured activity.</t>
+  </si>
+  <si>
+    <t>Engage in regular light exercises to help manage anxiety and enhance mood. | Maintain a consistent sleep schedule and practice relaxation techniques before bedtime. | Consider a balanced diet rich in fruits, vegetables, and lean proteins.</t>
+  </si>
+  <si>
+    <t>Close monitoring of John's symptoms is advised due to the severity of anxiety and confusion. | Encourage regular follow-ups to assess mental health status.</t>
+  </si>
+  <si>
+    <t>Schedule an appointment with a healthcare provider for a thorough assessment. | Implement a structured daily routine to help stabilize mood and anxiety levels. | Consider involving a mental health professional for additional support.</t>
+  </si>
+  <si>
+    <t>{"conditions":[{"condition_id":"6985cb0d41eeb53a74254efe","type":"disease","disease_title":"Alcohol Withdrawal","symptoms":[{"title":"confusion","records":[[7,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[6,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[5,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[6,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[5,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[4,"2026-02-19 18:00:00"],[3,"2026-02-19 20:00:00"],[4,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[5,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[4,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[5,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[4,"2026-02-21 12:00:00"],[3,"2026-02-21 14:00:00"],[4,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[4,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[4,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[3,"2026-02-23 14:00:00"],[2,"2026-02-23 16:00:00"],[3,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[3,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[3,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]},{"title":"sweating","records":[[6,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[5,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[4,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[5,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[4,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[3,"2026-02-19 18:00:00"],[4,"2026-02-19 20:00:00"],[3,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[4,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[3,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[4,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[3,"2026-02-21 12:00:00"],[4,"2026-02-21 14:00:00"],[3,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[3,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[3,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[2,"2026-02-23 14:00:00"],[3,"2026-02-23 16:00:00"],[2,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[2,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[2,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]},{"title":"anxiety","records":[[6,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[5,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[4,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[5,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[4,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[3,"2026-02-19 18:00:00"],[4,"2026-02-19 20:00:00"],[3,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[4,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[3,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[4,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[3,"2026-02-21 12:00:00"],[4,"2026-02-21 14:00:00"],[3,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[3,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[3,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[2,"2026-02-23 14:00:00"],[3,"2026-02-23 16:00:00"],[2,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[2,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[2,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]},{"title":"sleep","records":[[6,"2026-02-18 06:00:00"],[6,"2026-02-18 08:00:00"],[5,"2026-02-18 10:00:00"],[5,"2026-02-18 12:00:00"],[5,"2026-02-18 14:00:00"],[4,"2026-02-18 16:00:00"],[4,"2026-02-18 18:00:00"],[4,"2026-02-18 20:00:00"],[3,"2026-02-18 21:00:00"],[4,"2026-02-18 22:00:00"],[5,"2026-02-19 06:00:00"],[5,"2026-02-19 08:00:00"],[5,"2026-02-19 10:00:00"],[4,"2026-02-19 12:00:00"],[4,"2026-02-19 14:00:00"],[4,"2026-02-19 16:00:00"],[3,"2026-02-19 18:00:00"],[4,"2026-02-19 20:00:00"],[3,"2026-02-19 21:00:00"],[3,"2026-02-19 22:00:00"],[5,"2026-02-20 06:00:00"],[4,"2026-02-20 08:00:00"],[4,"2026-02-20 10:00:00"],[4,"2026-02-20 12:00:00"],[4,"2026-02-20 14:00:00"],[3,"2026-02-20 16:00:00"],[3,"2026-02-20 18:00:00"],[3,"2026-02-20 20:00:00"],[3,"2026-02-20 21:00:00"],[2,"2026-02-20 22:00:00"],[4,"2026-02-21 06:00:00"],[4,"2026-02-21 08:00:00"],[4,"2026-02-21 10:00:00"],[3,"2026-02-21 12:00:00"],[4,"2026-02-21 14:00:00"],[3,"2026-02-21 16:00:00"],[3,"2026-02-21 18:00:00"],[3,"2026-02-21 20:00:00"],[2,"2026-02-21 21:00:00"],[3,"2026-02-21 22:00:00"],[4,"2026-02-22 06:00:00"],[4,"2026-02-22 08:00:00"],[3,"2026-02-22 10:00:00"],[3,"2026-02-22 12:00:00"],[3,"2026-02-22 14:00:00"],[3,"2026-02-22 16:00:00"],[3,"2026-02-22 18:00:00"],[2,"2026-02-22 20:00:00"],[3,"2026-02-22 21:00:00"],[2,"2026-02-22 22:00:00"],[3,"2026-02-23 06:00:00"],[3,"2026-02-23 08:00:00"],[3,"2026-02-23 10:00:00"],[3,"2026-02-23 12:00:00"],[2,"2026-02-23 14:00:00"],[3,"2026-02-23 16:00:00"],[2,"2026-02-23 18:00:00"],[2,"2026-02-23 20:00:00"],[2,"2026-02-23 21:00:00"],[2,"2026-02-23 22:00:00"],[3,"2026-02-24 06:00:00"],[3,"2026-02-24 08:00:00"],[2,"2026-02-24 10:00:00"],[2,"2026-02-24 12:00:00"],[2,"2026-02-24 14:00:00"],[2,"2026-02-24 16:00:00"],[2,"2026-02-24 18:00:00"],[2,"2026-02-24 20:00:00"],[2,"2026-02-24 21:00:00"],[2,"2026-02-24 22:00:00"]]}]}],"patient":{"name":"John Doe","gender":"Male","age":36},"vitals":[{"recorded_at":"2026-02-18 06:00:00","vitals":[["HEART_RATE",76],["BLOOD_PRESSURE",{"systolic":124,"diastolic":84}],["SPO2",96]]},{"recorded_at":"2026-02-18 08:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-18 10:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",97]]},{"recorded_at":"2026-02-18 12:00:00","vitals":[["HEART_RATE",75],["BLOOD_PRESSURE",{"systolic":123,"diastolic":83}],["SPO2",97]]},{"recorded_at":"2026-02-18 14:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",98]]},{"recorded_at":"2026-02-18 16:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-18 18:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",98]]},{"recorded_at":"2026-02-18 20:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-18 21:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",99]]},{"recorded_at":"2026-02-18 22:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-19 06:00:00","vitals":[["HEART_RATE",75],["BLOOD_PRESSURE",{"systolic":123,"diastolic":83}],["SPO2",97]]},{"recorded_at":"2026-02-19 08:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",97]]},{"recorded_at":"2026-02-19 10:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-19 12:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",98]]},{"recorded_at":"2026-02-19 14:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-19 16:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-19 18:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",99]]},{"recorded_at":"2026-02-19 20:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-19 21:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-19 22:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-20 06:00:00","vitals":[["HEART_RATE",74],["BLOOD_PRESSURE",{"systolic":122,"diastolic":82}],["SPO2",97]]},{"recorded_at":"2026-02-20 08:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-20 10:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-20 12:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",98]]},{"recorded_at":"2026-02-20 14:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-20 16:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-20 18:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-20 20:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-20 21:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-20 22:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-21 06:00:00","vitals":[["HEART_RATE",73],["BLOOD_PRESSURE",{"systolic":121,"diastolic":81}],["SPO2",98]]},{"recorded_at":"2026-02-21 08:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-21 10:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",98]]},{"recorded_at":"2026-02-21 12:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",99]]},{"recorded_at":"2026-02-21 14:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-21 16:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-21 18:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-21 20:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-21 21:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-21 22:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-22 06:00:00","vitals":[["HEART_RATE",72],["BLOOD_PRESSURE",{"systolic":120,"diastolic":80}],["SPO2",98]]},{"recorded_at":"2026-02-22 08:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",98]]},{"recorded_at":"2026-02-22 10:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-22 12:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",99]]},{"recorded_at":"2026-02-22 14:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-22 16:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-22 18:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-22 20:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-22 21:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-22 22:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-23 06:00:00","vitals":[["HEART_RATE",71],["BLOOD_PRESSURE",{"systolic":119,"diastolic":79}],["SPO2",98]]},{"recorded_at":"2026-02-23 08:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-23 10:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-23 12:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-23 14:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-23 16:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-23 18:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-23 20:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-23 21:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-23 22:00:00","vitals":[["HEART_RATE",65],["BLOOD_PRESSURE",{"systolic":113,"diastolic":73}],["SPO2",99]]},{"recorded_at":"2026-02-24 06:00:00","vitals":[["HEART_RATE",70],["BLOOD_PRESSURE",{"systolic":118,"diastolic":78}],["SPO2",99]]},{"recorded_at":"2026-02-24 08:00:00","vitals":[["HEART_RATE",68],["BLOOD_PRESSURE",{"systolic":116,"diastolic":76}],["SPO2",99]]},{"recorded_at":"2026-02-24 10:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-24 12:00:00","vitals":[["HEART_RATE",69],["BLOOD_PRESSURE",{"systolic":117,"diastolic":77}],["SPO2",99]]},{"recorded_at":"2026-02-24 14:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-24 16:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-24 18:00:00","vitals":[["HEART_RATE",67],["BLOOD_PRESSURE",{"systolic":115,"diastolic":75}],["SPO2",99]]},{"recorded_at":"2026-02-24 20:00:00","vitals":[["HEART_RATE",65],["BLOOD_PRESSURE",{"systolic":113,"diastolic":73}],["SPO2",99]]},{"recorded_at":"2026-02-24 21:00:00","vitals":[["HEART_RATE",66],["BLOOD_PRESSURE",{"systolic":114,"diastolic":74}],["SPO2",99]]},{"recorded_at":"2026-02-24 22:00:00","vitals":[["HEART_RATE",64],["BLOOD_PRESSURE",{"systolic":112,"diastolic":72}],["SPO2",99]]}],"activities":[["Breakfast","2026-02-18 06:00:00"],["Morning Walk","2026-02-18 08:00:00"],["Snack","2026-02-18 10:00:00"],["Lunch","2026-02-18 12:00:00"],["Rest","2026-02-18 14:00:00"],["Light Exercise","2026-02-18 16:00:00"],["Dinner","2026-02-18 18:00:00"],["Evening Walk","2026-02-18 20:00:00"],["Snack","2026-02-18 21:00:00"],["Rest","2026-02-18 22:00:00"],["Breakfast","2026-02-19 06:00:00"],["Morning Walk","2026-02-19 08:00:00"],["Snack","2026-02-19 10:00:00"],["Lunch","2026-02-19 12:00:00"],["Rest","2026-02-19 14:00:00"],["Light Exercise","2026-02-19 16:00:00"],["Dinner","2026-02-19 18:00:00"],["Evening Walk","2026-02-19 20:00:00"],["Snack","2026-02-19 21:00:00"],["Rest","2026-02-19 22:00:00"],["Breakfast","2026-02-20 06:00:00"],["Morning Walk","2026-02-20 08:00:00"],["Snack","2026-02-20 10:00:00"],["Lunch","2026-02-20 12:00:00"],["Rest","2026-02-20 14:00:00"],["Light Exercise","2026-02-20 16:00:00"],["Dinner","2026-02-20 18:00:00"],["Evening Walk","2026-02-20 20:00:00"],["Snack","2026-02-20 21:00:00"],["Rest","2026-02-20 22:00:00"],["Breakfast","2026-02-21 06:00:00"],["Morning Walk","2026-02-21 08:00:00"],["Snack","2026-02-21 10:00:00"],["Lunch","2026-02-21 12:00:00"],["Rest","2026-02-21 14:00:00"],["Light Exercise","2026-02-21 16:00:00"],["Dinner","2026-02-21 18:00:00"],["Evening Walk","2026-02-21 20:00:00"],["Snack","2026-02-21 21:00:00"],["Rest","2026-02-21 22:00:00"],["Breakfast","2026-02-22 06:00:00"],["Morning Walk","2026-02-22 08:00:00"],["Snack","2026-02-22 10:00:00"],["Lunch","2026-02-22 12:00:00"],["Rest","2026-02-22 14:00:00"],["Light Exercise","2026-02-22 16:00:00"],["Dinner","2026-02-22 18:00:00"],["Evening Walk","2026-02-22 20:00:00"],["Snack","2026-02-22 21:00:00"],["Rest","2026-02-22 22:00:00"],["Breakfast","2026-02-23 06:00:00"],["Morning Walk","2026-02-23 08:00:00"],["Snack","2026-02-23 10:00:00"],["Lunch","2026-02-23 12:00:00"],["Rest","2026-02-23 14:00:00"],["Light Exercise","2026-02-23 16:00:00"],["Dinner","2026-02-23 18:00:00"],["Evening Walk","2026-02-23 20:00:00"],["Snack","2026-02-23 21:00:00"],["Rest","2026-02-23 22:00:00"],["Breakfast","2026-02-24 06:00:00"],["Morning Walk","2026-02-24 08:00:00"],["Snack","2026-02-24 10:00:00"],["Lunch","2026-02-24 12:00:00"],["Rest","2026-02-24 14:00:00"],["Light Exercise","2026-02-24 16:00:00"],["Dinner","2026-02-24 18:00:00"],["Evening Walk","2026-02-24 20:00:00"],["Snack","2026-02-24 21:00:00"],["Rest","2026-02-24 22:00:00"]]}</t>
   </si>
 </sst>
 </file>
@@ -2433,7 +2784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R86"/>
+  <dimension ref="A1:R108"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -6965,6 +7316,1238 @@
         <v>681</v>
       </c>
     </row>
+    <row r="87" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>682</v>
+      </c>
+      <c r="B87" t="s">
+        <v>19</v>
+      </c>
+      <c r="C87" t="s">
+        <v>20</v>
+      </c>
+      <c r="D87">
+        <v>36</v>
+      </c>
+      <c r="E87" t="s">
+        <v>310</v>
+      </c>
+      <c r="F87" t="s">
+        <v>311</v>
+      </c>
+      <c r="G87" t="s">
+        <v>683</v>
+      </c>
+      <c r="H87" t="s">
+        <v>684</v>
+      </c>
+      <c r="I87" t="s">
+        <v>685</v>
+      </c>
+      <c r="J87" t="s">
+        <v>686</v>
+      </c>
+      <c r="K87" t="s">
+        <v>687</v>
+      </c>
+      <c r="L87" t="s">
+        <v>688</v>
+      </c>
+      <c r="M87" t="s">
+        <v>689</v>
+      </c>
+      <c r="N87">
+        <v>3032</v>
+      </c>
+      <c r="O87">
+        <v>307</v>
+      </c>
+      <c r="P87">
+        <v>3339</v>
+      </c>
+      <c r="Q87" t="s">
+        <v>34</v>
+      </c>
+      <c r="R87" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="88" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>682</v>
+      </c>
+      <c r="B88" t="s">
+        <v>19</v>
+      </c>
+      <c r="C88" t="s">
+        <v>20</v>
+      </c>
+      <c r="D88">
+        <v>36</v>
+      </c>
+      <c r="E88" t="s">
+        <v>322</v>
+      </c>
+      <c r="F88" t="s">
+        <v>323</v>
+      </c>
+      <c r="G88" t="s">
+        <v>683</v>
+      </c>
+      <c r="H88" t="s">
+        <v>684</v>
+      </c>
+      <c r="I88" t="s">
+        <v>685</v>
+      </c>
+      <c r="J88" t="s">
+        <v>686</v>
+      </c>
+      <c r="K88" t="s">
+        <v>687</v>
+      </c>
+      <c r="L88" t="s">
+        <v>688</v>
+      </c>
+      <c r="M88" t="s">
+        <v>689</v>
+      </c>
+      <c r="N88">
+        <v>3032</v>
+      </c>
+      <c r="O88">
+        <v>307</v>
+      </c>
+      <c r="P88">
+        <v>3339</v>
+      </c>
+      <c r="Q88" t="s">
+        <v>34</v>
+      </c>
+      <c r="R88" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="89" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>691</v>
+      </c>
+      <c r="B89" t="s">
+        <v>19</v>
+      </c>
+      <c r="C89" t="s">
+        <v>20</v>
+      </c>
+      <c r="D89">
+        <v>36</v>
+      </c>
+      <c r="E89" t="s">
+        <v>310</v>
+      </c>
+      <c r="F89" t="s">
+        <v>311</v>
+      </c>
+      <c r="G89" t="s">
+        <v>692</v>
+      </c>
+      <c r="H89" t="s">
+        <v>693</v>
+      </c>
+      <c r="I89" t="s">
+        <v>694</v>
+      </c>
+      <c r="J89" t="s">
+        <v>695</v>
+      </c>
+      <c r="K89" t="s">
+        <v>696</v>
+      </c>
+      <c r="L89" t="s">
+        <v>697</v>
+      </c>
+      <c r="M89" t="s">
+        <v>698</v>
+      </c>
+      <c r="N89">
+        <v>3169</v>
+      </c>
+      <c r="O89">
+        <v>333</v>
+      </c>
+      <c r="P89">
+        <v>3502</v>
+      </c>
+      <c r="Q89" t="s">
+        <v>34</v>
+      </c>
+      <c r="R89" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="90" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>691</v>
+      </c>
+      <c r="B90" t="s">
+        <v>19</v>
+      </c>
+      <c r="C90" t="s">
+        <v>20</v>
+      </c>
+      <c r="D90">
+        <v>36</v>
+      </c>
+      <c r="E90" t="s">
+        <v>322</v>
+      </c>
+      <c r="F90" t="s">
+        <v>323</v>
+      </c>
+      <c r="G90" t="s">
+        <v>692</v>
+      </c>
+      <c r="H90" t="s">
+        <v>693</v>
+      </c>
+      <c r="I90" t="s">
+        <v>694</v>
+      </c>
+      <c r="J90" t="s">
+        <v>695</v>
+      </c>
+      <c r="K90" t="s">
+        <v>696</v>
+      </c>
+      <c r="L90" t="s">
+        <v>697</v>
+      </c>
+      <c r="M90" t="s">
+        <v>698</v>
+      </c>
+      <c r="N90">
+        <v>3169</v>
+      </c>
+      <c r="O90">
+        <v>333</v>
+      </c>
+      <c r="P90">
+        <v>3502</v>
+      </c>
+      <c r="Q90" t="s">
+        <v>34</v>
+      </c>
+      <c r="R90" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="91" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>700</v>
+      </c>
+      <c r="B91" t="s">
+        <v>19</v>
+      </c>
+      <c r="C91" t="s">
+        <v>20</v>
+      </c>
+      <c r="D91">
+        <v>36</v>
+      </c>
+      <c r="E91" t="s">
+        <v>310</v>
+      </c>
+      <c r="F91" t="s">
+        <v>311</v>
+      </c>
+      <c r="G91" t="s">
+        <v>701</v>
+      </c>
+      <c r="H91" t="s">
+        <v>702</v>
+      </c>
+      <c r="I91" t="s">
+        <v>703</v>
+      </c>
+      <c r="J91" t="s">
+        <v>704</v>
+      </c>
+      <c r="K91" t="s">
+        <v>705</v>
+      </c>
+      <c r="L91" t="s">
+        <v>706</v>
+      </c>
+      <c r="M91" t="s">
+        <v>707</v>
+      </c>
+      <c r="N91">
+        <v>1221</v>
+      </c>
+      <c r="O91">
+        <v>339</v>
+      </c>
+      <c r="P91">
+        <v>1560</v>
+      </c>
+      <c r="Q91" t="s">
+        <v>34</v>
+      </c>
+      <c r="R91" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="92" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>700</v>
+      </c>
+      <c r="B92" t="s">
+        <v>19</v>
+      </c>
+      <c r="C92" t="s">
+        <v>20</v>
+      </c>
+      <c r="D92">
+        <v>36</v>
+      </c>
+      <c r="E92" t="s">
+        <v>322</v>
+      </c>
+      <c r="F92" t="s">
+        <v>323</v>
+      </c>
+      <c r="G92" t="s">
+        <v>701</v>
+      </c>
+      <c r="H92" t="s">
+        <v>702</v>
+      </c>
+      <c r="I92" t="s">
+        <v>703</v>
+      </c>
+      <c r="J92" t="s">
+        <v>704</v>
+      </c>
+      <c r="K92" t="s">
+        <v>705</v>
+      </c>
+      <c r="L92" t="s">
+        <v>706</v>
+      </c>
+      <c r="M92" t="s">
+        <v>707</v>
+      </c>
+      <c r="N92">
+        <v>1221</v>
+      </c>
+      <c r="O92">
+        <v>339</v>
+      </c>
+      <c r="P92">
+        <v>1560</v>
+      </c>
+      <c r="Q92" t="s">
+        <v>34</v>
+      </c>
+      <c r="R92" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="93" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>709</v>
+      </c>
+      <c r="B93" t="s">
+        <v>19</v>
+      </c>
+      <c r="C93" t="s">
+        <v>20</v>
+      </c>
+      <c r="D93">
+        <v>36</v>
+      </c>
+      <c r="E93" t="s">
+        <v>310</v>
+      </c>
+      <c r="F93" t="s">
+        <v>311</v>
+      </c>
+      <c r="G93" t="s">
+        <v>710</v>
+      </c>
+      <c r="H93" t="s">
+        <v>711</v>
+      </c>
+      <c r="I93" t="s">
+        <v>712</v>
+      </c>
+      <c r="J93" t="s">
+        <v>713</v>
+      </c>
+      <c r="K93" t="s">
+        <v>714</v>
+      </c>
+      <c r="L93" t="s">
+        <v>715</v>
+      </c>
+      <c r="M93" t="s">
+        <v>716</v>
+      </c>
+      <c r="N93">
+        <v>1221</v>
+      </c>
+      <c r="O93">
+        <v>261</v>
+      </c>
+      <c r="P93">
+        <v>1482</v>
+      </c>
+      <c r="Q93" t="s">
+        <v>34</v>
+      </c>
+      <c r="R93" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="94" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>709</v>
+      </c>
+      <c r="B94" t="s">
+        <v>19</v>
+      </c>
+      <c r="C94" t="s">
+        <v>20</v>
+      </c>
+      <c r="D94">
+        <v>36</v>
+      </c>
+      <c r="E94" t="s">
+        <v>322</v>
+      </c>
+      <c r="F94" t="s">
+        <v>323</v>
+      </c>
+      <c r="G94" t="s">
+        <v>710</v>
+      </c>
+      <c r="H94" t="s">
+        <v>711</v>
+      </c>
+      <c r="I94" t="s">
+        <v>712</v>
+      </c>
+      <c r="J94" t="s">
+        <v>713</v>
+      </c>
+      <c r="K94" t="s">
+        <v>714</v>
+      </c>
+      <c r="L94" t="s">
+        <v>715</v>
+      </c>
+      <c r="M94" t="s">
+        <v>716</v>
+      </c>
+      <c r="N94">
+        <v>1221</v>
+      </c>
+      <c r="O94">
+        <v>261</v>
+      </c>
+      <c r="P94">
+        <v>1482</v>
+      </c>
+      <c r="Q94" t="s">
+        <v>34</v>
+      </c>
+      <c r="R94" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>718</v>
+      </c>
+      <c r="B95" t="s">
+        <v>19</v>
+      </c>
+      <c r="C95" t="s">
+        <v>20</v>
+      </c>
+      <c r="D95">
+        <v>36</v>
+      </c>
+      <c r="E95" t="s">
+        <v>310</v>
+      </c>
+      <c r="F95" t="s">
+        <v>311</v>
+      </c>
+      <c r="G95" t="s">
+        <v>719</v>
+      </c>
+      <c r="H95" t="s">
+        <v>720</v>
+      </c>
+      <c r="I95" t="s">
+        <v>721</v>
+      </c>
+      <c r="J95" t="s">
+        <v>722</v>
+      </c>
+      <c r="K95" t="s">
+        <v>723</v>
+      </c>
+      <c r="L95" t="s">
+        <v>724</v>
+      </c>
+      <c r="M95" t="s">
+        <v>725</v>
+      </c>
+      <c r="N95">
+        <v>1214</v>
+      </c>
+      <c r="O95">
+        <v>313</v>
+      </c>
+      <c r="P95">
+        <v>1527</v>
+      </c>
+      <c r="Q95" t="s">
+        <v>34</v>
+      </c>
+      <c r="R95" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="96" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>718</v>
+      </c>
+      <c r="B96" t="s">
+        <v>19</v>
+      </c>
+      <c r="C96" t="s">
+        <v>20</v>
+      </c>
+      <c r="D96">
+        <v>36</v>
+      </c>
+      <c r="E96" t="s">
+        <v>322</v>
+      </c>
+      <c r="F96" t="s">
+        <v>323</v>
+      </c>
+      <c r="G96" t="s">
+        <v>719</v>
+      </c>
+      <c r="H96" t="s">
+        <v>720</v>
+      </c>
+      <c r="I96" t="s">
+        <v>721</v>
+      </c>
+      <c r="J96" t="s">
+        <v>722</v>
+      </c>
+      <c r="K96" t="s">
+        <v>723</v>
+      </c>
+      <c r="L96" t="s">
+        <v>724</v>
+      </c>
+      <c r="M96" t="s">
+        <v>725</v>
+      </c>
+      <c r="N96">
+        <v>1214</v>
+      </c>
+      <c r="O96">
+        <v>313</v>
+      </c>
+      <c r="P96">
+        <v>1527</v>
+      </c>
+      <c r="Q96" t="s">
+        <v>34</v>
+      </c>
+      <c r="R96" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="97" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>727</v>
+      </c>
+      <c r="B97" t="s">
+        <v>19</v>
+      </c>
+      <c r="C97" t="s">
+        <v>20</v>
+      </c>
+      <c r="D97">
+        <v>36</v>
+      </c>
+      <c r="E97" t="s">
+        <v>310</v>
+      </c>
+      <c r="F97" t="s">
+        <v>311</v>
+      </c>
+      <c r="G97" t="s">
+        <v>728</v>
+      </c>
+      <c r="H97" t="s">
+        <v>729</v>
+      </c>
+      <c r="I97" t="s">
+        <v>730</v>
+      </c>
+      <c r="J97" t="s">
+        <v>731</v>
+      </c>
+      <c r="K97" t="s">
+        <v>732</v>
+      </c>
+      <c r="L97" t="s">
+        <v>733</v>
+      </c>
+      <c r="M97" t="s">
+        <v>734</v>
+      </c>
+      <c r="N97">
+        <v>1234</v>
+      </c>
+      <c r="O97">
+        <v>379</v>
+      </c>
+      <c r="P97">
+        <v>1613</v>
+      </c>
+      <c r="Q97" t="s">
+        <v>34</v>
+      </c>
+      <c r="R97" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="98" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>727</v>
+      </c>
+      <c r="B98" t="s">
+        <v>19</v>
+      </c>
+      <c r="C98" t="s">
+        <v>20</v>
+      </c>
+      <c r="D98">
+        <v>36</v>
+      </c>
+      <c r="E98" t="s">
+        <v>322</v>
+      </c>
+      <c r="F98" t="s">
+        <v>323</v>
+      </c>
+      <c r="G98" t="s">
+        <v>728</v>
+      </c>
+      <c r="H98" t="s">
+        <v>729</v>
+      </c>
+      <c r="I98" t="s">
+        <v>730</v>
+      </c>
+      <c r="J98" t="s">
+        <v>731</v>
+      </c>
+      <c r="K98" t="s">
+        <v>732</v>
+      </c>
+      <c r="L98" t="s">
+        <v>733</v>
+      </c>
+      <c r="M98" t="s">
+        <v>734</v>
+      </c>
+      <c r="N98">
+        <v>1234</v>
+      </c>
+      <c r="O98">
+        <v>379</v>
+      </c>
+      <c r="P98">
+        <v>1613</v>
+      </c>
+      <c r="Q98" t="s">
+        <v>34</v>
+      </c>
+      <c r="R98" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>736</v>
+      </c>
+      <c r="B99" t="s">
+        <v>19</v>
+      </c>
+      <c r="C99" t="s">
+        <v>20</v>
+      </c>
+      <c r="D99">
+        <v>36</v>
+      </c>
+      <c r="E99" t="s">
+        <v>310</v>
+      </c>
+      <c r="F99" t="s">
+        <v>311</v>
+      </c>
+      <c r="G99" t="s">
+        <v>737</v>
+      </c>
+      <c r="H99" t="s">
+        <v>738</v>
+      </c>
+      <c r="I99" t="s">
+        <v>739</v>
+      </c>
+      <c r="J99" t="s">
+        <v>740</v>
+      </c>
+      <c r="K99" t="s">
+        <v>741</v>
+      </c>
+      <c r="L99" t="s">
+        <v>742</v>
+      </c>
+      <c r="M99" t="s">
+        <v>743</v>
+      </c>
+      <c r="N99">
+        <v>1213</v>
+      </c>
+      <c r="O99">
+        <v>315</v>
+      </c>
+      <c r="P99">
+        <v>1528</v>
+      </c>
+      <c r="Q99" t="s">
+        <v>34</v>
+      </c>
+      <c r="R99" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="100" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>736</v>
+      </c>
+      <c r="B100" t="s">
+        <v>19</v>
+      </c>
+      <c r="C100" t="s">
+        <v>20</v>
+      </c>
+      <c r="D100">
+        <v>36</v>
+      </c>
+      <c r="E100" t="s">
+        <v>322</v>
+      </c>
+      <c r="F100" t="s">
+        <v>323</v>
+      </c>
+      <c r="G100" t="s">
+        <v>737</v>
+      </c>
+      <c r="H100" t="s">
+        <v>738</v>
+      </c>
+      <c r="I100" t="s">
+        <v>739</v>
+      </c>
+      <c r="J100" t="s">
+        <v>740</v>
+      </c>
+      <c r="K100" t="s">
+        <v>741</v>
+      </c>
+      <c r="L100" t="s">
+        <v>742</v>
+      </c>
+      <c r="M100" t="s">
+        <v>743</v>
+      </c>
+      <c r="N100">
+        <v>1213</v>
+      </c>
+      <c r="O100">
+        <v>315</v>
+      </c>
+      <c r="P100">
+        <v>1528</v>
+      </c>
+      <c r="Q100" t="s">
+        <v>34</v>
+      </c>
+      <c r="R100" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="101" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>745</v>
+      </c>
+      <c r="B101" t="s">
+        <v>19</v>
+      </c>
+      <c r="C101" t="s">
+        <v>20</v>
+      </c>
+      <c r="D101">
+        <v>36</v>
+      </c>
+      <c r="E101" t="s">
+        <v>310</v>
+      </c>
+      <c r="F101" t="s">
+        <v>311</v>
+      </c>
+      <c r="G101" t="s">
+        <v>746</v>
+      </c>
+      <c r="H101" t="s">
+        <v>747</v>
+      </c>
+      <c r="I101" t="s">
+        <v>748</v>
+      </c>
+      <c r="J101" t="s">
+        <v>749</v>
+      </c>
+      <c r="K101" t="s">
+        <v>750</v>
+      </c>
+      <c r="L101" t="s">
+        <v>751</v>
+      </c>
+      <c r="M101" t="s">
+        <v>752</v>
+      </c>
+      <c r="N101">
+        <v>1174</v>
+      </c>
+      <c r="O101">
+        <v>334</v>
+      </c>
+      <c r="P101">
+        <v>1508</v>
+      </c>
+      <c r="Q101" t="s">
+        <v>34</v>
+      </c>
+      <c r="R101" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="102" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>745</v>
+      </c>
+      <c r="B102" t="s">
+        <v>19</v>
+      </c>
+      <c r="C102" t="s">
+        <v>20</v>
+      </c>
+      <c r="D102">
+        <v>36</v>
+      </c>
+      <c r="E102" t="s">
+        <v>322</v>
+      </c>
+      <c r="F102" t="s">
+        <v>323</v>
+      </c>
+      <c r="G102" t="s">
+        <v>746</v>
+      </c>
+      <c r="H102" t="s">
+        <v>747</v>
+      </c>
+      <c r="I102" t="s">
+        <v>748</v>
+      </c>
+      <c r="J102" t="s">
+        <v>749</v>
+      </c>
+      <c r="K102" t="s">
+        <v>750</v>
+      </c>
+      <c r="L102" t="s">
+        <v>751</v>
+      </c>
+      <c r="M102" t="s">
+        <v>752</v>
+      </c>
+      <c r="N102">
+        <v>1174</v>
+      </c>
+      <c r="O102">
+        <v>334</v>
+      </c>
+      <c r="P102">
+        <v>1508</v>
+      </c>
+      <c r="Q102" t="s">
+        <v>34</v>
+      </c>
+      <c r="R102" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="103" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>754</v>
+      </c>
+      <c r="B103" t="s">
+        <v>19</v>
+      </c>
+      <c r="C103" t="s">
+        <v>20</v>
+      </c>
+      <c r="D103">
+        <v>36</v>
+      </c>
+      <c r="E103" t="s">
+        <v>310</v>
+      </c>
+      <c r="F103" t="s">
+        <v>311</v>
+      </c>
+      <c r="G103" t="s">
+        <v>755</v>
+      </c>
+      <c r="H103" t="s">
+        <v>756</v>
+      </c>
+      <c r="I103" t="s">
+        <v>757</v>
+      </c>
+      <c r="J103" t="s">
+        <v>758</v>
+      </c>
+      <c r="K103" t="s">
+        <v>759</v>
+      </c>
+      <c r="L103" t="s">
+        <v>760</v>
+      </c>
+      <c r="M103" t="s">
+        <v>761</v>
+      </c>
+      <c r="N103">
+        <v>1126</v>
+      </c>
+      <c r="O103">
+        <v>254</v>
+      </c>
+      <c r="P103">
+        <v>1380</v>
+      </c>
+      <c r="Q103" t="s">
+        <v>34</v>
+      </c>
+      <c r="R103" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="104" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>754</v>
+      </c>
+      <c r="B104" t="s">
+        <v>19</v>
+      </c>
+      <c r="C104" t="s">
+        <v>20</v>
+      </c>
+      <c r="D104">
+        <v>36</v>
+      </c>
+      <c r="E104" t="s">
+        <v>322</v>
+      </c>
+      <c r="F104" t="s">
+        <v>323</v>
+      </c>
+      <c r="G104" t="s">
+        <v>755</v>
+      </c>
+      <c r="H104" t="s">
+        <v>756</v>
+      </c>
+      <c r="I104" t="s">
+        <v>757</v>
+      </c>
+      <c r="J104" t="s">
+        <v>758</v>
+      </c>
+      <c r="K104" t="s">
+        <v>759</v>
+      </c>
+      <c r="L104" t="s">
+        <v>760</v>
+      </c>
+      <c r="M104" t="s">
+        <v>761</v>
+      </c>
+      <c r="N104">
+        <v>1126</v>
+      </c>
+      <c r="O104">
+        <v>254</v>
+      </c>
+      <c r="P104">
+        <v>1380</v>
+      </c>
+      <c r="Q104" t="s">
+        <v>34</v>
+      </c>
+      <c r="R104" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="105" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>763</v>
+      </c>
+      <c r="B105" t="s">
+        <v>19</v>
+      </c>
+      <c r="C105" t="s">
+        <v>20</v>
+      </c>
+      <c r="D105">
+        <v>36</v>
+      </c>
+      <c r="E105" t="s">
+        <v>356</v>
+      </c>
+      <c r="F105" t="s">
+        <v>357</v>
+      </c>
+      <c r="G105" t="s">
+        <v>764</v>
+      </c>
+      <c r="H105" t="s">
+        <v>765</v>
+      </c>
+      <c r="I105" t="s">
+        <v>766</v>
+      </c>
+      <c r="J105" t="s">
+        <v>767</v>
+      </c>
+      <c r="K105" t="s">
+        <v>768</v>
+      </c>
+      <c r="L105" t="s">
+        <v>769</v>
+      </c>
+      <c r="M105" t="s">
+        <v>770</v>
+      </c>
+      <c r="N105">
+        <v>1080</v>
+      </c>
+      <c r="O105">
+        <v>312</v>
+      </c>
+      <c r="P105">
+        <v>1392</v>
+      </c>
+      <c r="Q105" t="s">
+        <v>34</v>
+      </c>
+      <c r="R105" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="106" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>772</v>
+      </c>
+      <c r="B106" t="s">
+        <v>19</v>
+      </c>
+      <c r="C106" t="s">
+        <v>20</v>
+      </c>
+      <c r="D106">
+        <v>36</v>
+      </c>
+      <c r="E106" t="s">
+        <v>356</v>
+      </c>
+      <c r="F106" t="s">
+        <v>357</v>
+      </c>
+      <c r="G106" t="s">
+        <v>773</v>
+      </c>
+      <c r="H106" t="s">
+        <v>774</v>
+      </c>
+      <c r="I106" t="s">
+        <v>775</v>
+      </c>
+      <c r="J106" t="s">
+        <v>776</v>
+      </c>
+      <c r="K106" t="s">
+        <v>777</v>
+      </c>
+      <c r="L106" t="s">
+        <v>778</v>
+      </c>
+      <c r="M106" t="s">
+        <v>779</v>
+      </c>
+      <c r="N106">
+        <v>694</v>
+      </c>
+      <c r="O106">
+        <v>227</v>
+      </c>
+      <c r="P106">
+        <v>921</v>
+      </c>
+      <c r="Q106" t="s">
+        <v>34</v>
+      </c>
+      <c r="R106" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="107" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>781</v>
+      </c>
+      <c r="B107" t="s">
+        <v>19</v>
+      </c>
+      <c r="C107" t="s">
+        <v>20</v>
+      </c>
+      <c r="D107">
+        <v>36</v>
+      </c>
+      <c r="E107" t="s">
+        <v>356</v>
+      </c>
+      <c r="F107" t="s">
+        <v>357</v>
+      </c>
+      <c r="G107" t="s">
+        <v>782</v>
+      </c>
+      <c r="H107" t="s">
+        <v>783</v>
+      </c>
+      <c r="I107" t="s">
+        <v>784</v>
+      </c>
+      <c r="J107" t="s">
+        <v>785</v>
+      </c>
+      <c r="K107" t="s">
+        <v>786</v>
+      </c>
+      <c r="L107" t="s">
+        <v>787</v>
+      </c>
+      <c r="M107" t="s">
+        <v>788</v>
+      </c>
+      <c r="N107">
+        <v>8816</v>
+      </c>
+      <c r="O107">
+        <v>264</v>
+      </c>
+      <c r="P107">
+        <v>9080</v>
+      </c>
+      <c r="Q107" t="s">
+        <v>34</v>
+      </c>
+      <c r="R107" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="108" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>790</v>
+      </c>
+      <c r="B108" t="s">
+        <v>19</v>
+      </c>
+      <c r="C108" t="s">
+        <v>20</v>
+      </c>
+      <c r="D108">
+        <v>36</v>
+      </c>
+      <c r="E108" t="s">
+        <v>356</v>
+      </c>
+      <c r="F108" t="s">
+        <v>357</v>
+      </c>
+      <c r="G108" t="s">
+        <v>791</v>
+      </c>
+      <c r="H108" t="s">
+        <v>792</v>
+      </c>
+      <c r="I108" t="s">
+        <v>793</v>
+      </c>
+      <c r="J108" t="s">
+        <v>794</v>
+      </c>
+      <c r="K108" t="s">
+        <v>795</v>
+      </c>
+      <c r="L108" t="s">
+        <v>796</v>
+      </c>
+      <c r="M108" t="s">
+        <v>797</v>
+      </c>
+      <c r="N108">
+        <v>9772</v>
+      </c>
+      <c r="O108">
+        <v>323</v>
+      </c>
+      <c r="P108">
+        <v>10095</v>
+      </c>
+      <c r="Q108" t="s">
+        <v>34</v>
+      </c>
+      <c r="R108" t="s">
+        <v>798</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>